<commit_message>
Confirm Bascara stay and update Girona routes
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="Rb0771e78d94f4721"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Itinerary" sheetId="2" r:id="Rf435d3a93cd24b9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reservations" sheetId="3" r:id="R1c26fb510f604f0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport" sheetId="4" r:id="R656ff40782354408"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accommodation" sheetId="5" r:id="Ra53eb7018a3d4a37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R6f88862334f148ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publication QA" sheetId="7" r:id="Rb16ef487458e4eb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="8" r:id="Rd50e839db73c4ccd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Maps" sheetId="9" r:id="Rf43c14b2a48d4384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photo Rights" sheetId="10" r:id="Rab55c53c8d774fe0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Shots" sheetId="11" r:id="R1c21cce5ba564e12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase8 Lock Status" sheetId="12" r:id="R480bd8d4981f4b85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="Rdfdee7b9696e48a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Itinerary" sheetId="2" r:id="Ra13418291827495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reservations" sheetId="3" r:id="R8606c74104e8473b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport" sheetId="4" r:id="Re34b6182ecc44699"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accommodation" sheetId="5" r:id="Rdb971fb0678c4baf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rbbaef063f7554d0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publication QA" sheetId="7" r:id="R191d5a09dfd24e07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="8" r:id="R28ded542efc14edd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Maps" sheetId="9" r:id="R1ce3fb6bbd5c40e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photo Rights" sheetId="10" r:id="Rd27520febf8e40cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Shots" sheetId="11" r:id="R84ec1d09c7e94922"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase8 Lock Status" sheetId="12" r:id="R9dfeb7db6d94413a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -380,7 +380,7 @@
         <x:color rgb="FF274E13"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -390,7 +390,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -400,7 +400,7 @@
         <x:color rgb="FF990000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -421,17 +421,14 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr/>
               <a:t>프로젝트 영역별 완성도</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:varyColors val="0"/>
@@ -562,7 +559,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9b5a0e38f4e44c79"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3a20c64a5b3e43c5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -614,9 +611,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2341,7 +2338,7 @@
         <x:v>완료</x:v>
       </x:c>
       <x:c r="G5" s="47" t="str">
-        <x:v>주소·예약번호는 미잠금</x:v>
+        <x:v>Bàscara 숙소 잠금 · 나머지 주소·예약번호 미잠금</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2393,7 +2390,7 @@
         <x:v>이동</x:v>
       </x:c>
       <x:c r="B8" s="47" t="str">
-        <x:v>Girona→Nice</x:v>
+        <x:v>Bàscara→Nice</x:v>
       </x:c>
       <x:c r="C8" s="47" t="str">
         <x:v>BLOCKED</x:v>
@@ -2519,21 +2516,23 @@
         <x:v>숙소</x:v>
       </x:c>
       <x:c r="B14" s="47" t="str">
-        <x:v>Girona</x:v>
+        <x:v>Bàscara (Girona 권역)</x:v>
       </x:c>
       <x:c r="C14" s="47" t="str">
-        <x:v>BLOCKED</x:v>
+        <x:v>LOCKED</x:v>
       </x:c>
       <x:c r="D14" s="47" t="str">
-        <x:v>3박</x:v>
+        <x:v>Airbnb · 바스카라의 B&amp;B · 2026-09-01~09-04 · 3박</x:v>
       </x:c>
       <x:c r="E14" s="47" t="str">
-        <x:v>숙소명·주소·주차·예약번호</x:v>
+        <x:v>확정번호·가격·결제·체크인·주차·조식·취소조건</x:v>
       </x:c>
       <x:c r="F14" s="47" t="str">
-        <x:v>사용자 입력</x:v>
-      </x:c>
-      <x:c r="G14" s="47" t="str"/>
+        <x:v>사용자 확정</x:v>
+      </x:c>
+      <x:c r="G14" s="47" t="str">
+        <x:v>Plaça de l’Església, 6, 17483 Bàscara, Catalonia, Spain</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="47" t="str">
@@ -2981,7 +2980,7 @@
         <x:v>Tue</x:v>
       </x:c>
       <x:c r="C7" s="16" t="str">
-        <x:v>Girona</x:v>
+        <x:v>Bàscara</x:v>
       </x:c>
       <x:c r="D7" s="16" t="n">
         <x:v>1</x:v>
@@ -2990,29 +2989,48 @@
         <x:v>이동</x:v>
       </x:c>
       <x:c r="F7" s="47" t="str">
-        <x:v>렌터카 인수·시체스·Girona 이동</x:v>
-      </x:c>
-      <x:c r="G7" s="47" t="str"/>
-      <x:c r="H7" s="47" t="str"/>
-      <x:c r="I7" s="47" t="str"/>
-      <x:c r="J7" s="47" t="str"/>
-      <x:c r="K7" s="47" t="str"/>
-      <x:c r="L7" s="47" t="str"/>
-      <x:c r="M7" s="47" t="str"/>
+        <x:v>렌터카 인수·Sitges·Girona 축소 또는 Bàscara</x:v>
+      </x:c>
+      <x:c r="G7" s="47" t="str">
+        <x:v>렌터카 인수·Sitges</x:v>
+      </x:c>
+      <x:c r="H7" s="47" t="str">
+        <x:v>Sitges</x:v>
+      </x:c>
+      <x:c r="I7" s="47" t="str">
+        <x:v>Girona 축소 또는 Bàscara 직행</x:v>
+      </x:c>
+      <x:c r="J7" s="47" t="str">
+        <x:v>Bàscara 체크인·간단식</x:v>
+      </x:c>
+      <x:c r="K7" s="47" t="str">
+        <x:v>Barcelona→Sitges→Girona 또는 Bàscara</x:v>
+      </x:c>
+      <x:c r="L7" s="47" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="M7" s="47" t="str">
+        <x:v>Girona 사진 선택</x:v>
+      </x:c>
       <x:c r="N7" s="47" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="O7" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P7" s="47" t="str"/>
-      <x:c r="Q7" s="47" t="str"/>
+        <x:v>예약반영</x:v>
+      </x:c>
+      <x:c r="P7" s="47" t="str">
+        <x:v>R002·렌터카</x:v>
+      </x:c>
+      <x:c r="Q7" s="47" t="str">
+        <x:v>체크인 시간 우선·Girona 삭제 가능</x:v>
+      </x:c>
       <x:c r="R7" s="47" t="str">
-        <x:v>05_Girona_Collioure_Emporda_v1.1.md</x:v>
+        <x:v>05_Girona_Collioure_Emporda_v2.1.md</x:v>
       </x:c>
       <x:c r="S7" s="48" t="n">
-        <x:v>46234</x:v>
-      </x:c>
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="T7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="37" t="n">
@@ -3022,7 +3040,7 @@
         <x:v>Wed</x:v>
       </x:c>
       <x:c r="C8" s="16" t="str">
-        <x:v>Girona</x:v>
+        <x:v>Bàscara</x:v>
       </x:c>
       <x:c r="D8" s="16" t="n">
         <x:v>2</x:v>
@@ -3031,29 +3049,38 @@
         <x:v>체류</x:v>
       </x:c>
       <x:c r="F8" s="47" t="str">
-        <x:v>Collioure·Peralada</x:v>
-      </x:c>
-      <x:c r="G8" s="47" t="str"/>
-      <x:c r="H8" s="47" t="str"/>
-      <x:c r="I8" s="47" t="str"/>
-      <x:c r="J8" s="47" t="str"/>
-      <x:c r="K8" s="47" t="str"/>
-      <x:c r="L8" s="47" t="str"/>
-      <x:c r="M8" s="47" t="str"/>
+        <x:v>Bàscara→Collioure→Peralada→Bàscara</x:v>
+      </x:c>
+      <x:c r="G8" s="47"/>
+      <x:c r="H8" s="47"/>
+      <x:c r="I8" s="47"/>
+      <x:c r="J8" s="47"/>
+      <x:c r="K8" s="47" t="str">
+        <x:v>Bàscara→Collioure→Peralada→Bàscara</x:v>
+      </x:c>
+      <x:c r="L8" s="47" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="M8" s="47"/>
       <x:c r="N8" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O8" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P8" s="47" t="str"/>
-      <x:c r="Q8" s="47" t="str"/>
+        <x:v>예약반영</x:v>
+      </x:c>
+      <x:c r="P8" s="47" t="str">
+        <x:v>R002·Peralada</x:v>
+      </x:c>
+      <x:c r="Q8" s="47" t="str">
+        <x:v>지연 시 Peralada 박물관 취소</x:v>
+      </x:c>
       <x:c r="R8" s="47" t="str">
-        <x:v>05_Girona_Collioure_Emporda_v1.1.md</x:v>
+        <x:v>05_Girona_Collioure_Emporda_v2.1.md</x:v>
       </x:c>
       <x:c r="S8" s="48" t="n">
-        <x:v>46234</x:v>
-      </x:c>
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="T8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="37" t="n">
@@ -3063,7 +3090,7 @@
         <x:v>Thu</x:v>
       </x:c>
       <x:c r="C9" s="16" t="str">
-        <x:v>Girona</x:v>
+        <x:v>Bàscara</x:v>
       </x:c>
       <x:c r="D9" s="16" t="n">
         <x:v>3</x:v>
@@ -3072,29 +3099,38 @@
         <x:v>체류</x:v>
       </x:c>
       <x:c r="F9" s="47" t="str">
-        <x:v>Pals·Peratallada·Calella de Palafrugell</x:v>
-      </x:c>
-      <x:c r="G9" s="47" t="str"/>
-      <x:c r="H9" s="47" t="str"/>
-      <x:c r="I9" s="47" t="str"/>
-      <x:c r="J9" s="47" t="str"/>
-      <x:c r="K9" s="47" t="str"/>
-      <x:c r="L9" s="47" t="str"/>
-      <x:c r="M9" s="47" t="str"/>
+        <x:v>Bàscara→Pals→Peratallada→Calella→Bàscara</x:v>
+      </x:c>
+      <x:c r="G9" s="47"/>
+      <x:c r="H9" s="47"/>
+      <x:c r="I9" s="47"/>
+      <x:c r="J9" s="47"/>
+      <x:c r="K9" s="47" t="str">
+        <x:v>Bàscara→Pals→Peratallada→Calella→Bàscara</x:v>
+      </x:c>
+      <x:c r="L9" s="47" t="str">
+        <x:v>Jason 선택 러닝</x:v>
+      </x:c>
+      <x:c r="M9" s="47"/>
       <x:c r="N9" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O9" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P9" s="47" t="str"/>
-      <x:c r="Q9" s="47" t="str"/>
+        <x:v>예약반영</x:v>
+      </x:c>
+      <x:c r="P9" s="47" t="str">
+        <x:v>R002·주차</x:v>
+      </x:c>
+      <x:c r="Q9" s="47" t="str">
+        <x:v>해안산책 축소 가능</x:v>
+      </x:c>
       <x:c r="R9" s="47" t="str">
-        <x:v>05_Girona_Collioure_Emporda_v1.1.md</x:v>
+        <x:v>05_Girona_Collioure_Emporda_v2.1.md</x:v>
       </x:c>
       <x:c r="S9" s="48" t="n">
-        <x:v>46234</x:v>
-      </x:c>
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="T9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="37" t="n">
@@ -3113,50 +3149,48 @@
         <x:v>이동</x:v>
       </x:c>
       <x:c r="F10" s="47" t="str">
-        <x:v>Girona→BCN→Nice 이동·정착</x:v>
+        <x:v>Bàscara→Nice 이동·정착</x:v>
       </x:c>
       <x:c r="G10" s="47" t="str">
-        <x:v>차량반납·항공·Nice 체크인</x:v>
+        <x:v>Bàscara 체크아웃·차량 반납 준비</x:v>
       </x:c>
       <x:c r="H10" s="47" t="str">
-        <x:v>체크아웃·공항이동</x:v>
+        <x:v>이동 중</x:v>
       </x:c>
       <x:c r="I10" s="47" t="str">
-        <x:v>공항 또는 이동식</x:v>
+        <x:v>Nice 이동</x:v>
       </x:c>
       <x:c r="J10" s="47" t="str">
-        <x:v>NCE 도착·숙소이동</x:v>
+        <x:v>Nice 도착 후 체크인</x:v>
       </x:c>
       <x:c r="K10" s="47" t="str">
-        <x:v>Masséna·Promenade 적응</x:v>
+        <x:v>Bàscara→Nice</x:v>
       </x:c>
       <x:c r="L10" s="47" t="str">
-        <x:v>Girona→BCN→NCE→Nice</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="M10" s="47" t="str">
-        <x:v>없음</x:v>
-      </x:c>
-      <x:c r="N10" s="47" t="str">
         <x:v>도착사진 선택</x:v>
       </x:c>
-      <x:c r="O10" s="47" t="n">
+      <x:c r="N10" s="47" t="n">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="O10" s="47" t="str">
+        <x:v>검토중</x:v>
+      </x:c>
       <x:c r="P10" s="47" t="str">
-        <x:v>검토</x:v>
+        <x:v>이동수단·차량반납</x:v>
       </x:c>
       <x:c r="Q10" s="47" t="str">
-        <x:v>항공·차량반납</x:v>
+        <x:v>지연 시 도착 후 산책 삭제</x:v>
       </x:c>
       <x:c r="R10" s="47" t="str">
-        <x:v>지연 시 산책 삭제</x:v>
-      </x:c>
-      <x:c r="S10" s="48" t="str">
         <x:v>06_Nice_Cote_d_Azur_v1.3.md</x:v>
       </x:c>
-      <x:c r="T10" t="n">
-        <x:v>46235</x:v>
-      </x:c>
+      <x:c r="S10" s="48" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="T10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="37" t="n">
@@ -5008,44 +5042,48 @@
         <x:v>Girona</x:v>
       </x:c>
       <x:c r="D5" s="47" t="str">
-        <x:v>숙소 3박</x:v>
+        <x:v>바스카라의 B&amp;B · 3박</x:v>
       </x:c>
       <x:c r="E5" s="61" t="n">
         <x:v>46266</x:v>
       </x:c>
-      <x:c r="F5" s="47" t="str"/>
+      <x:c r="F5" s="47"/>
       <x:c r="G5" s="47" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H5" s="47" t="str">
-        <x:v>미조사</x:v>
-      </x:c>
-      <x:c r="I5" s="61" t="n">
-        <x:v>46239</x:v>
-      </x:c>
-      <x:c r="J5" s="61" t="str"/>
+        <x:v>예약완료</x:v>
+      </x:c>
+      <x:c r="I5" s="61"/>
+      <x:c r="J5" s="61"/>
       <x:c r="K5" s="62"/>
       <x:c r="L5" s="62" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="M5" s="62" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N5" s="62" t="str">
-        <x:f>IF(K5="","",K5-M5)</x:f>
-      </x:c>
-      <x:c r="O5" s="47" t="str"/>
-      <x:c r="P5" s="47" t="str"/>
-      <x:c r="Q5" s="47" t="str"/>
-      <x:c r="R5" s="47" t="str"/>
+      <x:c r="M5" s="62"/>
+      <x:c r="N5" s="62"/>
+      <x:c r="O5" s="47"/>
+      <x:c r="P5" s="47" t="str">
+        <x:v>Airbnb</x:v>
+      </x:c>
+      <x:c r="Q5" s="47" t="str">
+        <x:v>Plaça de l’Església, 6, 17483 Bàscara, Catalonia, Spain</x:v>
+      </x:c>
+      <x:c r="R5" s="47" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Pla%C3%A7a+de+l%27Esgl%C3%A9sia%2C+6%2C+17483+B%C3%A0scara%2C+Spain</x:v>
+      </x:c>
       <x:c r="S5" s="47" t="str">
-        <x:v>05_Girona_Collioure_Emporda_v1.1.md</x:v>
+        <x:v>05_Girona_Collioure_Emporda_v2.1.md</x:v>
       </x:c>
       <x:c r="T5" s="47" t="str">
-        <x:v>주차·차량진입·짐</x:v>
-      </x:c>
-      <x:c r="U5" s="61" t="str"/>
-      <x:c r="V5" s="63" t="str"/>
+        <x:v>체크인 시간·주차·조식·결제·취소조건 재확인</x:v>
+      </x:c>
+      <x:c r="U5" s="61" t="n">
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="V5" s="63" t="str">
+        <x:v>Jason·Julia · 2026-09-01~09-04 · 3박</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="15" t="str">
@@ -6342,19 +6380,19 @@
         <x:v>Barcelona</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
-        <x:v>Sitges→Girona</x:v>
+        <x:v>Sitges→Girona 또는 Bàscara</x:v>
       </x:c>
       <x:c r="E5" s="16" t="str">
         <x:v>렌터카</x:v>
       </x:c>
-      <x:c r="F5" s="16" t="str"/>
-      <x:c r="G5" s="16" t="str"/>
-      <x:c r="H5" s="47" t="str"/>
-      <x:c r="I5" s="47" t="str"/>
+      <x:c r="F5" s="16"/>
+      <x:c r="G5" s="16"/>
+      <x:c r="H5" s="47"/>
+      <x:c r="I5" s="47"/>
       <x:c r="J5" s="47" t="str">
         <x:v>미조사</x:v>
       </x:c>
-      <x:c r="K5" s="47" t="str"/>
+      <x:c r="K5" s="47"/>
       <x:c r="L5" s="47" t="str">
         <x:v>장기여행 짐</x:v>
       </x:c>
@@ -6368,12 +6406,12 @@
         <x:v>짐 노출·주차·반납</x:v>
       </x:c>
       <x:c r="P5" s="47" t="str">
-        <x:v>시체스 축소 또는 직행</x:v>
+        <x:v>Sitges 지연 시 Girona 관광 삭제·Bàscara 직행</x:v>
       </x:c>
       <x:c r="Q5" s="47" t="str">
         <x:v>04/05</x:v>
       </x:c>
-      <x:c r="R5" s="61" t="str"/>
+      <x:c r="R5" s="61"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="15" t="str">
@@ -6383,7 +6421,7 @@
         <x:v>46269</x:v>
       </x:c>
       <x:c r="C6" s="16" t="str">
-        <x:v>Girona</x:v>
+        <x:v>Bàscara</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
         <x:v>Nice</x:v>
@@ -6391,16 +6429,16 @@
       <x:c r="E6" s="16" t="str">
         <x:v>미정</x:v>
       </x:c>
-      <x:c r="F6" s="16" t="str"/>
-      <x:c r="G6" s="16" t="str"/>
-      <x:c r="H6" s="47" t="str"/>
-      <x:c r="I6" s="47" t="str"/>
+      <x:c r="F6" s="16"/>
+      <x:c r="G6" s="16"/>
+      <x:c r="H6" s="47"/>
+      <x:c r="I6" s="47"/>
       <x:c r="J6" s="47" t="str">
         <x:v>미조사</x:v>
       </x:c>
-      <x:c r="K6" s="47" t="str"/>
-      <x:c r="L6" s="47" t="str"/>
-      <x:c r="M6" s="47" t="str"/>
+      <x:c r="K6" s="47"/>
+      <x:c r="L6" s="47"/>
+      <x:c r="M6" s="47"/>
       <x:c r="N6" s="47" t="str">
         <x:v>90분</x:v>
       </x:c>
@@ -6408,12 +6446,12 @@
         <x:v>차량 반납·공항 이동·수하물</x:v>
       </x:c>
       <x:c r="P6" s="47" t="str">
-        <x:v>철도/항공 대체 비교</x:v>
+        <x:v>이동수단·차량 반납지 확정 후 실행</x:v>
       </x:c>
       <x:c r="Q6" s="47" t="str">
         <x:v>05/06</x:v>
       </x:c>
-      <x:c r="R6" s="61" t="str"/>
+      <x:c r="R6" s="61"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="15" t="str">
@@ -6884,7 +6922,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="str">
-        <x:v>Girona</x:v>
+        <x:v>Bàscara</x:v>
       </x:c>
       <x:c r="B5" s="37" t="n">
         <x:v>46266</x:v>
@@ -6896,38 +6934,42 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E5" s="16" t="str">
-        <x:v>미조사</x:v>
+        <x:v>예약완료</x:v>
       </x:c>
       <x:c r="F5" s="47" t="str">
-        <x:v>역–Plaça Catalunya–Gran Via</x:v>
+        <x:v>Airbnb · 바스카라의 B&amp;B</x:v>
       </x:c>
       <x:c r="G5" s="47" t="str">
         <x:v>EUR</x:v>
       </x:c>
       <x:c r="H5" s="62"/>
       <x:c r="I5" s="62"/>
-      <x:c r="J5" s="62" t="str">
-        <x:f>IF(OR(I5="",D5=0),"",I5/D5)</x:f>
-      </x:c>
-      <x:c r="K5" s="61" t="str"/>
-      <x:c r="L5" s="47" t="str"/>
-      <x:c r="M5" s="47" t="str"/>
-      <x:c r="N5" s="47" t="str"/>
+      <x:c r="J5" s="62"/>
+      <x:c r="K5" s="61"/>
+      <x:c r="L5" s="47"/>
+      <x:c r="M5" s="47" t="str">
+        <x:v>Plaça de l’Església, 6, 17483 Bàscara, Catalonia, Spain</x:v>
+      </x:c>
+      <x:c r="N5" s="47" t="str">
+        <x:v>재확인</x:v>
+      </x:c>
       <x:c r="O5" s="47" t="str">
-        <x:v>선택</x:v>
+        <x:v>재확인</x:v>
       </x:c>
       <x:c r="P5" s="47" t="str">
-        <x:v>선택</x:v>
+        <x:v>재확인</x:v>
       </x:c>
       <x:c r="Q5" s="47" t="str">
-        <x:v>필수</x:v>
+        <x:v>재확인</x:v>
       </x:c>
       <x:c r="R5" s="47" t="str">
-        <x:v>확인</x:v>
-      </x:c>
-      <x:c r="S5" s="47" t="str"/>
+        <x:v>재확인</x:v>
+      </x:c>
+      <x:c r="S5" s="47" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Pla%C3%A7a+de+l%27Esgl%C3%A9sia%2C+6%2C+17483+B%C3%A0scara%2C+Spain</x:v>
+      </x:c>
       <x:c r="T5" s="63" t="str">
-        <x:v>렌터카·주차 우선</x:v>
+        <x:v>Jason·Julia · 예약 확정 · 체크인 시간·주차·조식·결제·취소조건 재확인</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -8433,7 +8475,7 @@
       </x:c>
       <x:c r="E6" s="17" t="n">
         <x:f>COUNTIF(Reservations!H4:H200,"예약완료")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -8478,7 +8520,7 @@
       </x:c>
       <x:c r="E9" s="17" t="n">
         <x:f>COUNTIF(Reservations!H4:H200,"미조사")</x:f>
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -8493,7 +8535,7 @@
       </x:c>
       <x:c r="E10" s="20" t="n">
         <x:f>COUNTIFS(Reservations!B4:B200,"숙소",Reservations!H4:H200,"예약완료")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -8639,7 +8681,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R680dd9ed07d84386"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd641977db9464a22"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>

<commit_message>
Add Cadaques and Tossa routes from Bascara
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="Rdfdee7b9696e48a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Itinerary" sheetId="2" r:id="Ra13418291827495b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reservations" sheetId="3" r:id="R8606c74104e8473b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport" sheetId="4" r:id="Re34b6182ecc44699"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accommodation" sheetId="5" r:id="Rdb971fb0678c4baf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rbbaef063f7554d0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publication QA" sheetId="7" r:id="R191d5a09dfd24e07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="8" r:id="R28ded542efc14edd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Maps" sheetId="9" r:id="R1ce3fb6bbd5c40e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photo Rights" sheetId="10" r:id="Rd27520febf8e40cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Shots" sheetId="11" r:id="R84ec1d09c7e94922"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase8 Lock Status" sheetId="12" r:id="R9dfeb7db6d94413a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="1" r:id="R0b641c05b5564c9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Itinerary" sheetId="2" r:id="R2530d53033864a27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reservations" sheetId="3" r:id="R7c27852c6d0344c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transport" sheetId="4" r:id="R49097590a35d4e98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accommodation" sheetId="5" r:id="Rca6fd10b92c64d7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R2c1579d08cd34323"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Publication QA" sheetId="7" r:id="R600a1d529c074c65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="8" r:id="R814eb12ecfa449e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed Maps" sheetId="9" r:id="Rdd692238c64f467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photo Rights" sheetId="10" r:id="R50321a742ed5412c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Shots" sheetId="11" r:id="R935dc7b6946f4c7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase8 Lock Status" sheetId="12" r:id="R99115337dd694de3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -559,7 +559,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3a20c64a5b3e43c5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb3bba96787be4429"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2256,21 +2256,21 @@
       <x:c r="A1" s="110" t="str">
         <x:v>Phase 8 Reservation &amp; Operations Lock Status v1.0</x:v>
       </x:c>
-      <x:c r="B1" s="110" t="str"/>
-      <x:c r="C1" s="110" t="str"/>
-      <x:c r="D1" s="110" t="str"/>
-      <x:c r="E1" s="110" t="str"/>
-      <x:c r="F1" s="110" t="str"/>
-      <x:c r="G1" s="110" t="str"/>
+      <x:c r="B1" s="110"/>
+      <x:c r="C1" s="110"/>
+      <x:c r="D1" s="110"/>
+      <x:c r="E1" s="110"/>
+      <x:c r="F1" s="110"/>
+      <x:c r="G1" s="110"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str"/>
-      <x:c r="B2" t="str"/>
-      <x:c r="C2" t="str"/>
-      <x:c r="D2" t="str"/>
-      <x:c r="E2" t="str"/>
-      <x:c r="F2" t="str"/>
-      <x:c r="G2" t="str"/>
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="114" t="str">
@@ -2383,7 +2383,7 @@
       <x:c r="F7" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G7" s="47" t="str"/>
+      <x:c r="G7" s="47"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="47" t="str">
@@ -2404,7 +2404,7 @@
       <x:c r="F8" s="47" t="str">
         <x:v>사용자 결정</x:v>
       </x:c>
-      <x:c r="G8" s="47" t="str"/>
+      <x:c r="G8" s="47"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="47" t="str">
@@ -2425,7 +2425,7 @@
       <x:c r="F9" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G9" s="47" t="str"/>
+      <x:c r="G9" s="47"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="47" t="str">
@@ -2446,7 +2446,7 @@
       <x:c r="F10" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G10" s="47" t="str"/>
+      <x:c r="G10" s="47"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="47" t="str">
@@ -2467,7 +2467,7 @@
       <x:c r="F11" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G11" s="47" t="str"/>
+      <x:c r="G11" s="47"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="47" t="str">
@@ -2488,7 +2488,7 @@
       <x:c r="F12" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G12" s="47" t="str"/>
+      <x:c r="G12" s="47"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="47" t="str">
@@ -2509,7 +2509,7 @@
       <x:c r="F13" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G13" s="47" t="str"/>
+      <x:c r="G13" s="47"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="47" t="str">
@@ -2553,7 +2553,7 @@
       <x:c r="F15" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G15" s="47" t="str"/>
+      <x:c r="G15" s="47"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="47" t="str">
@@ -2574,7 +2574,7 @@
       <x:c r="F16" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G16" s="47" t="str"/>
+      <x:c r="G16" s="47"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="47" t="str">
@@ -2595,7 +2595,7 @@
       <x:c r="F17" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G17" s="47" t="str"/>
+      <x:c r="G17" s="47"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="47" t="str">
@@ -2616,7 +2616,7 @@
       <x:c r="F18" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G18" s="47" t="str"/>
+      <x:c r="G18" s="47"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="47" t="str">
@@ -2637,7 +2637,7 @@
       <x:c r="F19" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G19" s="47" t="str"/>
+      <x:c r="G19" s="47"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="47" t="str">
@@ -2658,7 +2658,7 @@
       <x:c r="F20" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G20" s="47" t="str"/>
+      <x:c r="G20" s="47"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="47" t="str">
@@ -2679,20 +2679,20 @@
       <x:c r="F21" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G21" s="47" t="str"/>
+      <x:c r="G21" s="47"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="47" t="str">
         <x:v>티켓</x:v>
       </x:c>
       <x:c r="B22" s="47" t="str">
-        <x:v>Peralada</x:v>
+        <x:v>Peralada — 본 일정에서 제외·실제 예약 없음</x:v>
       </x:c>
       <x:c r="C22" s="47" t="str">
-        <x:v>PARTIAL</x:v>
+        <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="D22" s="47" t="str">
-        <x:v>9/2 17:30 계획</x:v>
+        <x:v>본 일정에서 제외·실제 예약 없음</x:v>
       </x:c>
       <x:c r="E22" s="47" t="str">
         <x:v>예약번호·취소조건</x:v>
@@ -2700,7 +2700,7 @@
       <x:c r="F22" s="47" t="str">
         <x:v>사용자 입력</x:v>
       </x:c>
-      <x:c r="G22" s="47" t="str"/>
+      <x:c r="G22" s="47"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="47" t="str">
@@ -2721,7 +2721,7 @@
       <x:c r="F23" s="47" t="str">
         <x:v>사용자 결정</x:v>
       </x:c>
-      <x:c r="G23" s="47" t="str"/>
+      <x:c r="G23" s="47"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2789,6 +2789,29 @@
       <x:c r="Q1" s="32"/>
       <x:c r="R1" s="32"/>
       <x:c r="S1" s="32"/>
+      <x:c r="T1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
+      <x:c r="M2"/>
+      <x:c r="N2"/>
+      <x:c r="O2"/>
+      <x:c r="P2"/>
+      <x:c r="Q2"/>
+      <x:c r="R2"/>
+      <x:c r="S2"/>
+      <x:c r="T2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="12" t="str">
@@ -2848,6 +2871,7 @@
       <x:c r="S3" s="14" t="str">
         <x:v>최종갱신</x:v>
       </x:c>
+      <x:c r="T3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="37" t="n">
@@ -2868,27 +2892,28 @@
       <x:c r="F4" s="47" t="str">
         <x:v>바르셀로나 도착·정착</x:v>
       </x:c>
-      <x:c r="G4" s="47" t="str"/>
-      <x:c r="H4" s="47" t="str"/>
-      <x:c r="I4" s="47" t="str"/>
-      <x:c r="J4" s="47" t="str"/>
-      <x:c r="K4" s="47" t="str"/>
-      <x:c r="L4" s="47" t="str"/>
-      <x:c r="M4" s="47" t="str"/>
+      <x:c r="G4" s="47"/>
+      <x:c r="H4" s="47"/>
+      <x:c r="I4" s="47"/>
+      <x:c r="J4" s="47"/>
+      <x:c r="K4" s="47"/>
+      <x:c r="L4" s="47"/>
+      <x:c r="M4" s="47"/>
       <x:c r="N4" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O4" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P4" s="47" t="str"/>
-      <x:c r="Q4" s="47" t="str"/>
+      <x:c r="P4" s="47"/>
+      <x:c r="Q4" s="47"/>
       <x:c r="R4" s="47" t="str">
         <x:v>04_Barcelona_Sitges_v1.1.md</x:v>
       </x:c>
       <x:c r="S4" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="37" t="n">
@@ -2909,27 +2934,28 @@
       <x:c r="F5" s="47" t="str">
         <x:v>사그라다 파밀리아와 바르셀로나 재방문</x:v>
       </x:c>
-      <x:c r="G5" s="47" t="str"/>
-      <x:c r="H5" s="47" t="str"/>
-      <x:c r="I5" s="47" t="str"/>
-      <x:c r="J5" s="47" t="str"/>
-      <x:c r="K5" s="47" t="str"/>
-      <x:c r="L5" s="47" t="str"/>
-      <x:c r="M5" s="47" t="str"/>
+      <x:c r="G5" s="47"/>
+      <x:c r="H5" s="47"/>
+      <x:c r="I5" s="47"/>
+      <x:c r="J5" s="47"/>
+      <x:c r="K5" s="47"/>
+      <x:c r="L5" s="47"/>
+      <x:c r="M5" s="47"/>
       <x:c r="N5" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O5" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P5" s="47" t="str"/>
-      <x:c r="Q5" s="47" t="str"/>
+      <x:c r="P5" s="47"/>
+      <x:c r="Q5" s="47"/>
       <x:c r="R5" s="47" t="str">
         <x:v>04_Barcelona_Sitges_v1.1.md</x:v>
       </x:c>
       <x:c r="S5" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="37" t="n">
@@ -2950,27 +2976,28 @@
       <x:c r="F6" s="47" t="str">
         <x:v>운동·미술·도서관·생활권</x:v>
       </x:c>
-      <x:c r="G6" s="47" t="str"/>
-      <x:c r="H6" s="47" t="str"/>
-      <x:c r="I6" s="47" t="str"/>
-      <x:c r="J6" s="47" t="str"/>
-      <x:c r="K6" s="47" t="str"/>
-      <x:c r="L6" s="47" t="str"/>
-      <x:c r="M6" s="47" t="str"/>
+      <x:c r="G6" s="47"/>
+      <x:c r="H6" s="47"/>
+      <x:c r="I6" s="47"/>
+      <x:c r="J6" s="47"/>
+      <x:c r="K6" s="47"/>
+      <x:c r="L6" s="47"/>
+      <x:c r="M6" s="47"/>
       <x:c r="N6" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O6" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P6" s="47" t="str"/>
-      <x:c r="Q6" s="47" t="str"/>
+      <x:c r="P6" s="47"/>
+      <x:c r="Q6" s="47"/>
       <x:c r="R6" s="47" t="str">
         <x:v>04_Barcelona_Sitges_v1.1.md</x:v>
       </x:c>
       <x:c r="S6" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="37" t="n">
@@ -3049,14 +3076,14 @@
         <x:v>체류</x:v>
       </x:c>
       <x:c r="F8" s="47" t="str">
-        <x:v>Bàscara→Collioure→Peralada→Bàscara</x:v>
+        <x:v>Collioure → Cadaqués (해안 쪽 우회)</x:v>
       </x:c>
       <x:c r="G8" s="47"/>
       <x:c r="H8" s="47"/>
       <x:c r="I8" s="47"/>
       <x:c r="J8" s="47"/>
       <x:c r="K8" s="47" t="str">
-        <x:v>Bàscara→Collioure→Peralada→Bàscara</x:v>
+        <x:v>Collioure → Cadaqués (해안 쪽 우회)</x:v>
       </x:c>
       <x:c r="L8" s="47" t="str">
         <x:v>없음</x:v>
@@ -3099,14 +3126,14 @@
         <x:v>체류</x:v>
       </x:c>
       <x:c r="F9" s="47" t="str">
-        <x:v>Bàscara→Pals→Peratallada→Calella→Bàscara</x:v>
+        <x:v>Tossa de Mar → Sant Feliu de Guíxols → Pals → Peratallada</x:v>
       </x:c>
       <x:c r="G9" s="47"/>
       <x:c r="H9" s="47"/>
       <x:c r="I9" s="47"/>
       <x:c r="J9" s="47"/>
       <x:c r="K9" s="47" t="str">
-        <x:v>Bàscara→Pals→Peratallada→Calella→Bàscara</x:v>
+        <x:v>Tossa de Mar → Sant Feliu de Guíxols → Pals → Peratallada</x:v>
       </x:c>
       <x:c r="L9" s="47" t="str">
         <x:v>Jason 선택 러닝</x:v>
@@ -3707,27 +3734,28 @@
       <x:c r="F19" s="47" t="str">
         <x:v>Lourmarin/Cucuron 경유·농가 체크인</x:v>
       </x:c>
-      <x:c r="G19" s="47" t="str"/>
-      <x:c r="H19" s="47" t="str"/>
-      <x:c r="I19" s="47" t="str"/>
-      <x:c r="J19" s="47" t="str"/>
-      <x:c r="K19" s="47" t="str"/>
-      <x:c r="L19" s="47" t="str"/>
-      <x:c r="M19" s="47" t="str"/>
+      <x:c r="G19" s="47"/>
+      <x:c r="H19" s="47"/>
+      <x:c r="I19" s="47"/>
+      <x:c r="J19" s="47"/>
+      <x:c r="K19" s="47"/>
+      <x:c r="L19" s="47"/>
+      <x:c r="M19" s="47"/>
       <x:c r="N19" s="47" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="O19" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P19" s="47" t="str"/>
-      <x:c r="Q19" s="47" t="str"/>
+      <x:c r="P19" s="47"/>
+      <x:c r="Q19" s="47"/>
       <x:c r="R19" s="47" t="str">
         <x:v>08_Luberon_Farmhouse_v1.2.md</x:v>
       </x:c>
       <x:c r="S19" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="37" t="n">
@@ -3748,27 +3776,28 @@
       <x:c r="F20" s="47" t="str">
         <x:v>Luberon 마을·농가생활</x:v>
       </x:c>
-      <x:c r="G20" s="47" t="str"/>
-      <x:c r="H20" s="47" t="str"/>
-      <x:c r="I20" s="47" t="str"/>
-      <x:c r="J20" s="47" t="str"/>
-      <x:c r="K20" s="47" t="str"/>
-      <x:c r="L20" s="47" t="str"/>
-      <x:c r="M20" s="47" t="str"/>
+      <x:c r="G20" s="47"/>
+      <x:c r="H20" s="47"/>
+      <x:c r="I20" s="47"/>
+      <x:c r="J20" s="47"/>
+      <x:c r="K20" s="47"/>
+      <x:c r="L20" s="47"/>
+      <x:c r="M20" s="47"/>
       <x:c r="N20" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O20" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P20" s="47" t="str"/>
-      <x:c r="Q20" s="47" t="str"/>
+      <x:c r="P20" s="47"/>
+      <x:c r="Q20" s="47"/>
       <x:c r="R20" s="47" t="str">
         <x:v>08_Luberon_Farmhouse_v1.2.md</x:v>
       </x:c>
       <x:c r="S20" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T20"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="37" t="n">
@@ -3789,27 +3818,28 @@
       <x:c r="F21" s="47" t="str">
         <x:v>Gordes 권역</x:v>
       </x:c>
-      <x:c r="G21" s="47" t="str"/>
-      <x:c r="H21" s="47" t="str"/>
-      <x:c r="I21" s="47" t="str"/>
-      <x:c r="J21" s="47" t="str"/>
-      <x:c r="K21" s="47" t="str"/>
-      <x:c r="L21" s="47" t="str"/>
-      <x:c r="M21" s="47" t="str"/>
+      <x:c r="G21" s="47"/>
+      <x:c r="H21" s="47"/>
+      <x:c r="I21" s="47"/>
+      <x:c r="J21" s="47"/>
+      <x:c r="K21" s="47"/>
+      <x:c r="L21" s="47"/>
+      <x:c r="M21" s="47"/>
       <x:c r="N21" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O21" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P21" s="47" t="str"/>
-      <x:c r="Q21" s="47" t="str"/>
+      <x:c r="P21" s="47"/>
+      <x:c r="Q21" s="47"/>
       <x:c r="R21" s="47" t="str">
         <x:v>08_Luberon_Farmhouse_v1.2.md</x:v>
       </x:c>
       <x:c r="S21" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T21"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="37" t="n">
@@ -3830,27 +3860,28 @@
       <x:c r="F22" s="47" t="str">
         <x:v>농가생활·스케치·선택마을</x:v>
       </x:c>
-      <x:c r="G22" s="47" t="str"/>
-      <x:c r="H22" s="47" t="str"/>
-      <x:c r="I22" s="47" t="str"/>
-      <x:c r="J22" s="47" t="str"/>
-      <x:c r="K22" s="47" t="str"/>
-      <x:c r="L22" s="47" t="str"/>
-      <x:c r="M22" s="47" t="str"/>
+      <x:c r="G22" s="47"/>
+      <x:c r="H22" s="47"/>
+      <x:c r="I22" s="47"/>
+      <x:c r="J22" s="47"/>
+      <x:c r="K22" s="47"/>
+      <x:c r="L22" s="47"/>
+      <x:c r="M22" s="47"/>
       <x:c r="N22" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O22" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P22" s="47" t="str"/>
-      <x:c r="Q22" s="47" t="str"/>
+      <x:c r="P22" s="47"/>
+      <x:c r="Q22" s="47"/>
       <x:c r="R22" s="47" t="str">
         <x:v>08_Luberon_Farmhouse_v1.2.md</x:v>
       </x:c>
       <x:c r="S22" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T22"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="37" t="n">
@@ -3871,27 +3902,28 @@
       <x:c r="F23" s="47" t="str">
         <x:v>Luberon→Avignon 이동</x:v>
       </x:c>
-      <x:c r="G23" s="47" t="str"/>
-      <x:c r="H23" s="47" t="str"/>
-      <x:c r="I23" s="47" t="str"/>
-      <x:c r="J23" s="47" t="str"/>
-      <x:c r="K23" s="47" t="str"/>
-      <x:c r="L23" s="47" t="str"/>
-      <x:c r="M23" s="47" t="str"/>
+      <x:c r="G23" s="47"/>
+      <x:c r="H23" s="47"/>
+      <x:c r="I23" s="47"/>
+      <x:c r="J23" s="47"/>
+      <x:c r="K23" s="47"/>
+      <x:c r="L23" s="47"/>
+      <x:c r="M23" s="47"/>
       <x:c r="N23" s="47" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="O23" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P23" s="47" t="str"/>
-      <x:c r="Q23" s="47" t="str"/>
+      <x:c r="P23" s="47"/>
+      <x:c r="Q23" s="47"/>
       <x:c r="R23" s="47" t="str">
         <x:v>09_Avignon_Alpilles_Pont_du_Gard_v1.1.md</x:v>
       </x:c>
       <x:c r="S23" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T23"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="37" t="n">
@@ -3912,27 +3944,28 @@
       <x:c r="F24" s="47" t="str">
         <x:v>Avignon 핵심</x:v>
       </x:c>
-      <x:c r="G24" s="47" t="str"/>
-      <x:c r="H24" s="47" t="str"/>
-      <x:c r="I24" s="47" t="str"/>
-      <x:c r="J24" s="47" t="str"/>
-      <x:c r="K24" s="47" t="str"/>
-      <x:c r="L24" s="47" t="str"/>
-      <x:c r="M24" s="47" t="str"/>
+      <x:c r="G24" s="47"/>
+      <x:c r="H24" s="47"/>
+      <x:c r="I24" s="47"/>
+      <x:c r="J24" s="47"/>
+      <x:c r="K24" s="47"/>
+      <x:c r="L24" s="47"/>
+      <x:c r="M24" s="47"/>
       <x:c r="N24" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O24" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P24" s="47" t="str"/>
-      <x:c r="Q24" s="47" t="str"/>
+      <x:c r="P24" s="47"/>
+      <x:c r="Q24" s="47"/>
       <x:c r="R24" s="47" t="str">
         <x:v>09_Avignon_Alpilles_Pont_du_Gard_v1.1.md</x:v>
       </x:c>
       <x:c r="S24" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T24"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="37" t="n">
@@ -3953,27 +3986,28 @@
       <x:c r="F25" s="47" t="str">
         <x:v>Saint-Rémy·Les Baux</x:v>
       </x:c>
-      <x:c r="G25" s="47" t="str"/>
-      <x:c r="H25" s="47" t="str"/>
-      <x:c r="I25" s="47" t="str"/>
-      <x:c r="J25" s="47" t="str"/>
-      <x:c r="K25" s="47" t="str"/>
-      <x:c r="L25" s="47" t="str"/>
-      <x:c r="M25" s="47" t="str"/>
+      <x:c r="G25" s="47"/>
+      <x:c r="H25" s="47"/>
+      <x:c r="I25" s="47"/>
+      <x:c r="J25" s="47"/>
+      <x:c r="K25" s="47"/>
+      <x:c r="L25" s="47"/>
+      <x:c r="M25" s="47"/>
       <x:c r="N25" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O25" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P25" s="47" t="str"/>
-      <x:c r="Q25" s="47" t="str"/>
+      <x:c r="P25" s="47"/>
+      <x:c r="Q25" s="47"/>
       <x:c r="R25" s="47" t="str">
         <x:v>09_Avignon_Alpilles_Pont_du_Gard_v1.1.md</x:v>
       </x:c>
       <x:c r="S25" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="37" t="n">
@@ -3994,27 +4028,28 @@
       <x:c r="F26" s="47" t="str">
         <x:v>Uzès·Pont du Gard 또는 완충일</x:v>
       </x:c>
-      <x:c r="G26" s="47" t="str"/>
-      <x:c r="H26" s="47" t="str"/>
-      <x:c r="I26" s="47" t="str"/>
-      <x:c r="J26" s="47" t="str"/>
-      <x:c r="K26" s="47" t="str"/>
-      <x:c r="L26" s="47" t="str"/>
-      <x:c r="M26" s="47" t="str"/>
+      <x:c r="G26" s="47"/>
+      <x:c r="H26" s="47"/>
+      <x:c r="I26" s="47"/>
+      <x:c r="J26" s="47"/>
+      <x:c r="K26" s="47"/>
+      <x:c r="L26" s="47"/>
+      <x:c r="M26" s="47"/>
       <x:c r="N26" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O26" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P26" s="47" t="str"/>
-      <x:c r="Q26" s="47" t="str"/>
+      <x:c r="P26" s="47"/>
+      <x:c r="Q26" s="47"/>
       <x:c r="R26" s="47" t="str">
         <x:v>09_Avignon_Alpilles_Pont_du_Gard_v1.1.md</x:v>
       </x:c>
       <x:c r="S26" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T26"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="37" t="n">
@@ -4035,27 +4070,28 @@
       <x:c r="F27" s="47" t="str">
         <x:v>렌터카 반납·TGV·Lyon 도착</x:v>
       </x:c>
-      <x:c r="G27" s="47" t="str"/>
-      <x:c r="H27" s="47" t="str"/>
-      <x:c r="I27" s="47" t="str"/>
-      <x:c r="J27" s="47" t="str"/>
-      <x:c r="K27" s="47" t="str"/>
-      <x:c r="L27" s="47" t="str"/>
-      <x:c r="M27" s="47" t="str"/>
+      <x:c r="G27" s="47"/>
+      <x:c r="H27" s="47"/>
+      <x:c r="I27" s="47"/>
+      <x:c r="J27" s="47"/>
+      <x:c r="K27" s="47"/>
+      <x:c r="L27" s="47"/>
+      <x:c r="M27" s="47"/>
       <x:c r="N27" s="47" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="O27" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P27" s="47" t="str"/>
-      <x:c r="Q27" s="47" t="str"/>
+      <x:c r="P27" s="47"/>
+      <x:c r="Q27" s="47"/>
       <x:c r="R27" s="47" t="str">
         <x:v>10_Lyon_v1.2.md</x:v>
       </x:c>
       <x:c r="S27" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T27"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="37" t="n">
@@ -4076,27 +4112,28 @@
       <x:c r="F28" s="47" t="str">
         <x:v>Fourvière·Vieux Lyon</x:v>
       </x:c>
-      <x:c r="G28" s="47" t="str"/>
-      <x:c r="H28" s="47" t="str"/>
-      <x:c r="I28" s="47" t="str"/>
-      <x:c r="J28" s="47" t="str"/>
-      <x:c r="K28" s="47" t="str"/>
-      <x:c r="L28" s="47" t="str"/>
-      <x:c r="M28" s="47" t="str"/>
+      <x:c r="G28" s="47"/>
+      <x:c r="H28" s="47"/>
+      <x:c r="I28" s="47"/>
+      <x:c r="J28" s="47"/>
+      <x:c r="K28" s="47"/>
+      <x:c r="L28" s="47"/>
+      <x:c r="M28" s="47"/>
       <x:c r="N28" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O28" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P28" s="47" t="str"/>
-      <x:c r="Q28" s="47" t="str"/>
+      <x:c r="P28" s="47"/>
+      <x:c r="Q28" s="47"/>
       <x:c r="R28" s="47" t="str">
         <x:v>10_Lyon_v1.2.md</x:v>
       </x:c>
       <x:c r="S28" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T28"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="37" t="n">
@@ -4117,27 +4154,28 @@
       <x:c r="F29" s="47" t="str">
         <x:v>Annecy 당일치기</x:v>
       </x:c>
-      <x:c r="G29" s="47" t="str"/>
-      <x:c r="H29" s="47" t="str"/>
-      <x:c r="I29" s="47" t="str"/>
-      <x:c r="J29" s="47" t="str"/>
-      <x:c r="K29" s="47" t="str"/>
-      <x:c r="L29" s="47" t="str"/>
-      <x:c r="M29" s="47" t="str"/>
+      <x:c r="G29" s="47"/>
+      <x:c r="H29" s="47"/>
+      <x:c r="I29" s="47"/>
+      <x:c r="J29" s="47"/>
+      <x:c r="K29" s="47"/>
+      <x:c r="L29" s="47"/>
+      <x:c r="M29" s="47"/>
       <x:c r="N29" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O29" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P29" s="47" t="str"/>
-      <x:c r="Q29" s="47" t="str"/>
+      <x:c r="P29" s="47"/>
+      <x:c r="Q29" s="47"/>
       <x:c r="R29" s="47" t="str">
         <x:v>10_Lyon_v1.2.md</x:v>
       </x:c>
       <x:c r="S29" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T29"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="37" t="n">
@@ -4158,27 +4196,28 @@
       <x:c r="F30" s="47" t="str">
         <x:v>Lyon 미술·미식·생활</x:v>
       </x:c>
-      <x:c r="G30" s="47" t="str"/>
-      <x:c r="H30" s="47" t="str"/>
-      <x:c r="I30" s="47" t="str"/>
-      <x:c r="J30" s="47" t="str"/>
-      <x:c r="K30" s="47" t="str"/>
-      <x:c r="L30" s="47" t="str"/>
-      <x:c r="M30" s="47" t="str"/>
+      <x:c r="G30" s="47"/>
+      <x:c r="H30" s="47"/>
+      <x:c r="I30" s="47"/>
+      <x:c r="J30" s="47"/>
+      <x:c r="K30" s="47"/>
+      <x:c r="L30" s="47"/>
+      <x:c r="M30" s="47"/>
       <x:c r="N30" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O30" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P30" s="47" t="str"/>
-      <x:c r="Q30" s="47" t="str"/>
+      <x:c r="P30" s="47"/>
+      <x:c r="Q30" s="47"/>
       <x:c r="R30" s="47" t="str">
         <x:v>10_Lyon_v1.2.md</x:v>
       </x:c>
       <x:c r="S30" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="37" t="n">
@@ -4199,27 +4238,28 @@
       <x:c r="F31" s="47" t="str">
         <x:v>TGV·Paris 체크인·장보기</x:v>
       </x:c>
-      <x:c r="G31" s="47" t="str"/>
-      <x:c r="H31" s="47" t="str"/>
-      <x:c r="I31" s="47" t="str"/>
-      <x:c r="J31" s="47" t="str"/>
-      <x:c r="K31" s="47" t="str"/>
-      <x:c r="L31" s="47" t="str"/>
-      <x:c r="M31" s="47" t="str"/>
+      <x:c r="G31" s="47"/>
+      <x:c r="H31" s="47"/>
+      <x:c r="I31" s="47"/>
+      <x:c r="J31" s="47"/>
+      <x:c r="K31" s="47"/>
+      <x:c r="L31" s="47"/>
+      <x:c r="M31" s="47"/>
       <x:c r="N31" s="47" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="O31" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P31" s="47" t="str"/>
-      <x:c r="Q31" s="47" t="str"/>
+      <x:c r="P31" s="47"/>
+      <x:c r="Q31" s="47"/>
       <x:c r="R31" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S31" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T31"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="37" t="n">
@@ -4240,27 +4280,28 @@
       <x:c r="F32" s="47" t="str">
         <x:v>Paris 미술·세느강 권역 — v1.1 확인</x:v>
       </x:c>
-      <x:c r="G32" s="47" t="str"/>
-      <x:c r="H32" s="47" t="str"/>
-      <x:c r="I32" s="47" t="str"/>
-      <x:c r="J32" s="47" t="str"/>
-      <x:c r="K32" s="47" t="str"/>
-      <x:c r="L32" s="47" t="str"/>
-      <x:c r="M32" s="47" t="str"/>
+      <x:c r="G32" s="47"/>
+      <x:c r="H32" s="47"/>
+      <x:c r="I32" s="47"/>
+      <x:c r="J32" s="47"/>
+      <x:c r="K32" s="47"/>
+      <x:c r="L32" s="47"/>
+      <x:c r="M32" s="47"/>
       <x:c r="N32" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O32" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P32" s="47" t="str"/>
-      <x:c r="Q32" s="47" t="str"/>
+      <x:c r="P32" s="47"/>
+      <x:c r="Q32" s="47"/>
       <x:c r="R32" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S32" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T32"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="37" t="n">
@@ -4281,27 +4322,28 @@
       <x:c r="F33" s="47" t="str">
         <x:v>Paris 생활일·운동</x:v>
       </x:c>
-      <x:c r="G33" s="47" t="str"/>
-      <x:c r="H33" s="47" t="str"/>
-      <x:c r="I33" s="47" t="str"/>
-      <x:c r="J33" s="47" t="str"/>
-      <x:c r="K33" s="47" t="str"/>
-      <x:c r="L33" s="47" t="str"/>
-      <x:c r="M33" s="47" t="str"/>
+      <x:c r="G33" s="47"/>
+      <x:c r="H33" s="47"/>
+      <x:c r="I33" s="47"/>
+      <x:c r="J33" s="47"/>
+      <x:c r="K33" s="47"/>
+      <x:c r="L33" s="47"/>
+      <x:c r="M33" s="47"/>
       <x:c r="N33" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O33" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P33" s="47" t="str"/>
-      <x:c r="Q33" s="47" t="str"/>
+      <x:c r="P33" s="47"/>
+      <x:c r="Q33" s="47"/>
       <x:c r="R33" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S33" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T33"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="37" t="n">
@@ -4322,27 +4364,28 @@
       <x:c r="F34" s="47" t="str">
         <x:v>Paris 대표 미술관·도심</x:v>
       </x:c>
-      <x:c r="G34" s="47" t="str"/>
-      <x:c r="H34" s="47" t="str"/>
-      <x:c r="I34" s="47" t="str"/>
-      <x:c r="J34" s="47" t="str"/>
-      <x:c r="K34" s="47" t="str"/>
-      <x:c r="L34" s="47" t="str"/>
-      <x:c r="M34" s="47" t="str"/>
+      <x:c r="G34" s="47"/>
+      <x:c r="H34" s="47"/>
+      <x:c r="I34" s="47"/>
+      <x:c r="J34" s="47"/>
+      <x:c r="K34" s="47"/>
+      <x:c r="L34" s="47"/>
+      <x:c r="M34" s="47"/>
       <x:c r="N34" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O34" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P34" s="47" t="str"/>
-      <x:c r="Q34" s="47" t="str"/>
+      <x:c r="P34" s="47"/>
+      <x:c r="Q34" s="47"/>
       <x:c r="R34" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S34" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T34"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="37" t="n">
@@ -4363,27 +4406,28 @@
       <x:c r="F35" s="47" t="str">
         <x:v>라틴지구·도서관</x:v>
       </x:c>
-      <x:c r="G35" s="47" t="str"/>
-      <x:c r="H35" s="47" t="str"/>
-      <x:c r="I35" s="47" t="str"/>
-      <x:c r="J35" s="47" t="str"/>
-      <x:c r="K35" s="47" t="str"/>
-      <x:c r="L35" s="47" t="str"/>
-      <x:c r="M35" s="47" t="str"/>
+      <x:c r="G35" s="47"/>
+      <x:c r="H35" s="47"/>
+      <x:c r="I35" s="47"/>
+      <x:c r="J35" s="47"/>
+      <x:c r="K35" s="47"/>
+      <x:c r="L35" s="47"/>
+      <x:c r="M35" s="47"/>
       <x:c r="N35" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O35" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P35" s="47" t="str"/>
-      <x:c r="Q35" s="47" t="str"/>
+      <x:c r="P35" s="47"/>
+      <x:c r="Q35" s="47"/>
       <x:c r="R35" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S35" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T35"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="37" t="n">
@@ -4404,27 +4448,28 @@
       <x:c r="F36" s="47" t="str">
         <x:v>동네 산책·미술</x:v>
       </x:c>
-      <x:c r="G36" s="47" t="str"/>
-      <x:c r="H36" s="47" t="str"/>
-      <x:c r="I36" s="47" t="str"/>
-      <x:c r="J36" s="47" t="str"/>
-      <x:c r="K36" s="47" t="str"/>
-      <x:c r="L36" s="47" t="str"/>
-      <x:c r="M36" s="47" t="str"/>
+      <x:c r="G36" s="47"/>
+      <x:c r="H36" s="47"/>
+      <x:c r="I36" s="47"/>
+      <x:c r="J36" s="47"/>
+      <x:c r="K36" s="47"/>
+      <x:c r="L36" s="47"/>
+      <x:c r="M36" s="47"/>
       <x:c r="N36" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O36" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P36" s="47" t="str"/>
-      <x:c r="Q36" s="47" t="str"/>
+      <x:c r="P36" s="47"/>
+      <x:c r="Q36" s="47"/>
       <x:c r="R36" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S36" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T36"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="37" t="n">
@@ -4445,27 +4490,28 @@
       <x:c r="F37" s="47" t="str">
         <x:v>완충일·공연 후보</x:v>
       </x:c>
-      <x:c r="G37" s="47" t="str"/>
-      <x:c r="H37" s="47" t="str"/>
-      <x:c r="I37" s="47" t="str"/>
-      <x:c r="J37" s="47" t="str"/>
-      <x:c r="K37" s="47" t="str"/>
-      <x:c r="L37" s="47" t="str"/>
-      <x:c r="M37" s="47" t="str"/>
+      <x:c r="G37" s="47"/>
+      <x:c r="H37" s="47"/>
+      <x:c r="I37" s="47"/>
+      <x:c r="J37" s="47"/>
+      <x:c r="K37" s="47"/>
+      <x:c r="L37" s="47"/>
+      <x:c r="M37" s="47"/>
       <x:c r="N37" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O37" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P37" s="47" t="str"/>
-      <x:c r="Q37" s="47" t="str"/>
+      <x:c r="P37" s="47"/>
+      <x:c r="Q37" s="47"/>
       <x:c r="R37" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S37" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T37"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="37" t="n">
@@ -4486,27 +4532,28 @@
       <x:c r="F38" s="47" t="str">
         <x:v>Marais·도시사</x:v>
       </x:c>
-      <x:c r="G38" s="47" t="str"/>
-      <x:c r="H38" s="47" t="str"/>
-      <x:c r="I38" s="47" t="str"/>
-      <x:c r="J38" s="47" t="str"/>
-      <x:c r="K38" s="47" t="str"/>
-      <x:c r="L38" s="47" t="str"/>
-      <x:c r="M38" s="47" t="str"/>
+      <x:c r="G38" s="47"/>
+      <x:c r="H38" s="47"/>
+      <x:c r="I38" s="47"/>
+      <x:c r="J38" s="47"/>
+      <x:c r="K38" s="47"/>
+      <x:c r="L38" s="47"/>
+      <x:c r="M38" s="47"/>
       <x:c r="N38" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O38" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P38" s="47" t="str"/>
-      <x:c r="Q38" s="47" t="str"/>
+      <x:c r="P38" s="47"/>
+      <x:c r="Q38" s="47"/>
       <x:c r="R38" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S38" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T38"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="37" t="n">
@@ -4527,27 +4574,28 @@
       <x:c r="F39" s="47" t="str">
         <x:v>Paris 근교 1</x:v>
       </x:c>
-      <x:c r="G39" s="47" t="str"/>
-      <x:c r="H39" s="47" t="str"/>
-      <x:c r="I39" s="47" t="str"/>
-      <x:c r="J39" s="47" t="str"/>
-      <x:c r="K39" s="47" t="str"/>
-      <x:c r="L39" s="47" t="str"/>
-      <x:c r="M39" s="47" t="str"/>
+      <x:c r="G39" s="47"/>
+      <x:c r="H39" s="47"/>
+      <x:c r="I39" s="47"/>
+      <x:c r="J39" s="47"/>
+      <x:c r="K39" s="47"/>
+      <x:c r="L39" s="47"/>
+      <x:c r="M39" s="47"/>
       <x:c r="N39" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O39" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P39" s="47" t="str"/>
-      <x:c r="Q39" s="47" t="str"/>
+      <x:c r="P39" s="47"/>
+      <x:c r="Q39" s="47"/>
       <x:c r="R39" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S39" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T39"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="37" t="n">
@@ -4568,27 +4616,28 @@
       <x:c r="F40" s="47" t="str">
         <x:v>생활일·시장·스케치</x:v>
       </x:c>
-      <x:c r="G40" s="47" t="str"/>
-      <x:c r="H40" s="47" t="str"/>
-      <x:c r="I40" s="47" t="str"/>
-      <x:c r="J40" s="47" t="str"/>
-      <x:c r="K40" s="47" t="str"/>
-      <x:c r="L40" s="47" t="str"/>
-      <x:c r="M40" s="47" t="str"/>
+      <x:c r="G40" s="47"/>
+      <x:c r="H40" s="47"/>
+      <x:c r="I40" s="47"/>
+      <x:c r="J40" s="47"/>
+      <x:c r="K40" s="47"/>
+      <x:c r="L40" s="47"/>
+      <x:c r="M40" s="47"/>
       <x:c r="N40" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O40" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P40" s="47" t="str"/>
-      <x:c r="Q40" s="47" t="str"/>
+      <x:c r="P40" s="47"/>
+      <x:c r="Q40" s="47"/>
       <x:c r="R40" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S40" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T40"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="37" t="n">
@@ -4609,27 +4658,28 @@
       <x:c r="F41" s="47" t="str">
         <x:v>현대미술·건축</x:v>
       </x:c>
-      <x:c r="G41" s="47" t="str"/>
-      <x:c r="H41" s="47" t="str"/>
-      <x:c r="I41" s="47" t="str"/>
-      <x:c r="J41" s="47" t="str"/>
-      <x:c r="K41" s="47" t="str"/>
-      <x:c r="L41" s="47" t="str"/>
-      <x:c r="M41" s="47" t="str"/>
+      <x:c r="G41" s="47"/>
+      <x:c r="H41" s="47"/>
+      <x:c r="I41" s="47"/>
+      <x:c r="J41" s="47"/>
+      <x:c r="K41" s="47"/>
+      <x:c r="L41" s="47"/>
+      <x:c r="M41" s="47"/>
       <x:c r="N41" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O41" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P41" s="47" t="str"/>
-      <x:c r="Q41" s="47" t="str"/>
+      <x:c r="P41" s="47"/>
+      <x:c r="Q41" s="47"/>
       <x:c r="R41" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S41" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T41"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="37" t="n">
@@ -4650,27 +4700,28 @@
       <x:c r="F42" s="47" t="str">
         <x:v>특별전·미술 일정</x:v>
       </x:c>
-      <x:c r="G42" s="47" t="str"/>
-      <x:c r="H42" s="47" t="str"/>
-      <x:c r="I42" s="47" t="str"/>
-      <x:c r="J42" s="47" t="str"/>
-      <x:c r="K42" s="47" t="str"/>
-      <x:c r="L42" s="47" t="str"/>
-      <x:c r="M42" s="47" t="str"/>
+      <x:c r="G42" s="47"/>
+      <x:c r="H42" s="47"/>
+      <x:c r="I42" s="47"/>
+      <x:c r="J42" s="47"/>
+      <x:c r="K42" s="47"/>
+      <x:c r="L42" s="47"/>
+      <x:c r="M42" s="47"/>
       <x:c r="N42" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O42" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P42" s="47" t="str"/>
-      <x:c r="Q42" s="47" t="str"/>
+      <x:c r="P42" s="47"/>
+      <x:c r="Q42" s="47"/>
       <x:c r="R42" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S42" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T42"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="37" t="n">
@@ -4691,27 +4742,28 @@
       <x:c r="F43" s="47" t="str">
         <x:v>Paris 근교 2</x:v>
       </x:c>
-      <x:c r="G43" s="47" t="str"/>
-      <x:c r="H43" s="47" t="str"/>
-      <x:c r="I43" s="47" t="str"/>
-      <x:c r="J43" s="47" t="str"/>
-      <x:c r="K43" s="47" t="str"/>
-      <x:c r="L43" s="47" t="str"/>
-      <x:c r="M43" s="47" t="str"/>
+      <x:c r="G43" s="47"/>
+      <x:c r="H43" s="47"/>
+      <x:c r="I43" s="47"/>
+      <x:c r="J43" s="47"/>
+      <x:c r="K43" s="47"/>
+      <x:c r="L43" s="47"/>
+      <x:c r="M43" s="47"/>
       <x:c r="N43" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O43" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P43" s="47" t="str"/>
-      <x:c r="Q43" s="47" t="str"/>
+      <x:c r="P43" s="47"/>
+      <x:c r="Q43" s="47"/>
       <x:c r="R43" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S43" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T43"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="37" t="n">
@@ -4732,27 +4784,28 @@
       <x:c r="F44" s="47" t="str">
         <x:v>도서관·공연</x:v>
       </x:c>
-      <x:c r="G44" s="47" t="str"/>
-      <x:c r="H44" s="47" t="str"/>
-      <x:c r="I44" s="47" t="str"/>
-      <x:c r="J44" s="47" t="str"/>
-      <x:c r="K44" s="47" t="str"/>
-      <x:c r="L44" s="47" t="str"/>
-      <x:c r="M44" s="47" t="str"/>
+      <x:c r="G44" s="47"/>
+      <x:c r="H44" s="47"/>
+      <x:c r="I44" s="47"/>
+      <x:c r="J44" s="47"/>
+      <x:c r="K44" s="47"/>
+      <x:c r="L44" s="47"/>
+      <x:c r="M44" s="47"/>
       <x:c r="N44" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O44" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P44" s="47" t="str"/>
-      <x:c r="Q44" s="47" t="str"/>
+      <x:c r="P44" s="47"/>
+      <x:c r="Q44" s="47"/>
       <x:c r="R44" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S44" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T44"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="37" t="n">
@@ -4773,27 +4826,28 @@
       <x:c r="F45" s="47" t="str">
         <x:v>자유일·쇼핑·짐정리</x:v>
       </x:c>
-      <x:c r="G45" s="47" t="str"/>
-      <x:c r="H45" s="47" t="str"/>
-      <x:c r="I45" s="47" t="str"/>
-      <x:c r="J45" s="47" t="str"/>
-      <x:c r="K45" s="47" t="str"/>
-      <x:c r="L45" s="47" t="str"/>
-      <x:c r="M45" s="47" t="str"/>
+      <x:c r="G45" s="47"/>
+      <x:c r="H45" s="47"/>
+      <x:c r="I45" s="47"/>
+      <x:c r="J45" s="47"/>
+      <x:c r="K45" s="47"/>
+      <x:c r="L45" s="47"/>
+      <x:c r="M45" s="47"/>
       <x:c r="N45" s="47" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O45" s="47" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P45" s="47" t="str"/>
-      <x:c r="Q45" s="47" t="str"/>
+      <x:c r="P45" s="47"/>
+      <x:c r="Q45" s="47"/>
       <x:c r="R45" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="S45" s="48" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T45"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="37" t="n">
@@ -4805,34 +4859,35 @@
       <x:c r="C46" s="19" t="str">
         <x:v>귀국/기내</x:v>
       </x:c>
-      <x:c r="D46" s="19" t="str"/>
+      <x:c r="D46" s="19"/>
       <x:c r="E46" s="19" t="str">
         <x:v>귀국</x:v>
       </x:c>
       <x:c r="F46" s="49" t="str">
         <x:v>체크아웃·공항·귀국</x:v>
       </x:c>
-      <x:c r="G46" s="49" t="str"/>
-      <x:c r="H46" s="49" t="str"/>
-      <x:c r="I46" s="49" t="str"/>
-      <x:c r="J46" s="49" t="str"/>
-      <x:c r="K46" s="49" t="str"/>
-      <x:c r="L46" s="49" t="str"/>
-      <x:c r="M46" s="49" t="str"/>
+      <x:c r="G46" s="49"/>
+      <x:c r="H46" s="49"/>
+      <x:c r="I46" s="49"/>
+      <x:c r="J46" s="49"/>
+      <x:c r="K46" s="49"/>
+      <x:c r="L46" s="49"/>
+      <x:c r="M46" s="49"/>
       <x:c r="N46" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="O46" s="49" t="str">
         <x:v>초안</x:v>
       </x:c>
-      <x:c r="P46" s="49" t="str"/>
-      <x:c r="Q46" s="49" t="str"/>
+      <x:c r="P46" s="49"/>
+      <x:c r="Q46" s="49"/>
       <x:c r="R46" s="49" t="str">
         <x:v>전체 일정</x:v>
       </x:c>
       <x:c r="S46" s="50" t="n">
         <x:v>46234</x:v>
       </x:c>
+      <x:c r="T46"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4913,6 +4968,30 @@
       <x:c r="U1" s="32"/>
       <x:c r="V1" s="32"/>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
+      <x:c r="M2"/>
+      <x:c r="N2"/>
+      <x:c r="O2"/>
+      <x:c r="P2"/>
+      <x:c r="Q2"/>
+      <x:c r="R2"/>
+      <x:c r="S2"/>
+      <x:c r="T2"/>
+      <x:c r="U2"/>
+      <x:c r="V2"/>
+    </x:row>
     <x:row r="3">
       <x:c r="A3" s="12" t="str">
         <x:v>ID</x:v>
@@ -4997,7 +5076,7 @@
       <x:c r="E4" s="61" t="n">
         <x:v>46263</x:v>
       </x:c>
-      <x:c r="F4" s="47" t="str"/>
+      <x:c r="F4" s="47"/>
       <x:c r="G4" s="47" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -5007,7 +5086,7 @@
       <x:c r="I4" s="61" t="n">
         <x:v>46239</x:v>
       </x:c>
-      <x:c r="J4" s="61" t="str"/>
+      <x:c r="J4" s="61"/>
       <x:c r="K4" s="62"/>
       <x:c r="L4" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5015,21 +5094,19 @@
       <x:c r="M4" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N4" s="62" t="str">
-        <x:f>IF(K4="","",K4-M4)</x:f>
-      </x:c>
-      <x:c r="O4" s="47" t="str"/>
-      <x:c r="P4" s="47" t="str"/>
-      <x:c r="Q4" s="47" t="str"/>
-      <x:c r="R4" s="47" t="str"/>
+      <x:c r="N4" s="62"/>
+      <x:c r="O4" s="47"/>
+      <x:c r="P4" s="47"/>
+      <x:c r="Q4" s="47"/>
+      <x:c r="R4" s="47"/>
       <x:c r="S4" s="47" t="str">
         <x:v>04_Barcelona_Sitges_v1.1.md</x:v>
       </x:c>
       <x:c r="T4" s="47" t="str">
         <x:v>재고·총액·냉방·엘리베이터</x:v>
       </x:c>
-      <x:c r="U4" s="61" t="str"/>
-      <x:c r="V4" s="63" t="str"/>
+      <x:c r="U4" s="61"/>
+      <x:c r="V4" s="63"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="str">
@@ -5119,9 +5196,7 @@
       <x:c r="M6" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N6" s="62" t="str">
-        <x:f>IF(K6="","",K6-M6)</x:f>
-      </x:c>
+      <x:c r="N6" s="62"/>
       <x:c r="O6" s="47"/>
       <x:c r="P6" s="47"/>
       <x:c r="Q6" s="47"/>
@@ -5173,9 +5248,7 @@
       <x:c r="M7" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N7" s="62" t="str">
-        <x:f>IF(K7="","",K7-M7)</x:f>
-      </x:c>
+      <x:c r="N7" s="62"/>
       <x:c r="O7" s="47"/>
       <x:c r="P7" s="47"/>
       <x:c r="Q7" s="47"/>
@@ -5209,7 +5282,7 @@
       <x:c r="E8" s="61" t="n">
         <x:v>46278</x:v>
       </x:c>
-      <x:c r="F8" s="47" t="str"/>
+      <x:c r="F8" s="47"/>
       <x:c r="G8" s="47" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -5219,7 +5292,7 @@
       <x:c r="I8" s="61" t="n">
         <x:v>46239</x:v>
       </x:c>
-      <x:c r="J8" s="61" t="str"/>
+      <x:c r="J8" s="61"/>
       <x:c r="K8" s="62"/>
       <x:c r="L8" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5227,21 +5300,19 @@
       <x:c r="M8" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N8" s="62" t="str">
-        <x:f>IF(K8="","",K8-M8)</x:f>
-      </x:c>
-      <x:c r="O8" s="47" t="str"/>
-      <x:c r="P8" s="47" t="str"/>
-      <x:c r="Q8" s="47" t="str"/>
-      <x:c r="R8" s="47" t="str"/>
+      <x:c r="N8" s="62"/>
+      <x:c r="O8" s="47"/>
+      <x:c r="P8" s="47"/>
+      <x:c r="Q8" s="47"/>
+      <x:c r="R8" s="47"/>
       <x:c r="S8" s="47" t="str">
         <x:v>08_Luberon_Farmhouse_v1.2.md</x:v>
       </x:c>
       <x:c r="T8" s="47" t="str">
         <x:v>수영장 비필수; 입지·주방·세탁·주차 우선</x:v>
       </x:c>
-      <x:c r="U8" s="61" t="str"/>
-      <x:c r="V8" s="63" t="str"/>
+      <x:c r="U8" s="61"/>
+      <x:c r="V8" s="63"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="15" t="str">
@@ -5259,7 +5330,7 @@
       <x:c r="E9" s="61" t="n">
         <x:v>46282</x:v>
       </x:c>
-      <x:c r="F9" s="47" t="str"/>
+      <x:c r="F9" s="47"/>
       <x:c r="G9" s="47" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -5269,7 +5340,7 @@
       <x:c r="I9" s="61" t="n">
         <x:v>46239</x:v>
       </x:c>
-      <x:c r="J9" s="61" t="str"/>
+      <x:c r="J9" s="61"/>
       <x:c r="K9" s="62"/>
       <x:c r="L9" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5277,21 +5348,19 @@
       <x:c r="M9" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N9" s="62" t="str">
-        <x:f>IF(K9="","",K9-M9)</x:f>
-      </x:c>
-      <x:c r="O9" s="47" t="str"/>
-      <x:c r="P9" s="47" t="str"/>
-      <x:c r="Q9" s="47" t="str"/>
-      <x:c r="R9" s="47" t="str"/>
+      <x:c r="N9" s="62"/>
+      <x:c r="O9" s="47"/>
+      <x:c r="P9" s="47"/>
+      <x:c r="Q9" s="47"/>
+      <x:c r="R9" s="47"/>
       <x:c r="S9" s="47" t="str">
         <x:v>09_Avignon_Alpilles_Pont_du_Gard_v1.1.md</x:v>
       </x:c>
       <x:c r="T9" s="47" t="str">
         <x:v>주차·TGV 반납 동선</x:v>
       </x:c>
-      <x:c r="U9" s="61" t="str"/>
-      <x:c r="V9" s="63" t="str"/>
+      <x:c r="U9" s="61"/>
+      <x:c r="V9" s="63"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="15" t="str">
@@ -5309,7 +5378,7 @@
       <x:c r="E10" s="61" t="n">
         <x:v>46286</x:v>
       </x:c>
-      <x:c r="F10" s="47" t="str"/>
+      <x:c r="F10" s="47"/>
       <x:c r="G10" s="47" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -5319,7 +5388,7 @@
       <x:c r="I10" s="61" t="n">
         <x:v>46239</x:v>
       </x:c>
-      <x:c r="J10" s="61" t="str"/>
+      <x:c r="J10" s="61"/>
       <x:c r="K10" s="62"/>
       <x:c r="L10" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5327,21 +5396,19 @@
       <x:c r="M10" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N10" s="62" t="str">
-        <x:f>IF(K10="","",K10-M10)</x:f>
-      </x:c>
-      <x:c r="O10" s="47" t="str"/>
-      <x:c r="P10" s="47" t="str"/>
-      <x:c r="Q10" s="47" t="str"/>
-      <x:c r="R10" s="47" t="str"/>
+      <x:c r="N10" s="62"/>
+      <x:c r="O10" s="47"/>
+      <x:c r="P10" s="47"/>
+      <x:c r="Q10" s="47"/>
+      <x:c r="R10" s="47"/>
       <x:c r="S10" s="47" t="str">
         <x:v>10_Lyon_v1.2.md</x:v>
       </x:c>
       <x:c r="T10" s="47" t="str">
         <x:v>Part-Dieu 접근·야간 귀가</x:v>
       </x:c>
-      <x:c r="U10" s="61" t="str"/>
-      <x:c r="V10" s="63" t="str"/>
+      <x:c r="U10" s="61"/>
+      <x:c r="V10" s="63"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="15" t="str">
@@ -5359,7 +5426,7 @@
       <x:c r="E11" s="61" t="n">
         <x:v>46290</x:v>
       </x:c>
-      <x:c r="F11" s="47" t="str"/>
+      <x:c r="F11" s="47"/>
       <x:c r="G11" s="47" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -5369,7 +5436,7 @@
       <x:c r="I11" s="61" t="n">
         <x:v>46235</x:v>
       </x:c>
-      <x:c r="J11" s="61" t="str"/>
+      <x:c r="J11" s="61"/>
       <x:c r="K11" s="62"/>
       <x:c r="L11" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5377,21 +5444,19 @@
       <x:c r="M11" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N11" s="62" t="str">
-        <x:f>IF(K11="","",K11-M11)</x:f>
-      </x:c>
-      <x:c r="O11" s="47" t="str"/>
-      <x:c r="P11" s="47" t="str"/>
-      <x:c r="Q11" s="47" t="str"/>
-      <x:c r="R11" s="47" t="str"/>
+      <x:c r="N11" s="62"/>
+      <x:c r="O11" s="47"/>
+      <x:c r="P11" s="47"/>
+      <x:c r="Q11" s="47"/>
+      <x:c r="R11" s="47"/>
       <x:c r="S11" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="T11" s="47" t="str">
         <x:v>총액·저층/엘리베이터·세탁·생활권</x:v>
       </x:c>
-      <x:c r="U11" s="61" t="str"/>
-      <x:c r="V11" s="63" t="str"/>
+      <x:c r="U11" s="61"/>
+      <x:c r="V11" s="63"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="15" t="str">
@@ -5409,7 +5474,7 @@
       <x:c r="E12" s="61" t="n">
         <x:v>46266</x:v>
       </x:c>
-      <x:c r="F12" s="47" t="str"/>
+      <x:c r="F12" s="47"/>
       <x:c r="G12" s="47" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -5419,7 +5484,7 @@
       <x:c r="I12" s="61" t="n">
         <x:v>46235</x:v>
       </x:c>
-      <x:c r="J12" s="61" t="str"/>
+      <x:c r="J12" s="61"/>
       <x:c r="K12" s="62"/>
       <x:c r="L12" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5427,21 +5492,19 @@
       <x:c r="M12" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N12" s="62" t="str">
-        <x:f>IF(K12="","",K12-M12)</x:f>
-      </x:c>
-      <x:c r="O12" s="47" t="str"/>
-      <x:c r="P12" s="47" t="str"/>
-      <x:c r="Q12" s="47" t="str"/>
-      <x:c r="R12" s="47" t="str"/>
+      <x:c r="N12" s="62"/>
+      <x:c r="O12" s="47"/>
+      <x:c r="P12" s="47"/>
+      <x:c r="Q12" s="47"/>
+      <x:c r="R12" s="47"/>
       <x:c r="S12" s="47" t="str">
         <x:v>04/05</x:v>
       </x:c>
       <x:c r="T12" s="47" t="str">
         <x:v>짐 노출·국경·반납지</x:v>
       </x:c>
-      <x:c r="U12" s="61" t="str"/>
-      <x:c r="V12" s="63" t="str"/>
+      <x:c r="U12" s="61"/>
+      <x:c r="V12" s="63"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="15" t="str">
@@ -5459,7 +5522,7 @@
       <x:c r="E13" s="61" t="n">
         <x:v>46269</x:v>
       </x:c>
-      <x:c r="F13" s="47" t="str"/>
+      <x:c r="F13" s="47"/>
       <x:c r="G13" s="47" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -5469,7 +5532,7 @@
       <x:c r="I13" s="61" t="n">
         <x:v>46235</x:v>
       </x:c>
-      <x:c r="J13" s="61" t="str"/>
+      <x:c r="J13" s="61"/>
       <x:c r="K13" s="62"/>
       <x:c r="L13" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5477,21 +5540,19 @@
       <x:c r="M13" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N13" s="62" t="str">
-        <x:f>IF(K13="","",K13-M13)</x:f>
-      </x:c>
-      <x:c r="O13" s="47" t="str"/>
-      <x:c r="P13" s="47" t="str"/>
-      <x:c r="Q13" s="47" t="str"/>
-      <x:c r="R13" s="47" t="str"/>
+      <x:c r="N13" s="62"/>
+      <x:c r="O13" s="47"/>
+      <x:c r="P13" s="47"/>
+      <x:c r="Q13" s="47"/>
+      <x:c r="R13" s="47"/>
       <x:c r="S13" s="47" t="str">
         <x:v>05/06</x:v>
       </x:c>
       <x:c r="T13" s="47" t="str">
         <x:v>공항 이동·수하물·차량 반납</x:v>
       </x:c>
-      <x:c r="U13" s="61" t="str"/>
-      <x:c r="V13" s="63" t="str"/>
+      <x:c r="U13" s="61"/>
+      <x:c r="V13" s="63"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="15" t="str">
@@ -5521,7 +5582,7 @@
       <x:c r="I14" s="61" t="n">
         <x:v>46235</x:v>
       </x:c>
-      <x:c r="J14" s="61" t="str"/>
+      <x:c r="J14" s="61"/>
       <x:c r="K14" s="62"/>
       <x:c r="L14" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5529,21 +5590,19 @@
       <x:c r="M14" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N14" s="62" t="str">
-        <x:f>IF(K14="","",K14-M14)</x:f>
-      </x:c>
-      <x:c r="O14" s="47" t="str"/>
-      <x:c r="P14" s="47" t="str"/>
-      <x:c r="Q14" s="47" t="str"/>
-      <x:c r="R14" s="47" t="str"/>
+      <x:c r="N14" s="62"/>
+      <x:c r="O14" s="47"/>
+      <x:c r="P14" s="47"/>
+      <x:c r="Q14" s="47"/>
+      <x:c r="R14" s="47"/>
       <x:c r="S14" s="47" t="str">
         <x:v>06~09</x:v>
       </x:c>
       <x:c r="T14" s="47" t="str">
         <x:v>자동변속·편도수수료·보험·짐</x:v>
       </x:c>
-      <x:c r="U14" s="61" t="str"/>
-      <x:c r="V14" s="63" t="str"/>
+      <x:c r="U14" s="61"/>
+      <x:c r="V14" s="63"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="15" t="str">
@@ -5561,7 +5620,7 @@
       <x:c r="E15" s="61" t="n">
         <x:v>46286</x:v>
       </x:c>
-      <x:c r="F15" s="47" t="str"/>
+      <x:c r="F15" s="47"/>
       <x:c r="G15" s="47" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -5571,7 +5630,7 @@
       <x:c r="I15" s="61" t="n">
         <x:v>46244</x:v>
       </x:c>
-      <x:c r="J15" s="61" t="str"/>
+      <x:c r="J15" s="61"/>
       <x:c r="K15" s="62"/>
       <x:c r="L15" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5579,21 +5638,19 @@
       <x:c r="M15" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N15" s="62" t="str">
-        <x:f>IF(K15="","",K15-M15)</x:f>
-      </x:c>
-      <x:c r="O15" s="47" t="str"/>
-      <x:c r="P15" s="47" t="str"/>
-      <x:c r="Q15" s="47" t="str"/>
-      <x:c r="R15" s="47" t="str"/>
+      <x:c r="N15" s="62"/>
+      <x:c r="O15" s="47"/>
+      <x:c r="P15" s="47"/>
+      <x:c r="Q15" s="47"/>
+      <x:c r="R15" s="47"/>
       <x:c r="S15" s="47" t="str">
         <x:v>09/10</x:v>
       </x:c>
       <x:c r="T15" s="47" t="str">
         <x:v>반납·주유·플랫폼 버퍼</x:v>
       </x:c>
-      <x:c r="U15" s="61" t="str"/>
-      <x:c r="V15" s="63" t="str"/>
+      <x:c r="U15" s="61"/>
+      <x:c r="V15" s="63"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="15" t="str">
@@ -5611,7 +5668,7 @@
       <x:c r="E16" s="61" t="n">
         <x:v>46290</x:v>
       </x:c>
-      <x:c r="F16" s="47" t="str"/>
+      <x:c r="F16" s="47"/>
       <x:c r="G16" s="47" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -5621,7 +5678,7 @@
       <x:c r="I16" s="61" t="n">
         <x:v>46244</x:v>
       </x:c>
-      <x:c r="J16" s="61" t="str"/>
+      <x:c r="J16" s="61"/>
       <x:c r="K16" s="62"/>
       <x:c r="L16" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5629,21 +5686,19 @@
       <x:c r="M16" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N16" s="62" t="str">
-        <x:f>IF(K16="","",K16-M16)</x:f>
-      </x:c>
-      <x:c r="O16" s="47" t="str"/>
-      <x:c r="P16" s="47" t="str"/>
-      <x:c r="Q16" s="47" t="str"/>
-      <x:c r="R16" s="47" t="str"/>
+      <x:c r="N16" s="62"/>
+      <x:c r="O16" s="47"/>
+      <x:c r="P16" s="47"/>
+      <x:c r="Q16" s="47"/>
+      <x:c r="R16" s="47"/>
       <x:c r="S16" s="47" t="str">
         <x:v>10/11</x:v>
       </x:c>
       <x:c r="T16" s="47" t="str">
         <x:v>체크아웃·Paris 체크인</x:v>
       </x:c>
-      <x:c r="U16" s="61" t="str"/>
-      <x:c r="V16" s="63" t="str"/>
+      <x:c r="U16" s="61"/>
+      <x:c r="V16" s="63"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="15" t="str">
@@ -5673,7 +5728,7 @@
       <x:c r="I17" s="61" t="n">
         <x:v>46235</x:v>
       </x:c>
-      <x:c r="J17" s="61" t="str"/>
+      <x:c r="J17" s="61"/>
       <x:c r="K17" s="62"/>
       <x:c r="L17" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5681,34 +5736,32 @@
       <x:c r="M17" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N17" s="62" t="str">
-        <x:f>IF(K17="","",K17-M17)</x:f>
-      </x:c>
-      <x:c r="O17" s="47" t="str"/>
-      <x:c r="P17" s="47" t="str"/>
-      <x:c r="Q17" s="47" t="str"/>
-      <x:c r="R17" s="47" t="str"/>
+      <x:c r="N17" s="62"/>
+      <x:c r="O17" s="47"/>
+      <x:c r="P17" s="47"/>
+      <x:c r="Q17" s="47"/>
+      <x:c r="R17" s="47"/>
       <x:c r="S17" s="47" t="str">
         <x:v>04_Barcelona_Sitges_v1.1.md</x:v>
       </x:c>
       <x:c r="T17" s="47" t="str">
         <x:v>시간지정·성당 운영</x:v>
       </x:c>
-      <x:c r="U17" s="61" t="str"/>
-      <x:c r="V17" s="63" t="str"/>
+      <x:c r="U17" s="61"/>
+      <x:c r="V17" s="63"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="15" t="str">
         <x:v>R015</x:v>
       </x:c>
       <x:c r="B18" s="16" t="str">
-        <x:v>입장권</x:v>
+        <x:v>Peralada — 본 일정에서 제외·실제 예약 없음</x:v>
       </x:c>
       <x:c r="C18" s="16" t="str">
         <x:v>Girona/Peralada</x:v>
       </x:c>
       <x:c r="D18" s="47" t="str">
-        <x:v>Peralada 박물관 투어</x:v>
+        <x:v>Peralada — 본 일정에서 제외·실제 예약 없음</x:v>
       </x:c>
       <x:c r="E18" s="61" t="n">
         <x:v>46267</x:v>
@@ -5720,12 +5773,12 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="H18" s="47" t="str">
-        <x:v>미조사</x:v>
+        <x:v>재확인</x:v>
       </x:c>
       <x:c r="I18" s="61" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="J18" s="61" t="str"/>
+      <x:c r="J18" s="61"/>
       <x:c r="K18" s="62"/>
       <x:c r="L18" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5733,21 +5786,19 @@
       <x:c r="M18" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N18" s="62" t="str">
-        <x:f>IF(K18="","",K18-M18)</x:f>
-      </x:c>
-      <x:c r="O18" s="47" t="str"/>
-      <x:c r="P18" s="47" t="str"/>
-      <x:c r="Q18" s="47" t="str"/>
-      <x:c r="R18" s="47" t="str"/>
+      <x:c r="N18" s="62"/>
+      <x:c r="O18" s="47"/>
+      <x:c r="P18" s="47"/>
+      <x:c r="Q18" s="47"/>
+      <x:c r="R18" s="47"/>
       <x:c r="S18" s="47" t="str">
         <x:v>05_Girona_Collioure_Emporda_v1.1.md</x:v>
       </x:c>
       <x:c r="T18" s="47" t="str">
         <x:v>Collioure 지연 시 취소</x:v>
       </x:c>
-      <x:c r="U18" s="61" t="str"/>
-      <x:c r="V18" s="63" t="str"/>
+      <x:c r="U18" s="61"/>
+      <x:c r="V18" s="63"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="15" t="str">
@@ -5765,7 +5816,7 @@
       <x:c r="E19" s="61" t="n">
         <x:v>46271</x:v>
       </x:c>
-      <x:c r="F19" s="47" t="str"/>
+      <x:c r="F19" s="47"/>
       <x:c r="G19" s="47" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -5775,7 +5826,7 @@
       <x:c r="I19" s="61" t="n">
         <x:v>46259</x:v>
       </x:c>
-      <x:c r="J19" s="61" t="str"/>
+      <x:c r="J19" s="61"/>
       <x:c r="K19" s="62"/>
       <x:c r="L19" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5783,21 +5834,19 @@
       <x:c r="M19" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N19" s="62" t="str">
-        <x:f>IF(K19="","",K19-M19)</x:f>
-      </x:c>
-      <x:c r="O19" s="47" t="str"/>
-      <x:c r="P19" s="47" t="str"/>
-      <x:c r="Q19" s="47" t="str"/>
-      <x:c r="R19" s="47" t="str"/>
+      <x:c r="N19" s="62"/>
+      <x:c r="O19" s="47"/>
+      <x:c r="P19" s="47"/>
+      <x:c r="Q19" s="47"/>
+      <x:c r="R19" s="47"/>
       <x:c r="S19" s="47" t="str">
         <x:v>06_Nice_Cote_d_Azur_v1.2.md</x:v>
       </x:c>
       <x:c r="T19" s="47" t="str">
         <x:v>최신 날짜별 기본안 추출 필요</x:v>
       </x:c>
-      <x:c r="U19" s="61" t="str"/>
-      <x:c r="V19" s="63" t="str"/>
+      <x:c r="U19" s="61"/>
+      <x:c r="V19" s="63"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="15" t="str">
@@ -5815,7 +5864,7 @@
       <x:c r="E20" s="61" t="n">
         <x:v>46277</x:v>
       </x:c>
-      <x:c r="F20" s="47" t="str"/>
+      <x:c r="F20" s="47"/>
       <x:c r="G20" s="47" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -5825,7 +5874,7 @@
       <x:c r="I20" s="61" t="n">
         <x:v>46259</x:v>
       </x:c>
-      <x:c r="J20" s="61" t="str"/>
+      <x:c r="J20" s="61"/>
       <x:c r="K20" s="62"/>
       <x:c r="L20" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5833,21 +5882,19 @@
       <x:c r="M20" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N20" s="62" t="str">
-        <x:f>IF(K20="","",K20-M20)</x:f>
-      </x:c>
-      <x:c r="O20" s="47" t="str"/>
-      <x:c r="P20" s="47" t="str"/>
-      <x:c r="Q20" s="47" t="str"/>
-      <x:c r="R20" s="47" t="str"/>
+      <x:c r="N20" s="62"/>
+      <x:c r="O20" s="47"/>
+      <x:c r="P20" s="47"/>
+      <x:c r="Q20" s="47"/>
+      <x:c r="R20" s="47"/>
       <x:c r="S20" s="47" t="str">
         <x:v>07_Aix_en_Provence_v1.1.md</x:v>
       </x:c>
       <x:c r="T20" s="47" t="str">
         <x:v>운영·시간지정 확인</x:v>
       </x:c>
-      <x:c r="U20" s="61" t="str"/>
-      <x:c r="V20" s="63" t="str"/>
+      <x:c r="U20" s="61"/>
+      <x:c r="V20" s="63"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="15" t="str">
@@ -5865,7 +5912,7 @@
       <x:c r="E21" s="61" t="n">
         <x:v>46283</x:v>
       </x:c>
-      <x:c r="F21" s="47" t="str"/>
+      <x:c r="F21" s="47"/>
       <x:c r="G21" s="47" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -5875,7 +5922,7 @@
       <x:c r="I21" s="61" t="n">
         <x:v>46266</x:v>
       </x:c>
-      <x:c r="J21" s="61" t="str"/>
+      <x:c r="J21" s="61"/>
       <x:c r="K21" s="62"/>
       <x:c r="L21" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5883,21 +5930,19 @@
       <x:c r="M21" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N21" s="62" t="str">
-        <x:f>IF(K21="","",K21-M21)</x:f>
-      </x:c>
-      <x:c r="O21" s="47" t="str"/>
-      <x:c r="P21" s="47" t="str"/>
-      <x:c r="Q21" s="47" t="str"/>
-      <x:c r="R21" s="47" t="str"/>
+      <x:c r="N21" s="62"/>
+      <x:c r="O21" s="47"/>
+      <x:c r="P21" s="47"/>
+      <x:c r="Q21" s="47"/>
+      <x:c r="R21" s="47"/>
       <x:c r="S21" s="47" t="str">
         <x:v>09_Avignon_Alpilles_Pont_du_Gard_v1.1.md</x:v>
       </x:c>
       <x:c r="T21" s="47" t="str">
         <x:v>결합권·입장시간</x:v>
       </x:c>
-      <x:c r="U21" s="61" t="str"/>
-      <x:c r="V21" s="63" t="str"/>
+      <x:c r="U21" s="61"/>
+      <x:c r="V21" s="63"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="15" t="str">
@@ -5915,7 +5960,7 @@
       <x:c r="E22" s="61" t="n">
         <x:v>46288</x:v>
       </x:c>
-      <x:c r="F22" s="47" t="str"/>
+      <x:c r="F22" s="47"/>
       <x:c r="G22" s="47" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -5925,7 +5970,7 @@
       <x:c r="I22" s="61" t="n">
         <x:v>46266</x:v>
       </x:c>
-      <x:c r="J22" s="61" t="str"/>
+      <x:c r="J22" s="61"/>
       <x:c r="K22" s="62"/>
       <x:c r="L22" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5933,21 +5978,19 @@
       <x:c r="M22" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N22" s="62" t="str">
-        <x:f>IF(K22="","",K22-M22)</x:f>
-      </x:c>
-      <x:c r="O22" s="47" t="str"/>
-      <x:c r="P22" s="47" t="str"/>
-      <x:c r="Q22" s="47" t="str"/>
-      <x:c r="R22" s="47" t="str"/>
+      <x:c r="N22" s="62"/>
+      <x:c r="O22" s="47"/>
+      <x:c r="P22" s="47"/>
+      <x:c r="Q22" s="47"/>
+      <x:c r="R22" s="47"/>
       <x:c r="S22" s="47" t="str">
         <x:v>10_Lyon_v1.2.md</x:v>
       </x:c>
       <x:c r="T22" s="47" t="str">
         <x:v>왕복시간·혼잡·대체일</x:v>
       </x:c>
-      <x:c r="U22" s="61" t="str"/>
-      <x:c r="V22" s="63" t="str"/>
+      <x:c r="U22" s="61"/>
+      <x:c r="V22" s="63"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="15" t="str">
@@ -5965,7 +6008,7 @@
       <x:c r="E23" s="61" t="n">
         <x:v>46293</x:v>
       </x:c>
-      <x:c r="F23" s="47" t="str"/>
+      <x:c r="F23" s="47"/>
       <x:c r="G23" s="47" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -5975,7 +6018,7 @@
       <x:c r="I23" s="61" t="n">
         <x:v>46259</x:v>
       </x:c>
-      <x:c r="J23" s="61" t="str"/>
+      <x:c r="J23" s="61"/>
       <x:c r="K23" s="62"/>
       <x:c r="L23" s="62" t="str">
         <x:v>EUR</x:v>
@@ -5983,21 +6026,19 @@
       <x:c r="M23" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N23" s="62" t="str">
-        <x:f>IF(K23="","",K23-M23)</x:f>
-      </x:c>
-      <x:c r="O23" s="47" t="str"/>
-      <x:c r="P23" s="47" t="str"/>
-      <x:c r="Q23" s="47" t="str"/>
-      <x:c r="R23" s="47" t="str"/>
+      <x:c r="N23" s="62"/>
+      <x:c r="O23" s="47"/>
+      <x:c r="P23" s="47"/>
+      <x:c r="Q23" s="47"/>
+      <x:c r="R23" s="47"/>
       <x:c r="S23" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="T23" s="47" t="str">
         <x:v>휴관일·특별전 연동</x:v>
       </x:c>
-      <x:c r="U23" s="61" t="str"/>
-      <x:c r="V23" s="63" t="str"/>
+      <x:c r="U23" s="61"/>
+      <x:c r="V23" s="63"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="15" t="str">
@@ -6015,7 +6056,7 @@
       <x:c r="E24" s="61" t="n">
         <x:v>46296</x:v>
       </x:c>
-      <x:c r="F24" s="47" t="str"/>
+      <x:c r="F24" s="47"/>
       <x:c r="G24" s="47" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -6025,7 +6066,7 @@
       <x:c r="I24" s="61" t="n">
         <x:v>46244</x:v>
       </x:c>
-      <x:c r="J24" s="61" t="str"/>
+      <x:c r="J24" s="61"/>
       <x:c r="K24" s="62"/>
       <x:c r="L24" s="62" t="str">
         <x:v>EUR</x:v>
@@ -6033,21 +6074,19 @@
       <x:c r="M24" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N24" s="62" t="str">
-        <x:f>IF(K24="","",K24-M24)</x:f>
-      </x:c>
-      <x:c r="O24" s="47" t="str"/>
-      <x:c r="P24" s="47" t="str"/>
-      <x:c r="Q24" s="47" t="str"/>
-      <x:c r="R24" s="47" t="str"/>
+      <x:c r="N24" s="62"/>
+      <x:c r="O24" s="47"/>
+      <x:c r="P24" s="47"/>
+      <x:c r="Q24" s="47"/>
+      <x:c r="R24" s="47"/>
       <x:c r="S24" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="T24" s="47" t="str">
         <x:v>공연일에 저녁·교통 조정</x:v>
       </x:c>
-      <x:c r="U24" s="61" t="str"/>
-      <x:c r="V24" s="63" t="str"/>
+      <x:c r="U24" s="61"/>
+      <x:c r="V24" s="63"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="15" t="str">
@@ -6065,7 +6104,7 @@
       <x:c r="E25" s="61" t="n">
         <x:v>46299</x:v>
       </x:c>
-      <x:c r="F25" s="47" t="str"/>
+      <x:c r="F25" s="47"/>
       <x:c r="G25" s="47" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -6075,7 +6114,7 @@
       <x:c r="I25" s="61" t="n">
         <x:v>46244</x:v>
       </x:c>
-      <x:c r="J25" s="61" t="str"/>
+      <x:c r="J25" s="61"/>
       <x:c r="K25" s="62"/>
       <x:c r="L25" s="62" t="str">
         <x:v>EUR</x:v>
@@ -6083,21 +6122,19 @@
       <x:c r="M25" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N25" s="62" t="str">
-        <x:f>IF(K25="","",K25-M25)</x:f>
-      </x:c>
-      <x:c r="O25" s="47" t="str"/>
-      <x:c r="P25" s="47" t="str"/>
-      <x:c r="Q25" s="47" t="str"/>
-      <x:c r="R25" s="47" t="str"/>
+      <x:c r="N25" s="62"/>
+      <x:c r="O25" s="47"/>
+      <x:c r="P25" s="47"/>
+      <x:c r="Q25" s="47"/>
+      <x:c r="R25" s="47"/>
       <x:c r="S25" s="47" t="str">
         <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
       </x:c>
       <x:c r="T25" s="47" t="str">
         <x:v>경기일 확정 후 일정 교환</x:v>
       </x:c>
-      <x:c r="U25" s="61" t="str"/>
-      <x:c r="V25" s="63" t="str"/>
+      <x:c r="U25" s="61"/>
+      <x:c r="V25" s="63"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="15" t="str">
@@ -6115,7 +6152,7 @@
       <x:c r="E26" s="61" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="F26" s="47" t="str"/>
+      <x:c r="F26" s="47"/>
       <x:c r="G26" s="47" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -6125,7 +6162,7 @@
       <x:c r="I26" s="61" t="n">
         <x:v>46244</x:v>
       </x:c>
-      <x:c r="J26" s="61" t="str"/>
+      <x:c r="J26" s="61"/>
       <x:c r="K26" s="62"/>
       <x:c r="L26" s="62" t="str">
         <x:v>KRW</x:v>
@@ -6133,21 +6170,19 @@
       <x:c r="M26" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N26" s="62" t="str">
-        <x:f>IF(K26="","",K26-M26)</x:f>
-      </x:c>
-      <x:c r="O26" s="47" t="str"/>
-      <x:c r="P26" s="47" t="str"/>
-      <x:c r="Q26" s="47" t="str"/>
-      <x:c r="R26" s="47" t="str"/>
+      <x:c r="N26" s="62"/>
+      <x:c r="O26" s="47"/>
+      <x:c r="P26" s="47"/>
+      <x:c r="Q26" s="47"/>
+      <x:c r="R26" s="47"/>
       <x:c r="S26" s="47" t="str">
         <x:v>전체</x:v>
       </x:c>
       <x:c r="T26" s="47" t="str">
         <x:v>의료·렌터카·수하물 보장</x:v>
       </x:c>
-      <x:c r="U26" s="61" t="str"/>
-      <x:c r="V26" s="63" t="str"/>
+      <x:c r="U26" s="61"/>
+      <x:c r="V26" s="63"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="18" t="str">
@@ -6165,7 +6200,7 @@
       <x:c r="E27" s="61" t="n">
         <x:v>46259</x:v>
       </x:c>
-      <x:c r="F27" s="49" t="str"/>
+      <x:c r="F27" s="49"/>
       <x:c r="G27" s="49" t="str">
         <x:v>P2</x:v>
       </x:c>
@@ -6175,7 +6210,7 @@
       <x:c r="I27" s="61" t="n">
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="J27" s="61" t="str"/>
+      <x:c r="J27" s="61"/>
       <x:c r="K27" s="65"/>
       <x:c r="L27" s="65" t="str">
         <x:v>KRW</x:v>
@@ -6183,21 +6218,19 @@
       <x:c r="M27" s="65" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N27" s="65" t="str">
-        <x:f>IF(K27="","",K27-M27)</x:f>
-      </x:c>
-      <x:c r="O27" s="49" t="str"/>
-      <x:c r="P27" s="49" t="str"/>
-      <x:c r="Q27" s="49" t="str"/>
-      <x:c r="R27" s="49" t="str"/>
+      <x:c r="N27" s="65"/>
+      <x:c r="O27" s="49"/>
+      <x:c r="P27" s="49"/>
+      <x:c r="Q27" s="49"/>
+      <x:c r="R27" s="49"/>
       <x:c r="S27" s="49" t="str">
         <x:v>전체</x:v>
       </x:c>
       <x:c r="T27" s="49" t="str">
         <x:v>스페인·프랑스 전 구간</x:v>
       </x:c>
-      <x:c r="U27" s="61" t="str"/>
-      <x:c r="V27" s="66" t="str"/>
+      <x:c r="U27" s="61"/>
+      <x:c r="V27" s="66"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -8505,7 +8538,7 @@
       </x:c>
       <x:c r="E8" s="17" t="n">
         <x:f>COUNTIF(Reservations!H4:H200,"재확인")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -8520,7 +8553,7 @@
       </x:c>
       <x:c r="E9" s="17" t="n">
         <x:f>COUNTIF(Reservations!H4:H200,"미조사")</x:f>
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -8681,7 +8714,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd641977db9464a22"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77edbd1592924991"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>

<commit_message>
Rebuild Paris 15-night schedule around three fixed P0 events
Replace the museum-centric Paris plan (Day 28-43) with a schedule
anchored on Il Barbiere di Siviglia (10/1), Qatar Prix de l'Arc de
Triomphe (10/4), and Hamlet (10/9). Add Fashion Week public-route
half-day and Fete des Vendanges de Montmartre. Add event-action
link styles, extend the reservation guard to 28 entries (R001-R028),
and update the operations tracker accordingly.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -4220,7 +4220,7 @@
       <x:c r="T30"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="37" t="n">
+      <x:c r="A31" s="37">
         <x:v>46290</x:v>
       </x:c>
       <x:c r="B31" s="16" t="str">
@@ -4229,40 +4229,58 @@
       <x:c r="C31" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D31" s="16" t="n">
+      <x:c r="D31" s="16">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E31" s="16" t="str">
         <x:v>이동</x:v>
       </x:c>
       <x:c r="F31" s="47" t="str">
-        <x:v>TGV·Paris 체크인·장보기</x:v>
-      </x:c>
-      <x:c r="G31" s="47"/>
-      <x:c r="H31" s="47"/>
-      <x:c r="I31" s="47"/>
-      <x:c r="J31" s="47"/>
-      <x:c r="K31" s="47"/>
-      <x:c r="L31" s="47"/>
-      <x:c r="M31" s="47"/>
-      <x:c r="N31" s="47" t="n">
-        <x:v>5</x:v>
+        <x:v>Lyon→Paris·정착</x:v>
+      </x:c>
+      <x:c r="G31" s="47" t="str">
+        <x:v>Lyon 체크아웃·TGV</x:v>
+      </x:c>
+      <x:c r="H31" s="47" t="str">
+        <x:v>이동 중 가벼운 식사</x:v>
+      </x:c>
+      <x:c r="I31" s="47" t="str">
+        <x:v>체크인·장보기·동네 방향잡기</x:v>
+      </x:c>
+      <x:c r="J31" s="47" t="str">
+        <x:v>무예약·가벼운 동네저녁</x:v>
+      </x:c>
+      <x:c r="K31" s="47" t="str">
+        <x:v>Lyon→Paris·숙소</x:v>
+      </x:c>
+      <x:c r="L31" s="47" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="M31" s="47" t="str">
+        <x:v>숙소권 기록</x:v>
+      </x:c>
+      <x:c r="N31" s="47">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O31" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P31" s="47"/>
-      <x:c r="Q31" s="47"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P31" s="47" t="str">
+        <x:v>R013·R008</x:v>
+      </x:c>
+      <x:c r="Q31" s="47" t="str">
+        <x:v>지연 시 산책 삭제</x:v>
+      </x:c>
       <x:c r="R31" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S31" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S31" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T31"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="37" t="n">
+      <x:c r="A32" s="37">
         <x:v>46291</x:v>
       </x:c>
       <x:c r="B32" s="16" t="str">
@@ -4271,40 +4289,56 @@
       <x:c r="C32" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D32" s="16" t="n">
+      <x:c r="D32" s="16">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E32" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>로컬 라이프</x:v>
       </x:c>
       <x:c r="F32" s="47" t="str">
-        <x:v>Paris 미술·세느강 권역 — v1.1 확인</x:v>
-      </x:c>
-      <x:c r="G32" s="47"/>
-      <x:c r="H32" s="47"/>
-      <x:c r="I32" s="47"/>
-      <x:c r="J32" s="47"/>
-      <x:c r="K32" s="47"/>
-      <x:c r="L32" s="47"/>
-      <x:c r="M32" s="47"/>
-      <x:c r="N32" s="47" t="n">
-        <x:v>3</x:v>
+        <x:v>Saint-Germain·Luxembourg·Seine</x:v>
+      </x:c>
+      <x:c r="G32" s="47" t="str">
+        <x:v>늦은 시작·가벼운 운동</x:v>
+      </x:c>
+      <x:c r="H32" s="47" t="str">
+        <x:v>Saint-Germain 가벼운 점심</x:v>
+      </x:c>
+      <x:c r="I32" s="47" t="str">
+        <x:v>Luxembourg Gardens·Seine 산책</x:v>
+      </x:c>
+      <x:c r="J32" s="47" t="str">
+        <x:v>무예약·Il Barbiere 회차 제외</x:v>
+      </x:c>
+      <x:c r="K32" s="47" t="str">
+        <x:v>도보·메트로</x:v>
+      </x:c>
+      <x:c r="L32" s="47" t="str">
+        <x:v>가벼운 운동</x:v>
+      </x:c>
+      <x:c r="M32" s="47" t="str">
+        <x:v>공원·강변 스케치</x:v>
+      </x:c>
+      <x:c r="N32" s="47">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O32" s="47" t="str">
-        <x:v>초안</x:v>
+        <x:v>검토중</x:v>
       </x:c>
       <x:c r="P32" s="47"/>
-      <x:c r="Q32" s="47"/>
+      <x:c r="Q32" s="47" t="str">
+        <x:v>Luxembourg까지만</x:v>
+      </x:c>
       <x:c r="R32" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S32" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S32" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T32"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="37" t="n">
+      <x:c r="A33" s="37">
         <x:v>46292</x:v>
       </x:c>
       <x:c r="B33" s="16" t="str">
@@ -4313,40 +4347,58 @@
       <x:c r="C33" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D33" s="16" t="n">
+      <x:c r="D33" s="16">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E33" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>방향잡기</x:v>
       </x:c>
       <x:c r="F33" s="47" t="str">
-        <x:v>Paris 생활일·운동</x:v>
-      </x:c>
-      <x:c r="G33" s="47"/>
-      <x:c r="H33" s="47"/>
-      <x:c r="I33" s="47"/>
-      <x:c r="J33" s="47"/>
-      <x:c r="K33" s="47"/>
-      <x:c r="L33" s="47"/>
-      <x:c r="M33" s="47"/>
-      <x:c r="N33" s="47" t="n">
+        <x:v>고전 파리 오리엔테이션</x:v>
+      </x:c>
+      <x:c r="G33" s="47" t="str">
+        <x:v>Tuileries</x:v>
+      </x:c>
+      <x:c r="H33" s="47" t="str">
+        <x:v>Palais Royal 부근</x:v>
+      </x:c>
+      <x:c r="I33" s="47" t="str">
+        <x:v>Palais Royal·Opéra 지구·Garnier 외관/낮 관람</x:v>
+      </x:c>
+      <x:c r="J33" s="47" t="str">
+        <x:v>자유저녁</x:v>
+      </x:c>
+      <x:c r="K33" s="47" t="str">
+        <x:v>도보</x:v>
+      </x:c>
+      <x:c r="L33" s="47" t="str">
+        <x:v>산책</x:v>
+      </x:c>
+      <x:c r="M33" s="47" t="str">
+        <x:v>Palais Royal</x:v>
+      </x:c>
+      <x:c r="N33" s="47">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O33" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P33" s="47"/>
-      <x:c r="Q33" s="47"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P33" s="47" t="str">
+        <x:v>Garnier 조건부</x:v>
+      </x:c>
+      <x:c r="Q33" s="47" t="str">
+        <x:v>Garnier는 외관만</x:v>
+      </x:c>
       <x:c r="R33" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S33" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S33" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T33"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="37" t="n">
+      <x:c r="A34" s="37">
         <x:v>46293</x:v>
       </x:c>
       <x:c r="B34" s="16" t="str">
@@ -4355,40 +4407,56 @@
       <x:c r="C34" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D34" s="16" t="n">
+      <x:c r="D34" s="16">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E34" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>로컬 라이프</x:v>
       </x:c>
       <x:c r="F34" s="47" t="str">
-        <x:v>Paris 대표 미술관·도심</x:v>
-      </x:c>
-      <x:c r="G34" s="47"/>
-      <x:c r="H34" s="47"/>
-      <x:c r="I34" s="47"/>
-      <x:c r="J34" s="47"/>
-      <x:c r="K34" s="47"/>
-      <x:c r="L34" s="47"/>
-      <x:c r="M34" s="47"/>
-      <x:c r="N34" s="47" t="n">
-        <x:v>3</x:v>
+        <x:v>세탁·쇼핑·Fashion Week 개막</x:v>
+      </x:c>
+      <x:c r="G34" s="47" t="str">
+        <x:v>운동·세탁</x:v>
+      </x:c>
+      <x:c r="H34" s="47" t="str">
+        <x:v>숙소 또는 시장</x:v>
+      </x:c>
+      <x:c r="I34" s="47" t="str">
+        <x:v>쇼핑·북마레/주거지 산책</x:v>
+      </x:c>
+      <x:c r="J34" s="47" t="str">
+        <x:v>무예약·Fashion Week 개막 메모</x:v>
+      </x:c>
+      <x:c r="K34" s="47" t="str">
+        <x:v>숙소권·북마레</x:v>
+      </x:c>
+      <x:c r="L34" s="47" t="str">
+        <x:v>운동</x:v>
+      </x:c>
+      <x:c r="M34" s="47" t="str">
+        <x:v>생활기록</x:v>
+      </x:c>
+      <x:c r="N34" s="47">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O34" s="47" t="str">
-        <x:v>초안</x:v>
+        <x:v>검토중</x:v>
       </x:c>
       <x:c r="P34" s="47"/>
-      <x:c r="Q34" s="47"/>
+      <x:c r="Q34" s="47" t="str">
+        <x:v>숙소권 쇼핑만</x:v>
+      </x:c>
       <x:c r="R34" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S34" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S34" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T34"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="37" t="n">
+      <x:c r="A35" s="37">
         <x:v>46294</x:v>
       </x:c>
       <x:c r="B35" s="16" t="str">
@@ -4397,40 +4465,58 @@
       <x:c r="C35" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D35" s="16" t="n">
+      <x:c r="D35" s="16">
         <x:v>5</x:v>
       </x:c>
       <x:c r="E35" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>박물관</x:v>
       </x:c>
       <x:c r="F35" s="47" t="str">
-        <x:v>라틴지구·도서관</x:v>
-      </x:c>
-      <x:c r="G35" s="47"/>
-      <x:c r="H35" s="47"/>
-      <x:c r="I35" s="47"/>
-      <x:c r="J35" s="47"/>
-      <x:c r="K35" s="47"/>
-      <x:c r="L35" s="47"/>
-      <x:c r="M35" s="47"/>
-      <x:c r="N35" s="47" t="n">
+        <x:v>Orsay 또는 Orangerie</x:v>
+      </x:c>
+      <x:c r="G35" s="47" t="str">
+        <x:v>느린 아침</x:v>
+      </x:c>
+      <x:c r="H35" s="47" t="str">
+        <x:v>관람 전 점심</x:v>
+      </x:c>
+      <x:c r="I35" s="47" t="str">
+        <x:v>미술관 한 곳</x:v>
+      </x:c>
+      <x:c r="J35" s="47" t="str">
+        <x:v>저녁 비움</x:v>
+      </x:c>
+      <x:c r="K35" s="47" t="str">
+        <x:v>메트로·도보</x:v>
+      </x:c>
+      <x:c r="L35" s="47" t="str">
+        <x:v>선택 산책</x:v>
+      </x:c>
+      <x:c r="M35" s="47" t="str">
+        <x:v>미술관 스케치</x:v>
+      </x:c>
+      <x:c r="N35" s="47">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O35" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P35" s="47"/>
-      <x:c r="Q35" s="47"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P35" s="47" t="str">
+        <x:v>R020</x:v>
+      </x:c>
+      <x:c r="Q35" s="47" t="str">
+        <x:v>두 번째 관 금지</x:v>
+      </x:c>
       <x:c r="R35" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S35" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S35" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T35"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="37" t="n">
+      <x:c r="A36" s="37">
         <x:v>46295</x:v>
       </x:c>
       <x:c r="B36" s="16" t="str">
@@ -4439,40 +4525,58 @@
       <x:c r="C36" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D36" s="16" t="n">
+      <x:c r="D36" s="16">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E36" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>고정 경험</x:v>
       </x:c>
       <x:c r="F36" s="47" t="str">
-        <x:v>동네 산책·미술</x:v>
-      </x:c>
-      <x:c r="G36" s="47"/>
-      <x:c r="H36" s="47"/>
-      <x:c r="I36" s="47"/>
-      <x:c r="J36" s="47"/>
-      <x:c r="K36" s="47"/>
-      <x:c r="L36" s="47"/>
-      <x:c r="M36" s="47"/>
-      <x:c r="N36" s="47" t="n">
+        <x:v>Fashion Week 공개동선 반일</x:v>
+      </x:c>
+      <x:c r="G36" s="47" t="str">
+        <x:v>여유로운 오전</x:v>
+      </x:c>
+      <x:c r="H36" s="47" t="str">
+        <x:v>Palais de Tokyo 권역</x:v>
+      </x:c>
+      <x:c r="I36" s="47" t="str">
+        <x:v>Palais de Tokyo 일대→Avenue Montaigne→Rue Saint-Honoré→Palais Royal</x:v>
+      </x:c>
+      <x:c r="J36" s="47" t="str">
+        <x:v>늦은 행사 없이 귀가</x:v>
+      </x:c>
+      <x:c r="K36" s="47" t="str">
+        <x:v>도보·메트로</x:v>
+      </x:c>
+      <x:c r="L36" s="47" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="M36" s="47" t="str">
+        <x:v>거리 스타일 기록</x:v>
+      </x:c>
+      <x:c r="N36" s="47">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O36" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P36" s="47"/>
-      <x:c r="Q36" s="47"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P36" s="47" t="str">
+        <x:v>공개행사 재확인</x:v>
+      </x:c>
+      <x:c r="Q36" s="47" t="str">
+        <x:v>공식 공개 팝업만 추가</x:v>
+      </x:c>
       <x:c r="R36" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S36" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S36" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T36"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="37" t="n">
+      <x:c r="A37" s="37">
         <x:v>46296</x:v>
       </x:c>
       <x:c r="B37" s="16" t="str">
@@ -4481,40 +4585,58 @@
       <x:c r="C37" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D37" s="16" t="n">
+      <x:c r="D37" s="16">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E37" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>고정 공연</x:v>
       </x:c>
       <x:c r="F37" s="47" t="str">
-        <x:v>완충일·공연 후보</x:v>
-      </x:c>
-      <x:c r="G37" s="47"/>
-      <x:c r="H37" s="47"/>
-      <x:c r="I37" s="47"/>
-      <x:c r="J37" s="47"/>
-      <x:c r="K37" s="47"/>
-      <x:c r="L37" s="47"/>
-      <x:c r="M37" s="47"/>
-      <x:c r="N37" s="47" t="n">
-        <x:v>3</x:v>
+        <x:v>Rossini 오페라일</x:v>
+      </x:c>
+      <x:c r="G37" s="47" t="str">
+        <x:v>운동·느린 아침</x:v>
+      </x:c>
+      <x:c r="H37" s="47" t="str">
+        <x:v>가벼운 점심</x:v>
+      </x:c>
+      <x:c r="I37" s="47" t="str">
+        <x:v>Place des Vosges·Bastille 산책</x:v>
+      </x:c>
+      <x:c r="J37" s="47" t="str">
+        <x:v>17:30 이른 저녁·18:30–18:45 입장·Il Barbiere 19:30–약 22:45</x:v>
+      </x:c>
+      <x:c r="K37" s="47" t="str">
+        <x:v>Opéra Bastille 왕복</x:v>
+      </x:c>
+      <x:c r="L37" s="47" t="str">
+        <x:v>운동</x:v>
+      </x:c>
+      <x:c r="M37" s="47" t="str">
+        <x:v>Place des Vosges</x:v>
+      </x:c>
+      <x:c r="N37" s="47">
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O37" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P37" s="47"/>
-      <x:c r="Q37" s="47"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P37" s="47" t="str">
+        <x:v>R021</x:v>
+      </x:c>
+      <x:c r="Q37" s="47" t="str">
+        <x:v>10/7 공연 백업</x:v>
+      </x:c>
       <x:c r="R37" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S37" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S37" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T37"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="37" t="n">
+      <x:c r="A38" s="37">
         <x:v>46297</x:v>
       </x:c>
       <x:c r="B38" s="16" t="str">
@@ -4523,40 +4645,56 @@
       <x:c r="C38" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D38" s="16" t="n">
+      <x:c r="D38" s="16">
         <x:v>8</x:v>
       </x:c>
       <x:c r="E38" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>회복·로컬</x:v>
       </x:c>
       <x:c r="F38" s="47" t="str">
-        <x:v>Marais·도시사</x:v>
-      </x:c>
-      <x:c r="G38" s="47"/>
-      <x:c r="H38" s="47"/>
-      <x:c r="I38" s="47"/>
-      <x:c r="J38" s="47"/>
-      <x:c r="K38" s="47"/>
-      <x:c r="L38" s="47"/>
-      <x:c r="M38" s="47"/>
-      <x:c r="N38" s="47" t="n">
-        <x:v>3</x:v>
+        <x:v>오페라 뒤 회복일</x:v>
+      </x:c>
+      <x:c r="G38" s="47" t="str">
+        <x:v>늦은 시작</x:v>
+      </x:c>
+      <x:c r="H38" s="47" t="str">
+        <x:v>시장 또는 숙소</x:v>
+      </x:c>
+      <x:c r="I38" s="47" t="str">
+        <x:v>시장·서점·카페·스케치</x:v>
+      </x:c>
+      <x:c r="J38" s="47" t="str">
+        <x:v>고정행사 없음</x:v>
+      </x:c>
+      <x:c r="K38" s="47" t="str">
+        <x:v>숙소권</x:v>
+      </x:c>
+      <x:c r="L38" s="47" t="str">
+        <x:v>산책 선택</x:v>
+      </x:c>
+      <x:c r="M38" s="47" t="str">
+        <x:v>카페 스케치</x:v>
+      </x:c>
+      <x:c r="N38" s="47">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O38" s="47" t="str">
-        <x:v>초안</x:v>
+        <x:v>검토중</x:v>
       </x:c>
       <x:c r="P38" s="47"/>
-      <x:c r="Q38" s="47"/>
+      <x:c r="Q38" s="47" t="str">
+        <x:v>완전 휴식 가능</x:v>
+      </x:c>
       <x:c r="R38" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S38" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S38" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T38"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="37" t="n">
+      <x:c r="A39" s="37">
         <x:v>46298</x:v>
       </x:c>
       <x:c r="B39" s="16" t="str">
@@ -4565,40 +4703,58 @@
       <x:c r="C39" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D39" s="16" t="n">
+      <x:c r="D39" s="16">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E39" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>유연한 문화</x:v>
       </x:c>
       <x:c r="F39" s="47" t="str">
-        <x:v>Paris 근교 1</x:v>
-      </x:c>
-      <x:c r="G39" s="47"/>
-      <x:c r="H39" s="47"/>
-      <x:c r="I39" s="47"/>
-      <x:c r="J39" s="47"/>
-      <x:c r="K39" s="47"/>
-      <x:c r="L39" s="47"/>
-      <x:c r="M39" s="47"/>
-      <x:c r="N39" s="47" t="n">
-        <x:v>3</x:v>
+        <x:v>박물관·서점·동네 중 하나</x:v>
+      </x:c>
+      <x:c r="G39" s="47" t="str">
+        <x:v>느린 아침</x:v>
+      </x:c>
+      <x:c r="H39" s="47" t="str">
+        <x:v>선택지역 점심</x:v>
+      </x:c>
+      <x:c r="I39" s="47" t="str">
+        <x:v>문화시설 또는 동네 한 곳</x:v>
+      </x:c>
+      <x:c r="J39" s="47" t="str">
+        <x:v>무예약</x:v>
+      </x:c>
+      <x:c r="K39" s="47" t="str">
+        <x:v>시내</x:v>
+      </x:c>
+      <x:c r="L39" s="47" t="str">
+        <x:v>산책</x:v>
+      </x:c>
+      <x:c r="M39" s="47" t="str">
+        <x:v>선택</x:v>
+      </x:c>
+      <x:c r="N39" s="47">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O39" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P39" s="47"/>
-      <x:c r="Q39" s="47"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P39" s="47" t="str">
+        <x:v>R020 조건부</x:v>
+      </x:c>
+      <x:c r="Q39" s="47" t="str">
+        <x:v>Arc 토요일+Hamlet 조합 금지</x:v>
+      </x:c>
       <x:c r="R39" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S39" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S39" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T39"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="37" t="n">
+      <x:c r="A40" s="37">
         <x:v>46299</x:v>
       </x:c>
       <x:c r="B40" s="16" t="str">
@@ -4607,40 +4763,58 @@
       <x:c r="C40" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D40" s="16" t="n">
+      <x:c r="D40" s="16">
         <x:v>10</x:v>
       </x:c>
       <x:c r="E40" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>고정 스포츠</x:v>
       </x:c>
       <x:c r="F40" s="47" t="str">
-        <x:v>생활일·시장·스케치</x:v>
-      </x:c>
-      <x:c r="G40" s="47"/>
-      <x:c r="H40" s="47"/>
-      <x:c r="I40" s="47"/>
-      <x:c r="J40" s="47"/>
-      <x:c r="K40" s="47"/>
-      <x:c r="L40" s="47"/>
-      <x:c r="M40" s="47"/>
-      <x:c r="N40" s="47" t="n">
-        <x:v>3</x:v>
+        <x:v>Qatar Prix de l’Arc 메인 레이스</x:v>
+      </x:c>
+      <x:c r="G40" s="47" t="str">
+        <x:v>ParisLongchamp 이동</x:v>
+      </x:c>
+      <x:c r="H40" s="47" t="str">
+        <x:v>경기장 안 식사</x:v>
+      </x:c>
+      <x:c r="I40" s="47" t="str">
+        <x:v>메인 레이스 데이</x:v>
+      </x:c>
+      <x:c r="J40" s="47" t="str">
+        <x:v>저녁 비움·숙소 직행</x:v>
+      </x:c>
+      <x:c r="K40" s="47" t="str">
+        <x:v>ParisLongchamp 왕복</x:v>
+      </x:c>
+      <x:c r="L40" s="47" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="M40" s="47" t="str">
+        <x:v>레이스 분위기</x:v>
+      </x:c>
+      <x:c r="N40" s="47">
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O40" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P40" s="47"/>
-      <x:c r="Q40" s="47"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P40" s="47" t="str">
+        <x:v>R023</x:v>
+      </x:c>
+      <x:c r="Q40" s="47" t="str">
+        <x:v>취소 시 공원·스케치</x:v>
+      </x:c>
       <x:c r="R40" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S40" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S40" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T40"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="37" t="n">
+      <x:c r="A41" s="37">
         <x:v>46300</x:v>
       </x:c>
       <x:c r="B41" s="16" t="str">
@@ -4649,40 +4823,56 @@
       <x:c r="C41" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D41" s="16" t="n">
+      <x:c r="D41" s="16">
         <x:v>11</x:v>
       </x:c>
       <x:c r="E41" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>회복</x:v>
       </x:c>
       <x:c r="F41" s="47" t="str">
-        <x:v>현대미술·건축</x:v>
-      </x:c>
-      <x:c r="G41" s="47"/>
-      <x:c r="H41" s="47"/>
-      <x:c r="I41" s="47"/>
-      <x:c r="J41" s="47"/>
-      <x:c r="K41" s="47"/>
-      <x:c r="L41" s="47"/>
-      <x:c r="M41" s="47"/>
-      <x:c r="N41" s="47" t="n">
-        <x:v>3</x:v>
+        <x:v>Arc 뒤 회복일</x:v>
+      </x:c>
+      <x:c r="G41" s="47" t="str">
+        <x:v>늦은 아침·세탁</x:v>
+      </x:c>
+      <x:c r="H41" s="47" t="str">
+        <x:v>숙소</x:v>
+      </x:c>
+      <x:c r="I41" s="47" t="str">
+        <x:v>장보기·카페·선택 짧은 공원</x:v>
+      </x:c>
+      <x:c r="J41" s="47" t="str">
+        <x:v>무예약</x:v>
+      </x:c>
+      <x:c r="K41" s="47" t="str">
+        <x:v>숙소권</x:v>
+      </x:c>
+      <x:c r="L41" s="47" t="str">
+        <x:v>회복 산책</x:v>
+      </x:c>
+      <x:c r="M41" s="47" t="str">
+        <x:v>카페</x:v>
+      </x:c>
+      <x:c r="N41" s="47">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O41" s="47" t="str">
-        <x:v>초안</x:v>
+        <x:v>검토중</x:v>
       </x:c>
       <x:c r="P41" s="47"/>
-      <x:c r="Q41" s="47"/>
+      <x:c r="Q41" s="47" t="str">
+        <x:v>숙소에서 휴식</x:v>
+      </x:c>
       <x:c r="R41" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S41" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S41" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T41"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="37" t="n">
+      <x:c r="A42" s="37">
         <x:v>46301</x:v>
       </x:c>
       <x:c r="B42" s="16" t="str">
@@ -4691,40 +4881,58 @@
       <x:c r="C42" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D42" s="16" t="n">
+      <x:c r="D42" s="16">
         <x:v>12</x:v>
       </x:c>
       <x:c r="E42" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>로컬 라이프</x:v>
       </x:c>
       <x:c r="F42" s="47" t="str">
-        <x:v>특별전·미술 일정</x:v>
-      </x:c>
-      <x:c r="G42" s="47"/>
-      <x:c r="H42" s="47"/>
-      <x:c r="I42" s="47"/>
-      <x:c r="J42" s="47"/>
-      <x:c r="K42" s="47"/>
-      <x:c r="L42" s="47"/>
-      <x:c r="M42" s="47"/>
-      <x:c r="N42" s="47" t="n">
-        <x:v>3</x:v>
+        <x:v>동부 파리 또는 Hamlet 백업</x:v>
+      </x:c>
+      <x:c r="G42" s="47" t="str">
+        <x:v>Canal Saint-Martin</x:v>
+      </x:c>
+      <x:c r="H42" s="47" t="str">
+        <x:v>동부 파리</x:v>
+      </x:c>
+      <x:c r="I42" s="47" t="str">
+        <x:v>Belleville 또는 다른 동네</x:v>
+      </x:c>
+      <x:c r="J42" s="47" t="str">
+        <x:v>Hamlet 19:30은 10/9 매진 시만</x:v>
+      </x:c>
+      <x:c r="K42" s="47" t="str">
+        <x:v>동부 파리·Bastille 조건부</x:v>
+      </x:c>
+      <x:c r="L42" s="47" t="str">
+        <x:v>산책</x:v>
+      </x:c>
+      <x:c r="M42" s="47" t="str">
+        <x:v>Canal</x:v>
+      </x:c>
+      <x:c r="N42" s="47">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O42" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P42" s="47"/>
-      <x:c r="Q42" s="47"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P42" s="47" t="str">
+        <x:v>R022 백업</x:v>
+      </x:c>
+      <x:c r="Q42" s="47" t="str">
+        <x:v>백업 사용 시 산책 16:30 종료</x:v>
+      </x:c>
       <x:c r="R42" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S42" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S42" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T42"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="37" t="n">
+      <x:c r="A43" s="37">
         <x:v>46302</x:v>
       </x:c>
       <x:c r="B43" s="16" t="str">
@@ -4733,40 +4941,58 @@
       <x:c r="C43" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D43" s="16" t="n">
+      <x:c r="D43" s="16">
         <x:v>13</x:v>
       </x:c>
       <x:c r="E43" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>고정 축제</x:v>
       </x:c>
       <x:c r="F43" s="47" t="str">
-        <x:v>Paris 근교 2</x:v>
-      </x:c>
-      <x:c r="G43" s="47"/>
-      <x:c r="H43" s="47"/>
-      <x:c r="I43" s="47"/>
-      <x:c r="J43" s="47"/>
-      <x:c r="K43" s="47"/>
-      <x:c r="L43" s="47"/>
-      <x:c r="M43" s="47"/>
-      <x:c r="N43" s="47" t="n">
+        <x:v>Fête des Vendanges de Montmartre</x:v>
+      </x:c>
+      <x:c r="G43" s="47" t="str">
+        <x:v>낮 축제·Clos Montmartre 선택</x:v>
+      </x:c>
+      <x:c r="H43" s="47" t="str">
+        <x:v>축제권 가벼운 점심</x:v>
+      </x:c>
+      <x:c r="I43" s="47" t="str">
+        <x:v>포도밭 외관·마켓·골목</x:v>
+      </x:c>
+      <x:c r="J43" s="47" t="str">
+        <x:v>이른 귀가·추가 오페라 없음</x:v>
+      </x:c>
+      <x:c r="K43" s="47" t="str">
+        <x:v>Montmartre 왕복</x:v>
+      </x:c>
+      <x:c r="L43" s="47" t="str">
+        <x:v>언덕 산책</x:v>
+      </x:c>
+      <x:c r="M43" s="47" t="str">
+        <x:v>골목·축제</x:v>
+      </x:c>
+      <x:c r="N43" s="47">
         <x:v>3</x:v>
       </x:c>
       <x:c r="O43" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P43" s="47"/>
-      <x:c r="Q43" s="47"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P43" s="47" t="str">
+        <x:v>R025</x:v>
+      </x:c>
+      <x:c r="Q43" s="47" t="str">
+        <x:v>혼잡 시 17:30 종료</x:v>
+      </x:c>
       <x:c r="R43" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S43" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S43" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T43"/>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="37" t="n">
+      <x:c r="A44" s="37">
         <x:v>46303</x:v>
       </x:c>
       <x:c r="B44" s="16" t="str">
@@ -4775,40 +5001,58 @@
       <x:c r="C44" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D44" s="16" t="n">
+      <x:c r="D44" s="16">
         <x:v>14</x:v>
       </x:c>
       <x:c r="E44" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>선택 문화</x:v>
       </x:c>
       <x:c r="F44" s="47" t="str">
-        <x:v>도서관·공연</x:v>
-      </x:c>
-      <x:c r="G44" s="47"/>
-      <x:c r="H44" s="47"/>
-      <x:c r="I44" s="47"/>
-      <x:c r="J44" s="47"/>
-      <x:c r="K44" s="47"/>
-      <x:c r="L44" s="47"/>
-      <x:c r="M44" s="47"/>
-      <x:c r="N44" s="47" t="n">
-        <x:v>3</x:v>
+        <x:v>Chaillot·Este Mundo 선택</x:v>
+      </x:c>
+      <x:c r="G44" s="47" t="str">
+        <x:v>가벼운 오전</x:v>
+      </x:c>
+      <x:c r="H44" s="47" t="str">
+        <x:v>Trocadéro 부근</x:v>
+      </x:c>
+      <x:c r="I44" s="47" t="str">
+        <x:v>Trocadéro·Chaillot</x:v>
+      </x:c>
+      <x:c r="J44" s="47" t="str">
+        <x:v>Este Mundo 20:30 선택·Wagner 제외</x:v>
+      </x:c>
+      <x:c r="K44" s="47" t="str">
+        <x:v>Chaillot 왕복</x:v>
+      </x:c>
+      <x:c r="L44" s="47" t="str">
+        <x:v>가벼운 산책</x:v>
+      </x:c>
+      <x:c r="M44" s="47" t="str">
+        <x:v>Trocadéro</x:v>
+      </x:c>
+      <x:c r="N44" s="47">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O44" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P44" s="47"/>
-      <x:c r="Q44" s="47"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P44" s="47" t="str">
+        <x:v>R024 조건부</x:v>
+      </x:c>
+      <x:c r="Q44" s="47" t="str">
+        <x:v>피로하면 공연 삭제</x:v>
+      </x:c>
       <x:c r="R44" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S44" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S44" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T44"/>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="37" t="n">
+      <x:c r="A45" s="37">
         <x:v>46304</x:v>
       </x:c>
       <x:c r="B45" s="16" t="str">
@@ -4817,40 +5061,58 @@
       <x:c r="C45" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
-      <x:c r="D45" s="16" t="n">
+      <x:c r="D45" s="16">
         <x:v>15</x:v>
       </x:c>
       <x:c r="E45" s="16" t="str">
-        <x:v>체류</x:v>
+        <x:v>고정 공연</x:v>
       </x:c>
       <x:c r="F45" s="47" t="str">
-        <x:v>자유일·쇼핑·짐정리</x:v>
-      </x:c>
-      <x:c r="G45" s="47"/>
-      <x:c r="H45" s="47"/>
-      <x:c r="I45" s="47"/>
-      <x:c r="J45" s="47"/>
-      <x:c r="K45" s="47"/>
-      <x:c r="L45" s="47"/>
-      <x:c r="M45" s="47"/>
-      <x:c r="N45" s="47" t="n">
-        <x:v>3</x:v>
+        <x:v>Hamlet·최종 포장</x:v>
+      </x:c>
+      <x:c r="G45" s="47" t="str">
+        <x:v>늦은 시작·짐정리</x:v>
+      </x:c>
+      <x:c r="H45" s="47" t="str">
+        <x:v>남은 재료 점심</x:v>
+      </x:c>
+      <x:c r="I45" s="47" t="str">
+        <x:v>가벼운 동네산책·카페·이른 저녁</x:v>
+      </x:c>
+      <x:c r="J45" s="47" t="str">
+        <x:v>Hamlet 19:30·Jazz/교회공연 제외·직접 귀가</x:v>
+      </x:c>
+      <x:c r="K45" s="47" t="str">
+        <x:v>Opéra Bastille 왕복</x:v>
+      </x:c>
+      <x:c r="L45" s="47" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="M45" s="47" t="str">
+        <x:v>동네카페</x:v>
+      </x:c>
+      <x:c r="N45" s="47">
+        <x:v>5</x:v>
       </x:c>
       <x:c r="O45" s="47" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P45" s="47"/>
-      <x:c r="Q45" s="47"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P45" s="47" t="str">
+        <x:v>R022</x:v>
+      </x:c>
+      <x:c r="Q45" s="47" t="str">
+        <x:v>10/6 백업 사용 시 자유저녁</x:v>
+      </x:c>
       <x:c r="R45" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
-      </x:c>
-      <x:c r="S45" s="48" t="n">
-        <x:v>46234</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="S45" s="48">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T45"/>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="37" t="n">
+      <x:c r="A46" s="37">
         <x:v>46305</x:v>
       </x:c>
       <x:c r="B46" s="19" t="str">
@@ -4866,26 +5128,44 @@
       <x:c r="F46" s="49" t="str">
         <x:v>체크아웃·공항·귀국</x:v>
       </x:c>
-      <x:c r="G46" s="49"/>
-      <x:c r="H46" s="49"/>
-      <x:c r="I46" s="49"/>
-      <x:c r="J46" s="49"/>
-      <x:c r="K46" s="49"/>
-      <x:c r="L46" s="49"/>
-      <x:c r="M46" s="49"/>
-      <x:c r="N46" s="49" t="n">
-        <x:v>5</x:v>
+      <x:c r="G46" s="49" t="str">
+        <x:v>체크아웃·짐</x:v>
+      </x:c>
+      <x:c r="H46" s="49" t="str">
+        <x:v>이동 전 가벼운 식사</x:v>
+      </x:c>
+      <x:c r="I46" s="49" t="str">
+        <x:v>안전여유를 둔 공항 이동</x:v>
+      </x:c>
+      <x:c r="J46" s="49" t="str">
+        <x:v>Grand Défilé·고정공연 제외</x:v>
+      </x:c>
+      <x:c r="K46" s="49" t="str">
+        <x:v>Paris→공항</x:v>
+      </x:c>
+      <x:c r="L46" s="49" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="M46" s="49" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="N46" s="49">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="O46" s="49" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-      <x:c r="P46" s="49"/>
-      <x:c r="Q46" s="49"/>
+        <x:v>검토중</x:v>
+      </x:c>
+      <x:c r="P46" s="49" t="str">
+        <x:v>항공·공항이동</x:v>
+      </x:c>
+      <x:c r="Q46" s="49" t="str">
+        <x:v>도심 추가관광 금지</x:v>
+      </x:c>
       <x:c r="R46" s="49" t="str">
         <x:v>전체 일정</x:v>
       </x:c>
-      <x:c r="S46" s="50" t="n">
-        <x:v>46234</x:v>
+      <x:c r="S46" s="50">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="T46"/>
     </x:row>
@@ -6051,186 +6331,418 @@
         <x:v>Paris</x:v>
       </x:c>
       <x:c r="D24" s="47" t="str">
-        <x:v>오페라/클래식/재즈 1~2회</x:v>
-      </x:c>
-      <x:c r="E24" s="61" t="n">
+        <x:v>1/6 Il Barbiere di Siviglia — Opéra Bastille</x:v>
+      </x:c>
+      <x:c r="E24" s="61">
         <x:v>46296</x:v>
       </x:c>
-      <x:c r="F24" s="47"/>
+      <x:c r="F24" s="47" t="str">
+        <x:v>19:30</x:v>
+      </x:c>
       <x:c r="G24" s="47" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="H24" s="47" t="str">
-        <x:v>미조사</x:v>
-      </x:c>
-      <x:c r="I24" s="61" t="n">
-        <x:v>46244</x:v>
+        <x:v>예약대기</x:v>
+      </x:c>
+      <x:c r="I24" s="61">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="J24" s="61"/>
       <x:c r="K24" s="62"/>
       <x:c r="L24" s="62" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="M24" s="62" t="n">
+      <x:c r="M24" s="62">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N24" s="62"/>
       <x:c r="O24" s="47"/>
       <x:c r="P24" s="47"/>
       <x:c r="Q24" s="47"/>
-      <x:c r="R24" s="47"/>
+      <x:c r="R24" s="47" t="str">
+        <x:v>https://billetterie.operadeparis.fr/api/1/redirect/product/performance?id=10229122672727&amp;lang=en</x:v>
+      </x:c>
       <x:c r="S24" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
       </x:c>
       <x:c r="T24" s="47" t="str">
-        <x:v>공연일에 저녁·교통 조정</x:v>
-      </x:c>
-      <x:c r="U24" s="61"/>
-      <x:c r="V24" s="63"/>
+        <x:v>공식판매·공식 재판매만; 10/7 19:30 백업</x:v>
+      </x:c>
+      <x:c r="U24" s="61">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V24" s="63" t="str">
+        <x:v>3h15·이탈리아어·FR/EN 자막·현재 €77–205</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="15" t="str">
         <x:v>R022</x:v>
       </x:c>
       <x:c r="B25" s="16" t="str">
-        <x:v>축구</x:v>
+        <x:v>공연</x:v>
       </x:c>
       <x:c r="C25" s="16" t="str">
         <x:v>Paris</x:v>
       </x:c>
       <x:c r="D25" s="47" t="str">
-        <x:v>축구 경기 후보</x:v>
-      </x:c>
-      <x:c r="E25" s="61" t="n">
-        <x:v>46299</x:v>
-      </x:c>
-      <x:c r="F25" s="47"/>
+        <x:v>2/6 Hamlet — Opéra Bastille</x:v>
+      </x:c>
+      <x:c r="E25" s="61">
+        <x:v>46304</x:v>
+      </x:c>
+      <x:c r="F25" s="47" t="str">
+        <x:v>19:30</x:v>
+      </x:c>
       <x:c r="G25" s="47" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="H25" s="47" t="str">
-        <x:v>미조사</x:v>
-      </x:c>
-      <x:c r="I25" s="61" t="n">
-        <x:v>46244</x:v>
+        <x:v>예약대기</x:v>
+      </x:c>
+      <x:c r="I25" s="61">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="J25" s="61"/>
       <x:c r="K25" s="62"/>
       <x:c r="L25" s="62" t="str">
         <x:v>EUR</x:v>
       </x:c>
-      <x:c r="M25" s="62" t="n">
+      <x:c r="M25" s="62">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N25" s="62"/>
       <x:c r="O25" s="47"/>
       <x:c r="P25" s="47"/>
       <x:c r="Q25" s="47"/>
-      <x:c r="R25" s="47"/>
+      <x:c r="R25" s="47" t="str">
+        <x:v>https://billetterie.operadeparis.fr/api/1/redirect/product/performance?id=10229118155385&amp;lang=en</x:v>
+      </x:c>
       <x:c r="S25" s="47" t="str">
-        <x:v>11_Paris_Long_Stay_v1.1.md</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
       </x:c>
       <x:c r="T25" s="47" t="str">
-        <x:v>경기일 확정 후 일정 교환</x:v>
-      </x:c>
-      <x:c r="U25" s="61"/>
-      <x:c r="V25" s="63"/>
+        <x:v>공식판매·공식 재판매만; 10/6 19:30 백업</x:v>
+      </x:c>
+      <x:c r="U25" s="61">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V25" s="63" t="str">
+        <x:v>3h40·프랑스어·FR/EN 자막·현재 €28–155</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="15" t="str">
         <x:v>R023</x:v>
       </x:c>
       <x:c r="B26" s="16" t="str">
-        <x:v>기타</x:v>
+        <x:v>입장권</x:v>
       </x:c>
       <x:c r="C26" s="16" t="str">
-        <x:v>전체</x:v>
+        <x:v>Paris</x:v>
       </x:c>
       <x:c r="D26" s="47" t="str">
-        <x:v>여행자보험</x:v>
-      </x:c>
-      <x:c r="E26" s="61" t="n">
-        <x:v>46254</x:v>
+        <x:v>3/6 Qatar Prix de l’Arc de Triomphe</x:v>
+      </x:c>
+      <x:c r="E26" s="61">
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="F26" s="47"/>
       <x:c r="G26" s="47" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="H26" s="47" t="str">
-        <x:v>미조사</x:v>
-      </x:c>
-      <x:c r="I26" s="61" t="n">
-        <x:v>46244</x:v>
+        <x:v>예약대기</x:v>
+      </x:c>
+      <x:c r="I26" s="61">
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="J26" s="61"/>
       <x:c r="K26" s="62"/>
       <x:c r="L26" s="62" t="str">
-        <x:v>KRW</x:v>
-      </x:c>
-      <x:c r="M26" s="62" t="n">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="M26" s="62">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N26" s="62"/>
       <x:c r="O26" s="47"/>
       <x:c r="P26" s="47"/>
       <x:c r="Q26" s="47"/>
-      <x:c r="R26" s="47"/>
+      <x:c r="R26" s="47" t="str">
+        <x:v>https://billetterie.france-galop.com/en/event/qatar-prix-de-larc-de-triomphe/</x:v>
+      </x:c>
       <x:c r="S26" s="47" t="str">
-        <x:v>전체</x:v>
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
       </x:c>
       <x:c r="T26" s="47" t="str">
-        <x:v>의료·렌터카·수하물 보장</x:v>
-      </x:c>
-      <x:c r="U26" s="61"/>
-      <x:c r="V26" s="63"/>
+        <x:v>메인 레이스 데이; 저녁행사 금지</x:v>
+      </x:c>
+      <x:c r="U26" s="61">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V26" s="63" t="str">
+        <x:v>France Galop BOOK NOW 확인</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="18" t="str">
         <x:v>R024</x:v>
       </x:c>
       <x:c r="B27" s="19" t="str">
-        <x:v>기타</x:v>
+        <x:v>공연</x:v>
       </x:c>
       <x:c r="C27" s="19" t="str">
-        <x:v>전체</x:v>
+        <x:v>Paris</x:v>
       </x:c>
       <x:c r="D27" s="49" t="str">
-        <x:v>eSIM/통신</x:v>
-      </x:c>
-      <x:c r="E27" s="61" t="n">
-        <x:v>46259</x:v>
-      </x:c>
-      <x:c r="F27" s="49"/>
+        <x:v>4/6 Este Mundo — Chaillot (선택)</x:v>
+      </x:c>
+      <x:c r="E27" s="61">
+        <x:v>46303</x:v>
+      </x:c>
+      <x:c r="F27" s="49" t="str">
+        <x:v>20:30</x:v>
+      </x:c>
       <x:c r="G27" s="49" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="H27" s="49" t="str">
-        <x:v>미조사</x:v>
-      </x:c>
-      <x:c r="I27" s="61" t="n">
-        <x:v>46254</x:v>
+        <x:v>예약대기</x:v>
+      </x:c>
+      <x:c r="I27" s="61">
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="J27" s="61"/>
       <x:c r="K27" s="65"/>
       <x:c r="L27" s="65" t="str">
-        <x:v>KRW</x:v>
-      </x:c>
-      <x:c r="M27" s="65" t="n">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="M27" s="65">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N27" s="65"/>
       <x:c r="O27" s="49"/>
       <x:c r="P27" s="49"/>
       <x:c r="Q27" s="49"/>
-      <x:c r="R27" s="49"/>
+      <x:c r="R27" s="49" t="str">
+        <x:v>https://www.festival-automne.com/fr/edition-2026/bouchra-ouizguen-este-mundo</x:v>
+      </x:c>
       <x:c r="S27" s="49" t="str">
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="T27" s="49" t="str">
+        <x:v>10/7–9 연속 3일 피로를 수용할 때만 구매</x:v>
+      </x:c>
+      <x:c r="U27" s="61">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V27" s="66" t="str">
+        <x:v>1h·현재 €8–25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="18" t="str">
+        <x:v>R025</x:v>
+      </x:c>
+      <x:c r="B28" s="19" t="str">
+        <x:v>입장권</x:v>
+      </x:c>
+      <x:c r="C28" s="19" t="str">
+        <x:v>Paris</x:v>
+      </x:c>
+      <x:c r="D28" s="49" t="str">
+        <x:v>5/6 Clos Montmartre 제한 내부방문</x:v>
+      </x:c>
+      <x:c r="E28" s="61">
+        <x:v>46302</x:v>
+      </x:c>
+      <x:c r="F28" s="49" t="str">
+        <x:v>11:00</x:v>
+      </x:c>
+      <x:c r="G28" s="49" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="H28" s="49" t="str">
+        <x:v>재확인</x:v>
+      </x:c>
+      <x:c r="I28" s="61">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="J28" s="61"/>
+      <x:c r="K28" s="65"/>
+      <x:c r="L28" s="65" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="M28" s="65">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N28" s="65"/>
+      <x:c r="O28" s="49"/>
+      <x:c r="P28" s="49"/>
+      <x:c r="Q28" s="49"/>
+      <x:c r="R28" s="49" t="str">
+        <x:v>https://fetedesvendangesdemontmartre.com/le-programme/</x:v>
+      </x:c>
+      <x:c r="S28" s="49" t="str">
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="T28" s="49" t="str">
+        <x:v>예약 실패 시 외관·축제시장·골목만</x:v>
+      </x:c>
+      <x:c r="U28" s="61">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V28" s="66" t="str">
+        <x:v>공식 프로그램상 9/14 예약 오픈</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="18" t="str">
+        <x:v>R026</x:v>
+      </x:c>
+      <x:c r="B29" s="19" t="str">
+        <x:v>공연</x:v>
+      </x:c>
+      <x:c r="C29" s="19" t="str">
+        <x:v>Paris</x:v>
+      </x:c>
+      <x:c r="D29" s="49" t="str">
+        <x:v>6/6 교회 콘서트 — 정확한 프로그램 확인 후</x:v>
+      </x:c>
+      <x:c r="E29" s="61"/>
+      <x:c r="F29" s="49"/>
+      <x:c r="G29" s="49" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="H29" s="49" t="str">
+        <x:v>재확인</x:v>
+      </x:c>
+      <x:c r="I29" s="61">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="J29" s="61"/>
+      <x:c r="K29" s="65"/>
+      <x:c r="L29" s="65" t="str">
+        <x:v>EUR</x:v>
+      </x:c>
+      <x:c r="M29" s="65">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N29" s="65"/>
+      <x:c r="O29" s="49"/>
+      <x:c r="P29" s="49"/>
+      <x:c r="Q29" s="49"/>
+      <x:c r="R29" s="49"/>
+      <x:c r="S29" s="49" t="str">
+        <x:v>11_Paris_Long_Stay_v2.0.md</x:v>
+      </x:c>
+      <x:c r="T29" s="49" t="str">
+        <x:v>작품·연주자·날짜·공식판매처 검증 전 구매 금지</x:v>
+      </x:c>
+      <x:c r="U29" s="61">
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="V29" s="66" t="str">
+        <x:v>O2 패키지에서만 추가</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="18" t="str">
+        <x:v>R027</x:v>
+      </x:c>
+      <x:c r="B30" s="19" t="str">
+        <x:v>기타</x:v>
+      </x:c>
+      <x:c r="C30" s="19" t="str">
         <x:v>전체</x:v>
       </x:c>
-      <x:c r="T27" s="49" t="str">
+      <x:c r="D30" s="49" t="str">
+        <x:v>여행자보험</x:v>
+      </x:c>
+      <x:c r="E30" s="61">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="F30" s="49"/>
+      <x:c r="G30" s="49" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H30" s="49" t="str">
+        <x:v>미조사</x:v>
+      </x:c>
+      <x:c r="I30" s="61">
+        <x:v>46244</x:v>
+      </x:c>
+      <x:c r="J30" s="61"/>
+      <x:c r="K30" s="65"/>
+      <x:c r="L30" s="65" t="str">
+        <x:v>KRW</x:v>
+      </x:c>
+      <x:c r="M30" s="65">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N30" s="65"/>
+      <x:c r="O30" s="49"/>
+      <x:c r="P30" s="49"/>
+      <x:c r="Q30" s="49"/>
+      <x:c r="R30" s="49"/>
+      <x:c r="S30" s="49" t="str">
+        <x:v>전체</x:v>
+      </x:c>
+      <x:c r="T30" s="49" t="str">
+        <x:v>의료·렌터카·수하물 보장</x:v>
+      </x:c>
+      <x:c r="U30" s="61"/>
+      <x:c r="V30" s="66"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="18" t="str">
+        <x:v>R028</x:v>
+      </x:c>
+      <x:c r="B31" s="19" t="str">
+        <x:v>기타</x:v>
+      </x:c>
+      <x:c r="C31" s="19" t="str">
+        <x:v>전체</x:v>
+      </x:c>
+      <x:c r="D31" s="49" t="str">
+        <x:v>eSIM/통신</x:v>
+      </x:c>
+      <x:c r="E31" s="61">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="F31" s="49"/>
+      <x:c r="G31" s="49" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="H31" s="49" t="str">
+        <x:v>미조사</x:v>
+      </x:c>
+      <x:c r="I31" s="61">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="J31" s="61"/>
+      <x:c r="K31" s="65"/>
+      <x:c r="L31" s="65" t="str">
+        <x:v>KRW</x:v>
+      </x:c>
+      <x:c r="M31" s="65">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N31" s="65"/>
+      <x:c r="O31" s="49"/>
+      <x:c r="P31" s="49"/>
+      <x:c r="Q31" s="49"/>
+      <x:c r="R31" s="49"/>
+      <x:c r="S31" s="49" t="str">
+        <x:v>전체</x:v>
+      </x:c>
+      <x:c r="T31" s="49" t="str">
         <x:v>스페인·프랑스 전 구간</x:v>
       </x:c>
-      <x:c r="U27" s="61"/>
-      <x:c r="V27" s="66"/>
+      <x:c r="U31" s="61"/>
+      <x:c r="V31" s="66"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Scrub private stay exact address from working tree
Replace the Bàscara private stay's exact address, coordinates, and
Google Maps URL with a public approximate area across chapters, maps,
registers, and the tracker. Exact details live only in private copies.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -2531,7 +2531,7 @@
         <x:v>사용자 확정</x:v>
       </x:c>
       <x:c r="G14" s="47" t="str">
-        <x:v>Plaça de l’Església, 6, 17483 Bàscara, Catalonia, Spain</x:v>
+        <x:v>비공개 숙소 · 정확 주소는 개인 보관본에서 확인</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -5144,10 +5144,10 @@
         <x:v>Airbnb</x:v>
       </x:c>
       <x:c r="Q5" s="47" t="str">
-        <x:v>Plaça de l’Església, 6, 17483 Bàscara, Catalonia, Spain</x:v>
+        <x:v>비공개 숙소 · 정확 주소는 개인 보관본에서 확인</x:v>
       </x:c>
       <x:c r="R5" s="47" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Pla%C3%A7a+de+l%27Esgl%C3%A9sia%2C+6%2C+17483+B%C3%A0scara%2C+Spain</x:v>
+        <x:v/>
       </x:c>
       <x:c r="S5" s="47" t="str">
         <x:v>05_Girona_Collioure_Emporda_v2.1.md</x:v>
@@ -6981,7 +6981,7 @@
       <x:c r="K5" s="61"/>
       <x:c r="L5" s="47"/>
       <x:c r="M5" s="47" t="str">
-        <x:v>Plaça de l’Església, 6, 17483 Bàscara, Catalonia, Spain</x:v>
+        <x:v>비공개 숙소 · 정확 주소는 개인 보관본에서 확인</x:v>
       </x:c>
       <x:c r="N5" s="47" t="str">
         <x:v>재확인</x:v>
@@ -6999,7 +6999,7 @@
         <x:v>재확인</x:v>
       </x:c>
       <x:c r="S5" s="47" t="str">
-        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Pla%C3%A7a+de+l%27Esgl%C3%A9sia%2C+6%2C+17483+B%C3%A0scara%2C+Spain</x:v>
+        <x:v/>
       </x:c>
       <x:c r="T5" s="63" t="str">
         <x:v>Jason·Julia · 예약 확정 · 체크인 시간·주차·조식·결제·취소조건 재확인</x:v>

</xml_diff>

<commit_message>
feat: record Barcelona and Bàscara booking details
Barcelona (Occidental Barcelona 1929, Trip.com):
- confirmation 365585SG255002 · booking 1400827967207904
- prepaid KRW 701,054 (VAT incl.) + €46.2 due at hotel (city tax incl.,
  ~KRW 76,428); within the 800k budget
- guard: drop the Barcelona/R001 completed-without-ref exception —
  the row now meets the standard requirements
- remaining 재확인: free-cancellation deadline

Bàscara (Airbnb 바스카라의 B&B):
- check-in 2026-09-01 12:00 · check-out 09-04 11:00 · €330 ·
  code HM2YPHDRW5
- the exact address stays redacted in public files per the standing
  privacy policy (개인 보관본)
- remaining 재확인: payment terms, parking, breakfast, cancellation

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -3588,7 +3588,7 @@
       </c>
       <c r="E13" s="100" t="inlineStr">
         <is>
-          <t>예약번호·금액·취소기한</t>
+          <t>무료취소기한</t>
         </is>
       </c>
       <c r="F13" s="100" t="inlineStr">
@@ -3620,12 +3620,12 @@
       </c>
       <c r="D14" s="100" t="inlineStr">
         <is>
-          <t>Airbnb · 바스카라의 B&amp;B · 2026-09-01~09-04 · 3박</t>
+          <t>Airbnb · 바스카라의 B&amp;B · 2026-09-01 12:00~09-04 11:00 · 3박 · €330 · HM2YPHDRW5</t>
         </is>
       </c>
       <c r="E14" s="100" t="inlineStr">
         <is>
-          <t>확정번호·가격·결제·체크인·주차·조식·취소조건</t>
+          <t>결제·주차·조식·취소조건</t>
         </is>
       </c>
       <c r="F14" s="100" t="inlineStr">
@@ -7737,17 +7737,25 @@
         <v>46239</v>
       </c>
       <c r="J4" s="119" t="n"/>
-      <c r="K4" s="120" t="n"/>
+      <c r="K4" s="120" t="n">
+        <v>701054</v>
+      </c>
       <c r="L4" s="120" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>KRW</t>
         </is>
       </c>
       <c r="M4" s="120" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="120" t="n"/>
-      <c r="O4" s="100" t="n"/>
+        <v>701054</v>
+      </c>
+      <c r="N4" s="120" t="n">
+        <v>76428</v>
+      </c>
+      <c r="O4" s="100" t="inlineStr">
+        <is>
+          <t>365585SG255002 · Trip.com 1400827967207904</t>
+        </is>
+      </c>
       <c r="P4" s="100" t="inlineStr">
         <is>
           <t>Occidental Barcelona 1929</t>
@@ -7778,7 +7786,7 @@
       </c>
       <c r="V4" s="63" t="inlineStr">
         <is>
-          <t>전화 +34 936 26 88 44 · 체크아웃 09:30–12:00 · 예약번호·총액·취소기한 재확인</t>
+          <t>Trip.com 예약 · 전화 +34 936 26 88 44 · 체크아웃 09:30–12:00 · 잔액은 현장 결제 €46.2(도시세 포함)의 원화 환산 약치 · 무료취소기한 재확인</t>
         </is>
       </c>
     </row>
@@ -7806,7 +7814,11 @@
       <c r="E5" s="119" t="n">
         <v>46266</v>
       </c>
-      <c r="F5" s="100" t="n"/>
+      <c r="F5" s="100" t="inlineStr">
+        <is>
+          <t>체크인 12:00</t>
+        </is>
+      </c>
       <c r="G5" s="100" t="inlineStr">
         <is>
           <t>P0</t>
@@ -7819,7 +7831,9 @@
       </c>
       <c r="I5" s="119" t="n"/>
       <c r="J5" s="119" t="n"/>
-      <c r="K5" s="120" t="n"/>
+      <c r="K5" s="120" t="n">
+        <v>330</v>
+      </c>
       <c r="L5" s="120" t="inlineStr">
         <is>
           <t>EUR</t>
@@ -7827,7 +7841,11 @@
       </c>
       <c r="M5" s="120" t="n"/>
       <c r="N5" s="120" t="n"/>
-      <c r="O5" s="100" t="n"/>
+      <c r="O5" s="100" t="inlineStr">
+        <is>
+          <t>HM2YPHDRW5</t>
+        </is>
+      </c>
       <c r="P5" s="100" t="inlineStr">
         <is>
           <t>Airbnb</t>
@@ -7846,11 +7864,11 @@
       </c>
       <c r="T5" s="100" t="inlineStr">
         <is>
-          <t>체크인 시간·주차·조식·결제·취소조건 재확인</t>
+          <t>주차·조식·결제·취소조건 재확인</t>
         </is>
       </c>
       <c r="U5" s="119" t="n">
-        <v>46237</v>
+        <v>46239</v>
       </c>
       <c r="V5" s="63" t="inlineStr">
         <is>
@@ -10664,13 +10682,19 @@
       <c r="H4" s="120" t="n">
         <v>800000</v>
       </c>
-      <c r="I4" s="120" t="n"/>
+      <c r="I4" s="120" t="n">
+        <v>701054</v>
+      </c>
       <c r="J4" s="120">
         <f>IF(OR(I4="",D4=0),"",I4/D4)</f>
         <v/>
       </c>
       <c r="K4" s="119" t="str"/>
-      <c r="L4" s="100" t="str"/>
+      <c r="L4" s="100" t="inlineStr">
+        <is>
+          <t>365585SG255002 · Trip.com 1400827967207904</t>
+        </is>
+      </c>
       <c r="M4" s="100" t="inlineStr">
         <is>
           <t>Carrer de la Creu Coberta, 20-22, 08014 Barcelona, Catalonia, Spain</t>
@@ -10708,7 +10732,7 @@
       </c>
       <c r="T4" s="63" t="inlineStr">
         <is>
-          <t>2인 3박 · 전화 +34 936 26 88 44 · 예약번호·총액·취소기한 재확인</t>
+          <t>2인 3박 · Trip.com 예약 · 전화 +34 936 26 88 44 · 현장 추가결제 €46.2(도시세 포함, 약 KRW 76,428) · 무료취소기한 재확인</t>
         </is>
       </c>
     </row>
@@ -10743,10 +10767,16 @@
         </is>
       </c>
       <c r="H5" s="120" t="n"/>
-      <c r="I5" s="120" t="n"/>
+      <c r="I5" s="120" t="n">
+        <v>330</v>
+      </c>
       <c r="J5" s="120" t="n"/>
       <c r="K5" s="119" t="n"/>
-      <c r="L5" s="100" t="n"/>
+      <c r="L5" s="100" t="inlineStr">
+        <is>
+          <t>HM2YPHDRW5</t>
+        </is>
+      </c>
       <c r="M5" s="100" t="inlineStr">
         <is>
           <t>비공개 숙소 · 정확 주소는 개인 보관본에서 확인</t>
@@ -10754,7 +10784,7 @@
       </c>
       <c r="N5" s="100" t="inlineStr">
         <is>
-          <t>재확인</t>
+          <t>체크인 12:00 · 체크아웃 11:00</t>
         </is>
       </c>
       <c r="O5" s="100" t="inlineStr">
@@ -10780,7 +10810,7 @@
       <c r="S5" s="100" t="n"/>
       <c r="T5" s="63" t="inlineStr">
         <is>
-          <t>Jason·Julia · 예약 확정 · 체크인 시간·주차·조식·결제·취소조건 재확인</t>
+          <t>Jason·Julia · 예약 확정 · €330 · 주차·조식·결제·취소조건 재확인</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(booking): reflect confirmed BCN-NCE flight, two Hertz rentals, Avignon-Lyon TGV
Vueling VY1521 (9/4 15:30 BCN T1 -> 16:55 NCE T1, NMGI4Q), Hertz
L671E2E0288 (9/1 07:00 Sants -> 9/4 14:00 El Prat) and L672E080313
(9/9 09:00 Nice station -> 9/20 09:00 Avignon TGV — pickup moved off
NCE T2), and TGV INOUI 12176 (9/20 10:22 -> 11:28, 1st class) land in
the tracker, master itinerary, execution audit, gate calendar, and the
Nice chapter. Dashboard/accommodation formulas flattened to their
cached values so openpyxl edits keep the build guards readable.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -7582,6 +7582,7 @@
       <c r="U1" s="98" t="n"/>
       <c r="V1" s="98" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -8326,13 +8327,17 @@
       </c>
       <c r="D12" s="100" t="inlineStr">
         <is>
-          <t>BCN 구간 차량 인수·반납</t>
+          <t>BCN 렌터카 — Sants 인수→El Prat 반납</t>
         </is>
       </c>
       <c r="E12" s="119" t="n">
         <v>46266</v>
       </c>
-      <c r="F12" s="100" t="n"/>
+      <c r="F12" s="100" t="inlineStr">
+        <is>
+          <t>9/1 07:00 인수 · 9/4 14:00 반납</t>
+        </is>
+      </c>
       <c r="G12" s="100" t="inlineStr">
         <is>
           <t>P0</t>
@@ -8340,7 +8345,7 @@
       </c>
       <c r="H12" s="100" t="inlineStr">
         <is>
-          <t>미조사</t>
+          <t>예약완료</t>
         </is>
       </c>
       <c r="I12" s="119" t="n">
@@ -8356,11 +8361,29 @@
       <c r="M12" s="120" t="n">
         <v>0</v>
       </c>
-      <c r="N12" s="120" t="n"/>
-      <c r="O12" s="100" t="n"/>
-      <c r="P12" s="100" t="n"/>
-      <c r="Q12" s="100" t="n"/>
-      <c r="R12" s="100" t="n"/>
+      <c r="N12" s="120" t="n">
+        <v>176.01</v>
+      </c>
+      <c r="O12" s="100" t="inlineStr">
+        <is>
+          <t>L671E2E0288</t>
+        </is>
+      </c>
+      <c r="P12" s="100" t="inlineStr">
+        <is>
+          <t>Hertz</t>
+        </is>
+      </c>
+      <c r="Q12" s="100" t="inlineStr">
+        <is>
+          <t>Barcelona Sants (C/ Viriat 45) → El Prat Airport T1·2</t>
+        </is>
+      </c>
+      <c r="R12" s="100" t="inlineStr">
+        <is>
+          <t>https://www.hertz.com</t>
+        </is>
+      </c>
       <c r="S12" s="100" t="inlineStr">
         <is>
           <t>04/05</t>
@@ -8371,8 +8394,14 @@
           <t>짐 노출·국경·반납지</t>
         </is>
       </c>
-      <c r="U12" s="119" t="n"/>
-      <c r="V12" s="63" t="n"/>
+      <c r="U12" s="119" t="n">
+        <v>46243</v>
+      </c>
+      <c r="V12" s="63" t="inlineStr">
+        <is>
+          <t>Ford Puma급(E0 CDAR) · 후지불 €176.01 · VISA ASIA CARDS 10% · 무제한 주행</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
@@ -8392,13 +8421,17 @@
       </c>
       <c r="D13" s="100" t="inlineStr">
         <is>
-          <t>Girona권→Nice 이동</t>
+          <t>BCN→NCE 항공 VY1521</t>
         </is>
       </c>
       <c r="E13" s="119" t="n">
         <v>46269</v>
       </c>
-      <c r="F13" s="100" t="n"/>
+      <c r="F13" s="100" t="inlineStr">
+        <is>
+          <t>15:30–16:55</t>
+        </is>
+      </c>
       <c r="G13" s="100" t="inlineStr">
         <is>
           <t>P0</t>
@@ -8406,7 +8439,7 @@
       </c>
       <c r="H13" s="100" t="inlineStr">
         <is>
-          <t>미조사</t>
+          <t>예약완료</t>
         </is>
       </c>
       <c r="I13" s="119" t="n">
@@ -8423,10 +8456,26 @@
         <v>0</v>
       </c>
       <c r="N13" s="120" t="n"/>
-      <c r="O13" s="100" t="n"/>
-      <c r="P13" s="100" t="n"/>
-      <c r="Q13" s="100" t="n"/>
-      <c r="R13" s="100" t="n"/>
+      <c r="O13" s="100" t="inlineStr">
+        <is>
+          <t>NMGI4Q</t>
+        </is>
+      </c>
+      <c r="P13" s="100" t="inlineStr">
+        <is>
+          <t>Vueling Airlines</t>
+        </is>
+      </c>
+      <c r="Q13" s="100" t="inlineStr">
+        <is>
+          <t>Josep Tarradellas Barcelona-El Prat T1 → Nice Côte d'Azur T1</t>
+        </is>
+      </c>
+      <c r="R13" s="100" t="inlineStr">
+        <is>
+          <t>https://www.vueling.com/en</t>
+        </is>
+      </c>
       <c r="S13" s="100" t="inlineStr">
         <is>
           <t>05/06</t>
@@ -8437,8 +8486,14 @@
           <t>공항 이동·수하물·차량 반납</t>
         </is>
       </c>
-      <c r="U13" s="119" t="n"/>
-      <c r="V13" s="63" t="n"/>
+      <c r="U13" s="119" t="n">
+        <v>46243</v>
+      </c>
+      <c r="V13" s="63" t="inlineStr">
+        <is>
+          <t>Economy · E-ticket 번호는 발권메일 확인 후 기입</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
@@ -8458,7 +8513,7 @@
       </c>
       <c r="D14" s="100" t="inlineStr">
         <is>
-          <t>NCE 인수→Avignon TGV 반납</t>
+          <t>니스 렌터카 — Nice역 인수→Avignon TGV역 반납</t>
         </is>
       </c>
       <c r="E14" s="119" t="n">
@@ -8466,7 +8521,7 @@
       </c>
       <c r="F14" s="100" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>9/9 09:00 인수 · 9/20 09:00 반납</t>
         </is>
       </c>
       <c r="G14" s="100" t="inlineStr">
@@ -8476,7 +8531,7 @@
       </c>
       <c r="H14" s="100" t="inlineStr">
         <is>
-          <t>재확인</t>
+          <t>예약완료</t>
         </is>
       </c>
       <c r="I14" s="119" t="n">
@@ -8492,11 +8547,29 @@
       <c r="M14" s="120" t="n">
         <v>0</v>
       </c>
-      <c r="N14" s="120" t="n"/>
-      <c r="O14" s="100" t="n"/>
-      <c r="P14" s="100" t="n"/>
-      <c r="Q14" s="100" t="n"/>
-      <c r="R14" s="100" t="n"/>
+      <c r="N14" s="120" t="n">
+        <v>608.09</v>
+      </c>
+      <c r="O14" s="100" t="inlineStr">
+        <is>
+          <t>L672E080313</t>
+        </is>
+      </c>
+      <c r="P14" s="100" t="inlineStr">
+        <is>
+          <t>Hertz</t>
+        </is>
+      </c>
+      <c r="Q14" s="100" t="inlineStr">
+        <is>
+          <t>Nice Railway Station (Avenue Thiers) → Avignon TGV (Place de l'Europe)</t>
+        </is>
+      </c>
+      <c r="R14" s="100" t="inlineStr">
+        <is>
+          <t>https://www.hertz.com</t>
+        </is>
+      </c>
       <c r="S14" s="100" t="inlineStr">
         <is>
           <t>itinerary.json / v2.0 지역 챕터</t>
@@ -8508,11 +8581,11 @@
         </is>
       </c>
       <c r="U14" s="119" t="n">
-        <v>46238</v>
+        <v>46243</v>
       </c>
       <c r="V14" s="63" t="inlineStr">
         <is>
-          <t>자동변속·편도수수료·보험·짐</t>
+          <t>Renault Captur급(F0 CDAR) · 후지불 €608.09 (drop-off €180 포함) · 무제한 주행 · 기존 NCE T2 계획에서 인수지 변경</t>
         </is>
       </c>
     </row>
@@ -8534,13 +8607,17 @@
       </c>
       <c r="D15" s="100" t="inlineStr">
         <is>
-          <t>Avignon TGV→Lyon</t>
+          <t>Avignon TGV→Lyon Part Dieu — INOUI 12176 1등석</t>
         </is>
       </c>
       <c r="E15" s="119" t="n">
         <v>46285</v>
       </c>
-      <c r="F15" s="100" t="n"/>
+      <c r="F15" s="100" t="inlineStr">
+        <is>
+          <t>10:22→11:28</t>
+        </is>
+      </c>
       <c r="G15" s="100" t="inlineStr">
         <is>
           <t>P0</t>
@@ -8548,7 +8625,7 @@
       </c>
       <c r="H15" s="100" t="inlineStr">
         <is>
-          <t>재확인</t>
+          <t>예약완료</t>
         </is>
       </c>
       <c r="I15" s="119" t="n">
@@ -8565,10 +8642,26 @@
         <v>0</v>
       </c>
       <c r="N15" s="120" t="n"/>
-      <c r="O15" s="100" t="n"/>
-      <c r="P15" s="100" t="n"/>
-      <c r="Q15" s="100" t="n"/>
-      <c r="R15" s="100" t="n"/>
+      <c r="O15" s="100" t="inlineStr">
+        <is>
+          <t>PNR 미표기 — 발권메일 확인</t>
+        </is>
+      </c>
+      <c r="P15" s="100" t="inlineStr">
+        <is>
+          <t>SNCF (TGV INOUI)</t>
+        </is>
+      </c>
+      <c r="Q15" s="100" t="inlineStr">
+        <is>
+          <t>3호차 308번 · Duo Côte à Côte</t>
+        </is>
+      </c>
+      <c r="R15" s="100" t="inlineStr">
+        <is>
+          <t>https://www.sncf-connect.com</t>
+        </is>
+      </c>
       <c r="S15" s="100" t="inlineStr">
         <is>
           <t>itinerary.json / v2.0 지역 챕터</t>
@@ -8580,11 +8673,11 @@
         </is>
       </c>
       <c r="U15" s="119" t="n">
-        <v>46238</v>
+        <v>46243</v>
       </c>
       <c r="V15" s="63" t="inlineStr">
         <is>
-          <t>반납·주유·플랫폼 버퍼</t>
+          <t>승차권 이미지 기준 · PNR 은 발권메일에서 확인 후 기입</t>
         </is>
       </c>
     </row>
@@ -9788,6 +9881,7 @@
       <c r="Q1" s="98" t="n"/>
       <c r="R1" s="98" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -9956,11 +10050,20 @@
           <t>렌터카</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>07:00 인수</t>
+        </is>
+      </c>
       <c r="H5" s="100" t="n"/>
-      <c r="I5" s="100" t="n"/>
+      <c r="I5" s="100" t="inlineStr">
+        <is>
+          <t>Hertz L671E2E0288</t>
+        </is>
+      </c>
       <c r="J5" s="100" t="inlineStr">
         <is>
-          <t>미조사</t>
+          <t>예약완료</t>
         </is>
       </c>
       <c r="K5" s="100" t="n"/>
@@ -9971,7 +10074,7 @@
       </c>
       <c r="M5" s="100" t="inlineStr">
         <is>
-          <t>Barcelona 인수 / 반납 미정</t>
+          <t>Sants 07:00 인수 · Bàscara까지</t>
         </is>
       </c>
       <c r="N5" s="100" t="inlineStr">
@@ -9994,7 +10097,9 @@
           <t>04/05</t>
         </is>
       </c>
-      <c r="R5" s="119" t="n"/>
+      <c r="R5" s="119" t="n">
+        <v>46243</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -10017,19 +10122,37 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>미정</t>
+          <t>렌터카 반납 후 항공</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>16:55</t>
         </is>
       </c>
       <c r="H6" s="100" t="n"/>
-      <c r="I6" s="100" t="n"/>
+      <c r="I6" s="100" t="inlineStr">
+        <is>
+          <t>Vueling VY1521</t>
+        </is>
+      </c>
       <c r="J6" s="100" t="inlineStr">
         <is>
-          <t>미조사</t>
+          <t>예약완료</t>
         </is>
       </c>
       <c r="K6" s="100" t="n"/>
       <c r="L6" s="100" t="n"/>
-      <c r="M6" s="100" t="n"/>
+      <c r="M6" s="100" t="inlineStr">
+        <is>
+          <t>BCN T1 출발 · NCE T1 도착</t>
+        </is>
+      </c>
       <c r="N6" s="100" t="inlineStr">
         <is>
           <t>90분</t>
@@ -10050,7 +10173,9 @@
           <t>05/06</t>
         </is>
       </c>
-      <c r="R6" s="119" t="n"/>
+      <c r="R6" s="119" t="n">
+        <v>46243</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -10078,14 +10203,18 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>09:00 인수</t>
         </is>
       </c>
       <c r="H7" s="100" t="n"/>
-      <c r="I7" s="100" t="n"/>
+      <c r="I7" s="100" t="inlineStr">
+        <is>
+          <t>Hertz L672E080313</t>
+        </is>
+      </c>
       <c r="J7" s="100" t="inlineStr">
         <is>
-          <t>미조사</t>
+          <t>예약완료</t>
         </is>
       </c>
       <c r="K7" s="100" t="n"/>
@@ -10096,7 +10225,7 @@
       </c>
       <c r="M7" s="100" t="inlineStr">
         <is>
-          <t>NCE T2 인수</t>
+          <t>Nice Railway Station 인수 (NCE T2 아님)</t>
         </is>
       </c>
       <c r="N7" s="100" t="inlineStr">
@@ -10120,7 +10249,7 @@
         </is>
       </c>
       <c r="R7" s="119" t="n">
-        <v>46235</v>
+        <v>46243</v>
       </c>
     </row>
     <row r="8">
@@ -10258,21 +10387,35 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>렌터카+TGV</t>
+          <t>렌터카 반납+TGV</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>10:22</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>11:28</t>
         </is>
       </c>
       <c r="H10" s="100" t="str"/>
-      <c r="I10" s="100" t="str"/>
+      <c r="I10" s="100" t="inlineStr">
+        <is>
+          <t>TGV INOUI 12176</t>
+        </is>
+      </c>
       <c r="J10" s="100" t="inlineStr">
         <is>
-          <t>재확인</t>
+          <t>예약완료</t>
         </is>
       </c>
       <c r="K10" s="100" t="str"/>
       <c r="L10" s="100" t="str"/>
       <c r="M10" s="100" t="inlineStr">
         <is>
-          <t>Avignon TGV 반납</t>
+          <t>Avignon TGV역 09:00 반납 후 승차</t>
         </is>
       </c>
       <c r="N10" s="100" t="inlineStr">
@@ -10296,7 +10439,7 @@
         </is>
       </c>
       <c r="R10" s="119" t="n">
-        <v>46238</v>
+        <v>46243</v>
       </c>
     </row>
     <row r="11">
@@ -10685,10 +10828,7 @@
       <c r="I4" s="120" t="n">
         <v>701054</v>
       </c>
-      <c r="J4" s="120">
-        <f>IF(OR(I4="",D4=0),"",I4/D4)</f>
-        <v/>
-      </c>
+      <c r="J4" s="120" t="n"/>
       <c r="K4" s="119" t="str"/>
       <c r="L4" s="100" t="inlineStr">
         <is>
@@ -10982,10 +11122,7 @@
       </c>
       <c r="H8" s="120" t="n"/>
       <c r="I8" s="120" t="n"/>
-      <c r="J8" s="120">
-        <f>IF(OR(I8="",D8=0),"",I8/D8)</f>
-        <v/>
-      </c>
+      <c r="J8" s="120" t="n"/>
       <c r="K8" s="119" t="str"/>
       <c r="L8" s="100" t="str"/>
       <c r="M8" s="100" t="str"/>
@@ -11049,10 +11186,7 @@
       </c>
       <c r="H9" s="120" t="n"/>
       <c r="I9" s="120" t="n"/>
-      <c r="J9" s="120">
-        <f>IF(OR(I9="",D9=0),"",I9/D9)</f>
-        <v/>
-      </c>
+      <c r="J9" s="120" t="n"/>
       <c r="K9" s="119" t="str"/>
       <c r="L9" s="100" t="str"/>
       <c r="M9" s="100" t="str"/>
@@ -11116,10 +11250,7 @@
       </c>
       <c r="H10" s="120" t="n"/>
       <c r="I10" s="120" t="n"/>
-      <c r="J10" s="120">
-        <f>IF(OR(I10="",D10=0),"",I10/D10)</f>
-        <v/>
-      </c>
+      <c r="J10" s="120" t="n"/>
       <c r="K10" s="119" t="str"/>
       <c r="L10" s="100" t="str"/>
       <c r="M10" s="100" t="str"/>
@@ -11185,10 +11316,7 @@
         <v>5000000</v>
       </c>
       <c r="I11" s="121" t="n"/>
-      <c r="J11" s="121">
-        <f>IF(OR(I11="",D11=0),"",I11/D11)</f>
-        <v/>
-      </c>
+      <c r="J11" s="121" t="n"/>
       <c r="K11" s="122" t="str"/>
       <c r="L11" s="49" t="str"/>
       <c r="M11" s="49" t="str"/>
@@ -13008,10 +13136,7 @@
           <t>전체 예약항목</t>
         </is>
       </c>
-      <c r="E4" s="17">
-        <f>COUNTA(Reservations!A4:A200)</f>
-        <v/>
-      </c>
+      <c r="E4" s="17" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -13027,10 +13152,7 @@
           <t>P0 항목</t>
         </is>
       </c>
-      <c r="E5" s="17">
-        <f>COUNTIF(Reservations!G4:G200,"P0")</f>
-        <v/>
-      </c>
+      <c r="E5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -13046,10 +13168,7 @@
           <t>예약완료</t>
         </is>
       </c>
-      <c r="E6" s="17">
-        <f>COUNTIF(Reservations!H4:H200,"예약완료")</f>
-        <v/>
-      </c>
+      <c r="E6" s="17" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -13065,10 +13184,7 @@
           <t>예약대기</t>
         </is>
       </c>
-      <c r="E7" s="17">
-        <f>COUNTIF(Reservations!H4:H200,"예약대기")</f>
-        <v/>
-      </c>
+      <c r="E7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -13084,10 +13200,7 @@
           <t>재확인</t>
         </is>
       </c>
-      <c r="E8" s="17">
-        <f>COUNTIF(Reservations!H4:H200,"재확인")</f>
-        <v/>
-      </c>
+      <c r="E8" s="17" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
@@ -13103,10 +13216,7 @@
           <t>미조사</t>
         </is>
       </c>
-      <c r="E9" s="17">
-        <f>COUNTIF(Reservations!H4:H200,"미조사")</f>
-        <v/>
-      </c>
+      <c r="E9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="18" t="inlineStr">
@@ -13122,10 +13232,7 @@
           <t>숙소 예약완료</t>
         </is>
       </c>
-      <c r="E10" s="20">
-        <f>COUNTIFS(Reservations!B4:B200,"숙소",Reservations!H4:H200,"예약완료")</f>
-        <v/>
-      </c>
+      <c r="E10" s="20" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">

</xml_diff>

<commit_message>
feat: withdraw Paris opera plans (D-14), keep evening slots as pending
Il Barbiere (10/1) and Hamlet (10/9) are no longer attended: R021/R022
cancelled in the tracker, the Paris chapter's schedules, booking gates,
budget and control tables rebuilt without them (§27 becomes a
withdrawal record), master itinerary / execution audit / gate calendar
/ daily routes / itinerary sheet realigned, and every affected evening
reads "공연 대체안 검토 중" with a pending badge — no invented
replacements. Arc (10/4), Vendanges (10/7) and Este Mundo (10/8,
optional) stay. Also records D-13: PWA full-store size stays as-is.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -6221,7 +6221,7 @@
       </c>
       <c r="J32" s="100" t="inlineStr">
         <is>
-          <t>무예약·Il Barbiere 회차 제외</t>
+          <t>무예약</t>
         </is>
       </c>
       <c r="K32" s="100" t="inlineStr">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>고정 공연</t>
+          <t>동네 산책</t>
         </is>
       </c>
       <c r="F37" s="100" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="J37" s="100" t="inlineStr">
         <is>
-          <t>17:30 이른 저녁·18:30–18:45 입장·Il Barbiere 19:30–약 22:45</t>
+          <t>저녁 — 공연 대체안 검토 중</t>
         </is>
       </c>
       <c r="K37" s="100" t="inlineStr">
@@ -6865,7 +6865,7 @@
       </c>
       <c r="Q39" s="100" t="inlineStr">
         <is>
-          <t>Arc 토요일+Hamlet 조합 금지</t>
+          <t>다음 날 Arc 대비 저강도 유지</t>
         </is>
       </c>
       <c r="R39" s="100" t="inlineStr">
@@ -7075,7 +7075,7 @@
       </c>
       <c r="F42" s="100" t="inlineStr">
         <is>
-          <t>동부 파리 또는 Hamlet 백업</t>
+          <t>동부 파리 생활일</t>
         </is>
       </c>
       <c r="G42" s="100" t="inlineStr">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="J42" s="100" t="inlineStr">
         <is>
-          <t>Hamlet 19:30은 10/9 매진 시만</t>
+          <t>무예약</t>
         </is>
       </c>
       <c r="K42" s="100" t="inlineStr">
@@ -7337,12 +7337,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>고정 공연</t>
+          <t>짐 포장</t>
         </is>
       </c>
       <c r="F45" s="100" t="inlineStr">
         <is>
-          <t>Hamlet·최종 포장</t>
+          <t>최종 포장·마지막 저녁</t>
         </is>
       </c>
       <c r="G45" s="100" t="inlineStr">
@@ -7362,7 +7362,7 @@
       </c>
       <c r="J45" s="100" t="inlineStr">
         <is>
-          <t>Hamlet 19:30·Jazz/교회공연 제외·직접 귀가</t>
+          <t>저녁 — 공연 대체안 검토 중</t>
         </is>
       </c>
       <c r="K45" s="100" t="inlineStr">
@@ -7582,7 +7582,6 @@
       <c r="U1" s="98" t="n"/>
       <c r="V1" s="98" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -9271,7 +9270,7 @@
       </c>
       <c r="H24" s="100" t="inlineStr">
         <is>
-          <t>예약대기</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="I24" s="119" t="n">
@@ -9307,11 +9306,11 @@
         </is>
       </c>
       <c r="U24" s="119" t="n">
-        <v>46239</v>
+        <v>46244</v>
       </c>
       <c r="V24" s="63" t="inlineStr">
         <is>
-          <t>3h15·이탈리아어·FR/EN 자막·현재 €77–205</t>
+          <t>2026-08-10 사용자 결정 — 파리 오페라 관람 제외 · 저녁 대체안 검토 중</t>
         </is>
       </c>
     </row>
@@ -9351,7 +9350,7 @@
       </c>
       <c r="H25" s="100" t="inlineStr">
         <is>
-          <t>예약대기</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="I25" s="119" t="n">
@@ -9387,11 +9386,11 @@
         </is>
       </c>
       <c r="U25" s="119" t="n">
-        <v>46239</v>
+        <v>46244</v>
       </c>
       <c r="V25" s="63" t="inlineStr">
         <is>
-          <t>3h40·프랑스어·FR/EN 자막·현재 €28–155</t>
+          <t>2026-08-10 사용자 결정 — 파리 오페라 관람 제외 · 저녁 대체안 검토 중</t>
         </is>
       </c>
     </row>
@@ -9881,7 +9880,6 @@
       <c r="Q1" s="98" t="n"/>
       <c r="R1" s="98" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: align tracker, gates and daily routes with the three-performance withdrawal
Adopt main's chapter/itinerary/audit (PR #102) in the merge, cancel
R024 alongside R021/R022, and scrub Este Mundo from the 10/7-10/8 gate
row and the Day 41 route while keeping the daytime Chaillot stops.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -7582,6 +7582,7 @@
       <c r="U1" s="98" t="n"/>
       <c r="V1" s="98" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -9506,7 +9507,7 @@
       </c>
       <c r="H27" s="49" t="inlineStr">
         <is>
-          <t>예약대기</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="I27" s="119" t="n">
@@ -9542,11 +9543,11 @@
         </is>
       </c>
       <c r="U27" s="119" t="n">
-        <v>46239</v>
+        <v>46244</v>
       </c>
       <c r="V27" s="66" t="inlineStr">
         <is>
-          <t>1h·현재 €8–25</t>
+          <t>2026-08-10 사용자 결정 — 파리 공연 3건 철회 · 자유 저녁</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(tracker): log both international flights, Nice Airbnb reference
The tracker had no row for the flights that open and close the trip — the
one place someone checks in the field for a booking reference. R029 holds
OZ511 (8/29 ICN 11:50 → BCN 19:10, ref FRRL7R, 예약완료) and R030 holds
OZ502 (10/9 CDG 19:10 → ICN 10/10 14:10), which stays 재확인 because the
reference is not issued yet; the Phase 8 guard moves to R001~R030 / 15 P0
rows to match.

Nice carries its Airbnb reference HMJ3HX8QAY across tracker, chapter,
decision register and cards 07–12. It stays 재확인 rather than 예약완료 on
purpose: the guard wants a real total, and we do not have one yet.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -7531,7 +7531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V31"/>
+  <dimension ref="A1:V33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="92" min="1" max="1"/>
@@ -7933,8 +7933,16 @@
         <v>0</v>
       </c>
       <c r="N6" s="120" t="n"/>
-      <c r="O6" s="100" t="n"/>
-      <c r="P6" s="100" t="n"/>
+      <c r="O6" s="100" t="inlineStr">
+        <is>
+          <t>HMJ3HX8QAY</t>
+        </is>
+      </c>
+      <c r="P6" s="100" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
       <c r="Q6" s="100" t="inlineStr">
         <is>
           <t>12 Rue Verdi, Palais ALZIRA, 06000 Nice, France</t>
@@ -7948,7 +7956,7 @@
       </c>
       <c r="T6" s="100" t="inlineStr">
         <is>
-          <t>총액·예약번호·플랫폼 미기입 · 9/9 09:00 렌터카 인수와 11:00 체크아웃 순서</t>
+          <t>총액 미기입 · 9/9 09:00 렌터카 인수와 11:00 체크아웃 순서</t>
         </is>
       </c>
       <c r="U6" s="119" t="n">
@@ -7956,7 +7964,7 @@
       </c>
       <c r="V6" s="63" t="inlineStr">
         <is>
-          <t>2026-08-13 사용자 확정 — 9/4 15:00 체크인 · 9/9 11:00 체크아웃. 예약번호·총액·사업자 입력 필요</t>
+          <t>2026-08-13 사용자 확정 — Airbnb HMJ3HX8QAY · 9/4 15:00 체크인 · 9/9 11:00 체크아웃. 실제총액 입력 시 예약완료로 잠근다</t>
         </is>
       </c>
     </row>
@@ -9806,6 +9814,173 @@
       <c r="T31" t="inlineStr">
         <is>
           <t>스페인·프랑스 전 구간</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>R029</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>항공</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>인천→바르셀로나 국제선 OZ511</t>
+        </is>
+      </c>
+      <c r="E32" s="128" t="n">
+        <v>46263</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>ICN T2 11:50 → BCN T1 19:10</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>예약완료</t>
+        </is>
+      </c>
+      <c r="I32" s="128" t="n">
+        <v>46244</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>FRRL7R</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>아시아나항공</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>인천공항 T2 → 바르셀로나 엘프라트 T1</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>https://flyasiana.com</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>04_Barcelona_Sitges_v2.0.md</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>야간 도착 — Day 1은 도착·체크인만, 수하물 규정 확인</t>
+        </is>
+      </c>
+      <c r="U32" s="128" t="n">
+        <v>46247</v>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>2026-08-10 발권 확정 · 비행 약 14시간 20분</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>R030</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>항공</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>파리→인천 국제선 OZ502</t>
+        </is>
+      </c>
+      <c r="E33" s="128" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>CDG 19:10 → ICN 10/10 14:10</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>재확인</t>
+        </is>
+      </c>
+      <c r="I33" s="128" t="n">
+        <v>46247</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>KRW</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>아시아나항공</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>파리 샤를드골 → 인천공항</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>https://flyasiana.com</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>11_Paris_Long_Stay_v2.0.md</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>예약번호·터미널 미확정 · 파업 시 최악 시나리오 — 전날 항공편 상태 확인</t>
+        </is>
+      </c>
+      <c r="U33" s="128" t="n">
+        <v>46247</v>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>2026-08-13 편명·시각 확정 · 예약번호 미확정 (확정 시 예약완료로 전환)</t>
         </is>
       </c>
     </row>
@@ -10986,7 +11161,7 @@
       </c>
       <c r="F6" s="100" t="inlineStr">
         <is>
-          <t>Palais ALZIRA · 12 Rue Verdi (Nice 06000)</t>
+          <t>Airbnb · Palais ALZIRA · 12 Rue Verdi (Nice 06000)</t>
         </is>
       </c>
       <c r="G6" s="100" t="inlineStr">
@@ -10998,7 +11173,11 @@
       <c r="I6" s="120" t="n"/>
       <c r="J6" s="120" t="n"/>
       <c r="K6" s="119" t="n"/>
-      <c r="L6" s="100" t="n"/>
+      <c r="L6" s="100" t="inlineStr">
+        <is>
+          <t>HMJ3HX8QAY</t>
+        </is>
+      </c>
       <c r="M6" s="100" t="inlineStr">
         <is>
           <t>12 Rue Verdi, Palais ALZIRA, 06000 Nice, France</t>
@@ -11032,7 +11211,7 @@
       <c r="S6" s="100" t="n"/>
       <c r="T6" s="63" t="inlineStr">
         <is>
-          <t>2026-08-13 사용자 확정 — 예약 완료(체크인 9/4 15:00 · 체크아웃 9/9 11:00). 트래커 잠금에는 총액·예약번호·소스 URL 입력 필요</t>
+          <t>2026-08-13 사용자 확정 — Airbnb HMJ3HX8QAY · 체크인 9/4 15:00 · 체크아웃 9/9 11:00. 실제총액 입력 시 예약완료로 잠근다</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(guard): R1b — 확정 사실 토큰 가드 감시 범위 확장(Tracker·Manifest 연동) 및 13 tests 완료
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -7590,6 +7590,7 @@
       <c r="U1" s="98" t="n"/>
       <c r="V1" s="98" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -7761,7 +7762,7 @@
       </c>
       <c r="O4" s="100" t="inlineStr">
         <is>
-          <t>365585SG255002 · Trip.com 1400827967207904</t>
+          <t>36558SG255002 · Trip.com 1400827967207904</t>
         </is>
       </c>
       <c r="P4" s="100" t="inlineStr">
@@ -10901,6 +10902,7 @@
       <c r="S1" s="98" t="n"/>
       <c r="T1" s="98" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -11043,7 +11045,7 @@
       <c r="K4" s="119" t="str"/>
       <c r="L4" s="100" t="inlineStr">
         <is>
-          <t>365585SG255002 · Trip.com 1400827967207904</t>
+          <t>36558SG255002 · Trip.com 1400827967207904</t>
         </is>
       </c>
       <c r="M4" s="100" t="inlineStr">

</xml_diff>

<commit_message>
fix(ops): update Master Tracker Accommodation and Itinerary for Gordes 2N and Avignon 5N
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -5351,7 +5351,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Gordes</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="F19" s="100" t="inlineStr">
         <is>
-          <t>Lourmarin·장보기·농가 체크인</t>
+          <t>Aix 체크아웃 → Lourmarin → Gordes 1박차</t>
         </is>
       </c>
       <c r="G19" s="100" t="n"/>
@@ -5416,7 +5416,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Gordes</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="F20" s="100" t="inlineStr">
         <is>
-          <t>Roussillon + Goult 또는 Bonnieux</t>
+          <t>Roussillon · 선택마을 · Sénanque → Gordes 2박차</t>
         </is>
       </c>
       <c r="G20" s="100" t="n"/>
@@ -5481,20 +5481,20 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Avignon</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>체류</t>
+          <t>이동</t>
         </is>
       </c>
       <c r="F21" s="100" t="inlineStr">
         <is>
-          <t>Gordes·Village des Bories + 선택마을</t>
+          <t>Gordes 체크아웃 → 물의 마을 → Avignon 체크인</t>
         </is>
       </c>
       <c r="G21" s="100" t="n"/>
@@ -5550,16 +5550,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>이동</t>
+          <t>체류</t>
         </is>
       </c>
       <c r="F22" s="100" t="inlineStr">
         <is>
-          <t>농가 체크아웃·Avignon 이동·정착</t>
+          <t>수요시장 · Van Gogh · Alpilles 석회암 풍경</t>
         </is>
       </c>
       <c r="G22" s="100" t="n"/>
@@ -5615,7 +5615,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -5624,7 +5624,7 @@
       </c>
       <c r="F23" s="100" t="inlineStr">
         <is>
-          <t>Avignon 핵심 관광</t>
+          <t>Uzès · Pont du Gard · Nîmes &amp; 렌터카 최종 반납</t>
         </is>
       </c>
       <c r="G23" s="100" t="n"/>
@@ -5680,7 +5680,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -5689,7 +5689,7 @@
       </c>
       <c r="F24" s="100" t="inlineStr">
         <is>
-          <t>Uzès 구시가지·Pont du Gard</t>
+          <t>Arles 철도 당일치기</t>
         </is>
       </c>
       <c r="G24" s="100" t="n"/>
@@ -5745,7 +5745,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -5754,7 +5754,7 @@
       </c>
       <c r="F25" s="100" t="inlineStr">
         <is>
-          <t>Arles 당일치기</t>
+          <t>교황도시 핵심 (Avignon 시내 도보일)</t>
         </is>
       </c>
       <c r="G25" s="100" t="n"/>
@@ -11363,17 +11363,17 @@
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Gordes</t>
         </is>
       </c>
       <c r="B8" s="116" t="n">
         <v>46278</v>
       </c>
       <c r="C8" s="116" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -11382,7 +11382,7 @@
       </c>
       <c r="F8" s="100" t="inlineStr">
         <is>
-          <t>Gordes–Goult–Roussillon–Bonnieux</t>
+          <t>Gordes 및 루베롱 북부 권역 (후보 미정)</t>
         </is>
       </c>
       <c r="G8" s="100" t="inlineStr">
@@ -11420,7 +11420,7 @@
       <c r="S8" s="100" t="str"/>
       <c r="T8" s="63" t="inlineStr">
         <is>
-          <t>기존 4박→3박 예약 변경 필요</t>
+          <t>Gordes 2박 숙소 후보 확정 필요</t>
         </is>
       </c>
     </row>
@@ -11431,13 +11431,13 @@
         </is>
       </c>
       <c r="B9" s="116" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="C9" s="116" t="n">
         <v>46285</v>
       </c>
       <c r="D9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -11446,7 +11446,7 @@
       </c>
       <c r="F9" s="100" t="inlineStr">
         <is>
-          <t>성벽 안 외곽/남·동쪽</t>
+          <t>성벽 안(intra-muros) 도보 생활권 · La Terrasse du Clocher 등</t>
         </is>
       </c>
       <c r="G9" s="100" t="inlineStr">
@@ -11484,7 +11484,7 @@
       <c r="S9" s="100" t="str"/>
       <c r="T9" s="63" t="inlineStr">
         <is>
-          <t>기존 9/17 체크인 예약 변경 필요</t>
+          <t>Avignon 5박 숙소·주차·체크인 창 확정 필요</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(itinerary): align Provence content with canonical schedule
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -2214,6 +2214,7 @@
       <c r="G1" s="98" t="n"/>
       <c r="H1" s="98" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="88" t="inlineStr">
         <is>
@@ -2726,17 +2727,17 @@
       </c>
       <c r="B15" s="100" t="inlineStr">
         <is>
-          <t>Gordes</t>
+          <t>L'Isle-sur-la-Sorgue·Avignon</t>
         </is>
       </c>
       <c r="C15" s="100" t="inlineStr">
         <is>
-          <t>시장·돌마을·장바구니</t>
+          <t>수로·물레방아·Avignon 체크인</t>
         </is>
       </c>
       <c r="D15" s="100" t="inlineStr">
         <is>
-          <t>오전</t>
+          <t>오전·오후</t>
         </is>
       </c>
       <c r="E15" s="100" t="inlineStr">
@@ -2746,7 +2747,7 @@
       </c>
       <c r="F15" s="100" t="inlineStr">
         <is>
-          <t>마을생활</t>
+          <t>물의 Provence·거점 전환</t>
         </is>
       </c>
       <c r="G15" s="100" t="inlineStr">
@@ -2768,17 +2769,17 @@
       </c>
       <c r="B16" s="100" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Saint-Rémy·Les Baux</t>
         </is>
       </c>
       <c r="C16" s="100" t="inlineStr">
         <is>
-          <t>농가 식탁·스케치·세탁</t>
+          <t>수요시장·석회암 마을</t>
         </is>
       </c>
       <c r="D16" s="100" t="inlineStr">
         <is>
-          <t>오후</t>
+          <t>오전·오후</t>
         </is>
       </c>
       <c r="E16" s="100" t="inlineStr">
@@ -2788,7 +2789,7 @@
       </c>
       <c r="F16" s="100" t="inlineStr">
         <is>
-          <t>농가체험 핵심</t>
+          <t>시장·Alpilles</t>
         </is>
       </c>
       <c r="G16" s="100" t="inlineStr">
@@ -2810,17 +2811,17 @@
       </c>
       <c r="B17" s="100" t="inlineStr">
         <is>
-          <t>Avignon</t>
+          <t>Arles</t>
         </is>
       </c>
       <c r="C17" s="100" t="inlineStr">
         <is>
-          <t>Palais–Pont 파노라마</t>
+          <t>Arènes·Théâtre·Saint-Trophime</t>
         </is>
       </c>
       <c r="D17" s="100" t="inlineStr">
         <is>
-          <t>오후</t>
+          <t>전일</t>
         </is>
       </c>
       <c r="E17" s="100" t="inlineStr">
@@ -2830,7 +2831,7 @@
       </c>
       <c r="F17" s="100" t="inlineStr">
         <is>
-          <t>도시상징</t>
+          <t>JEP·로마유산</t>
         </is>
       </c>
       <c r="G17" s="100" t="inlineStr">
@@ -2852,17 +2853,17 @@
       </c>
       <c r="B18" s="100" t="inlineStr">
         <is>
-          <t>Uzès</t>
+          <t>Avignon</t>
         </is>
       </c>
       <c r="C18" s="100" t="inlineStr">
         <is>
-          <t>시장 장보기</t>
+          <t>Les Halles·Palais·Rocher·Pont</t>
         </is>
       </c>
       <c r="D18" s="100" t="inlineStr">
         <is>
-          <t>오전</t>
+          <t>전일</t>
         </is>
       </c>
       <c r="E18" s="100" t="inlineStr">
@@ -2872,7 +2873,7 @@
       </c>
       <c r="F18" s="100" t="inlineStr">
         <is>
-          <t>프로방스 시장</t>
+          <t>교황도시 핵심</t>
         </is>
       </c>
       <c r="G18" s="100" t="inlineStr">
@@ -3289,7 +3290,7 @@
       </c>
       <c r="G4" s="100" t="inlineStr">
         <is>
-          <t>Nice 5·Aix 4·Luberon 3·Avignon 4·Lyon 4·Paris 15박 + 기내 1박(10/9→10/10)</t>
+          <t>Barcelona 3·Bàscara 3·Nice 5·Aix 4·Gordes 2·Avignon 5·Lyon 4·Paris 15박 + 기내 1박</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3312,7 @@
       </c>
       <c r="D5" s="100" t="inlineStr">
         <is>
-          <t>3/3/5/4/3/4/4/15박</t>
+          <t>3/3/5/4/2/5/4/15박</t>
         </is>
       </c>
       <c r="E5" s="100" t="inlineStr">
@@ -3326,7 +3327,7 @@
       </c>
       <c r="G5" s="100" t="inlineStr">
         <is>
-          <t>Luberon·Avignon·Lyon·Paris 기존 예약 변경 필요 · 마지막 밤은 기내</t>
+          <t>Gordes·Avignon 숙소 후보 확정 필요 · 마지막 밤은 기내</t>
         </is>
       </c>
     </row>
@@ -3488,12 +3489,12 @@
       </c>
       <c r="D10" s="100" t="inlineStr">
         <is>
-          <t>9/9 NCE 인수, 9/20 Avignon 반납</t>
+          <t>9/9 Nice-Ville 인수, 9/17 Avignon TGV 반납</t>
         </is>
       </c>
       <c r="E10" s="100" t="inlineStr">
         <is>
-          <t>업체·예약번호·9/20 반납 변경 확인</t>
+          <t>기존 9/20 계약을 9/17 18:30 이전 반납으로 변경</t>
         </is>
       </c>
       <c r="F10" s="100" t="inlineStr">
@@ -3717,7 +3718,7 @@
       </c>
       <c r="B17" s="100" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Gordes</t>
         </is>
       </c>
       <c r="C17" s="100" t="inlineStr">
@@ -3727,12 +3728,12 @@
       </c>
       <c r="D17" s="100" t="inlineStr">
         <is>
-          <t>3박 · 예약 변경 필요</t>
+          <t>2박 · 9/13~9/15</t>
         </is>
       </c>
       <c r="E17" s="100" t="inlineStr">
         <is>
-          <t>기존 4박 예약을 9/13~9/16으로 변경</t>
+          <t>숙소 후보·주차·체크인 확정</t>
         </is>
       </c>
       <c r="F17" s="100" t="inlineStr">
@@ -3760,12 +3761,12 @@
       </c>
       <c r="D18" s="100" t="inlineStr">
         <is>
-          <t>4박 · 9/16~9/20</t>
+          <t>5박 · 9/15~9/20</t>
         </is>
       </c>
       <c r="E18" s="100" t="inlineStr">
         <is>
-          <t>기존 체크인일 변경 확인</t>
+          <t>숙소 후보·주차·체크인 확정</t>
         </is>
       </c>
       <c r="F18" s="100" t="inlineStr">
@@ -3996,7 +3997,7 @@
     <row r="1" ht="30" customHeight="1" s="92">
       <c r="A1" s="115" t="inlineStr">
         <is>
-          <t>TP Europe Travel — Master Itinerary v1.2 (43일·42박 · Paris 16박)</t>
+          <t>TP Europe Travel — Master Itinerary v1.2 (43일·42박 · Paris 15박 + 기내 1박)</t>
         </is>
       </c>
       <c r="B1" s="98" t="n"/>
@@ -5373,13 +5374,13 @@
       <c r="J19" s="100" t="n"/>
       <c r="K19" s="100" t="inlineStr">
         <is>
-          <t>Aix→Lourmarin→농가</t>
+          <t>Aix→Lourmarin→Gordes</t>
         </is>
       </c>
       <c r="L19" s="100" t="n"/>
       <c r="M19" s="100" t="n"/>
       <c r="N19" s="100" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O19" s="100" t="inlineStr">
         <is>
@@ -5388,12 +5389,12 @@
       </c>
       <c r="P19" s="100" t="inlineStr">
         <is>
-          <t>농가 3박 변경</t>
+          <t>Gordes 2박·Lourmarin 점심</t>
         </is>
       </c>
       <c r="Q19" s="100" t="inlineStr">
         <is>
-          <t>경유지 축소</t>
+          <t>Lacoste→Bonnieux 순으로 삭제</t>
         </is>
       </c>
       <c r="R19" s="100" t="inlineStr">
@@ -5402,7 +5403,7 @@
         </is>
       </c>
       <c r="S19" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="20">
@@ -5438,7 +5439,7 @@
       <c r="J20" s="100" t="n"/>
       <c r="K20" s="100" t="inlineStr">
         <is>
-          <t>농가↔Roussillon·선택마을</t>
+          <t>Gordes↔Roussillon·Sénanque</t>
         </is>
       </c>
       <c r="L20" s="100" t="n"/>
@@ -5453,12 +5454,12 @@
       </c>
       <c r="P20" s="100" t="inlineStr">
         <is>
-          <t>주차·오커길</t>
+          <t>Sénanque 슬롯·오커길</t>
         </is>
       </c>
       <c r="Q20" s="100" t="inlineStr">
         <is>
-          <t>두 번째 마을 삭제</t>
+          <t>Goult→Ménerbes 순으로 삭제</t>
         </is>
       </c>
       <c r="R20" s="100" t="inlineStr">
@@ -5467,7 +5468,7 @@
         </is>
       </c>
       <c r="S20" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="21">
@@ -5503,7 +5504,7 @@
       <c r="J21" s="100" t="n"/>
       <c r="K21" s="100" t="inlineStr">
         <is>
-          <t>농가↔Gordes·Bories</t>
+          <t>Gordes→L'Isle→Avignon</t>
         </is>
       </c>
       <c r="L21" s="100" t="n"/>
@@ -5518,21 +5519,21 @@
       </c>
       <c r="P21" s="100" t="inlineStr">
         <is>
-          <t>시장·주차</t>
+          <t>Avignon 5박·주차</t>
         </is>
       </c>
       <c r="Q21" s="100" t="inlineStr">
         <is>
-          <t>Ménerbes/Oppède 삭제</t>
+          <t>Fontaine 삭제 후 Avignon 직행</t>
         </is>
       </c>
       <c r="R21" s="100" t="inlineStr">
         <is>
-          <t>08_Luberon_Farmhouse_v2.0.md</t>
+          <t>09_Avignon_Alpilles_Pont_du_Gard_v2.0.md</t>
         </is>
       </c>
       <c r="S21" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="22">
@@ -5568,13 +5569,13 @@
       <c r="J22" s="100" t="n"/>
       <c r="K22" s="100" t="inlineStr">
         <is>
-          <t>Luberon→Avignon</t>
+          <t>Avignon↔Saint-Rémy·Les Baux</t>
         </is>
       </c>
       <c r="L22" s="100" t="n"/>
       <c r="M22" s="100" t="n"/>
       <c r="N22" s="100" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O22" s="100" t="inlineStr">
         <is>
@@ -5583,12 +5584,12 @@
       </c>
       <c r="P22" s="100" t="inlineStr">
         <is>
-          <t>농가·Avignon 숙소 변경</t>
+          <t>시장·Château 운영</t>
         </is>
       </c>
       <c r="Q22" s="100" t="inlineStr">
         <is>
-          <t>추가마을·저녁관람 삭제</t>
+          <t>Orange 삭제</t>
         </is>
       </c>
       <c r="R22" s="100" t="inlineStr">
@@ -5597,7 +5598,7 @@
         </is>
       </c>
       <c r="S22" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="23">
@@ -5633,13 +5634,13 @@
       <c r="J23" s="100" t="n"/>
       <c r="K23" s="100" t="inlineStr">
         <is>
-          <t>성벽 안 도보</t>
+          <t>Avignon→Uzès→Pont du Gard→Nîmes→Avignon TGV</t>
         </is>
       </c>
       <c r="L23" s="100" t="n"/>
       <c r="M23" s="100" t="n"/>
       <c r="N23" s="100" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O23" s="100" t="inlineStr">
         <is>
@@ -5648,12 +5649,12 @@
       </c>
       <c r="P23" s="100" t="inlineStr">
         <is>
-          <t>Palais des Papes</t>
+          <t>18:30 이전 Hertz 조기 반납</t>
         </is>
       </c>
       <c r="Q23" s="100" t="inlineStr">
         <is>
-          <t>추가 미술관 삭제</t>
+          <t>Nîmes 체류부터 축소</t>
         </is>
       </c>
       <c r="R23" s="100" t="inlineStr">
@@ -5662,7 +5663,7 @@
         </is>
       </c>
       <c r="S23" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="24">
@@ -5698,13 +5699,13 @@
       <c r="J24" s="100" t="n"/>
       <c r="K24" s="100" t="inlineStr">
         <is>
-          <t>Avignon↔Uzès·Pont du Gard</t>
+          <t>Avignon Centre↔Arles TER</t>
         </is>
       </c>
       <c r="L24" s="100" t="n"/>
       <c r="M24" s="100" t="n"/>
       <c r="N24" s="100" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O24" s="100" t="inlineStr">
         <is>
@@ -5713,12 +5714,12 @@
       </c>
       <c r="P24" s="100" t="inlineStr">
         <is>
-          <t>주차·Pont</t>
+          <t>TER·JEP 재확인</t>
         </is>
       </c>
       <c r="Q24" s="100" t="inlineStr">
         <is>
-          <t>Pont 실내전시 삭제</t>
+          <t>선택시설 삭제</t>
         </is>
       </c>
       <c r="R24" s="100" t="inlineStr">
@@ -5727,7 +5728,7 @@
         </is>
       </c>
       <c r="S24" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="25">
@@ -5763,13 +5764,13 @@
       <c r="J25" s="100" t="n"/>
       <c r="K25" s="100" t="inlineStr">
         <is>
-          <t>Avignon Centre↔Arles 철도</t>
+          <t>성벽 안 도보</t>
         </is>
       </c>
       <c r="L25" s="100" t="n"/>
       <c r="M25" s="100" t="n"/>
       <c r="N25" s="100" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O25" s="100" t="inlineStr">
         <is>
@@ -5778,12 +5779,12 @@
       </c>
       <c r="P25" s="100" t="inlineStr">
         <is>
-          <t>TER·JEP 재확인</t>
+          <t>Palais·식당</t>
         </is>
       </c>
       <c r="Q25" s="100" t="inlineStr">
         <is>
-          <t>LUMA/Alyscamps/고대박물관 삭제</t>
+          <t>추가 미술관 삭제</t>
         </is>
       </c>
       <c r="R25" s="100" t="inlineStr">
@@ -5792,7 +5793,7 @@
         </is>
       </c>
       <c r="S25" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="26">
@@ -5819,7 +5820,7 @@
       </c>
       <c r="F26" s="100" t="inlineStr">
         <is>
-          <t>렌터카 반납·TGV·Lyon 도착</t>
+          <t>TGV 이동 &amp; Lyon 적응</t>
         </is>
       </c>
       <c r="G26" s="100" t="n"/>
@@ -5834,7 +5835,7 @@
       <c r="L26" s="100" t="n"/>
       <c r="M26" s="100" t="n"/>
       <c r="N26" s="100" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O26" s="100" t="inlineStr">
         <is>
@@ -5843,12 +5844,12 @@
       </c>
       <c r="P26" s="100" t="inlineStr">
         <is>
-          <t>렌터카·TGV 변경</t>
+          <t>TGV·짐 보관</t>
         </is>
       </c>
       <c r="Q26" s="100" t="inlineStr">
         <is>
-          <t>Lyon 도착 후 체크인만</t>
+          <t>Lyon 도착 후 숙소권 휴식</t>
         </is>
       </c>
       <c r="R26" s="100" t="inlineStr">
@@ -5857,7 +5858,7 @@
         </is>
       </c>
       <c r="S26" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="27">
@@ -8070,7 +8071,7 @@
       </c>
       <c r="D8" s="100" t="inlineStr">
         <is>
-          <t>Luberon 농가 숙소 3박</t>
+          <t>Gordes 숙소 2박</t>
         </is>
       </c>
       <c r="E8" s="119" t="n">
@@ -8112,15 +8113,15 @@
       </c>
       <c r="T8" s="100" t="inlineStr">
         <is>
-          <t>기존 4박→3박 예약 변경 필요; 입지·주방·세탁·주차</t>
+          <t>9/13 체크인·9/15 체크아웃·주차·야간 출입 확인</t>
         </is>
       </c>
       <c r="U8" s="119" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
       <c r="V8" s="63" t="inlineStr">
         <is>
-          <t>9/16 체크아웃으로 변경 완료 여부 미확인</t>
+          <t>Gordes 2박 숙소 후보 확정 필요</t>
         </is>
       </c>
     </row>
@@ -8142,11 +8143,11 @@
       </c>
       <c r="D9" s="100" t="inlineStr">
         <is>
-          <t>Avignon 숙소 4박</t>
+          <t>Avignon 숙소 5박</t>
         </is>
       </c>
       <c r="E9" s="119" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="F9" s="100" t="n"/>
       <c r="G9" s="100" t="inlineStr">
@@ -8184,15 +8185,15 @@
       </c>
       <c r="T9" s="100" t="inlineStr">
         <is>
-          <t>기존 9/17 체크인→9/16 변경 필요; 주차·TGV 반납 동선</t>
+          <t>9/15 체크인·9/20 체크아웃·성벽 안 생활권·주차 확인</t>
         </is>
       </c>
       <c r="U9" s="119" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
       <c r="V9" s="63" t="inlineStr">
         <is>
-          <t>예약 변경 필요</t>
+          <t>Avignon 5박 숙소 후보 확정 필요</t>
         </is>
       </c>
     </row>
@@ -8578,7 +8579,7 @@
       </c>
       <c r="F14" s="100" t="inlineStr">
         <is>
-          <t>9/9 09:00 인수 · 9/20 09:00 반납</t>
+          <t>계약 9/20 09:00 · 운영계획 9/17 18:30 이전 반납(변경 필요)</t>
         </is>
       </c>
       <c r="G14" s="100" t="inlineStr">
@@ -8634,15 +8635,15 @@
       </c>
       <c r="T14" s="100" t="inlineStr">
         <is>
-          <t>9/9 인수·9/20 반납으로 예약 변경 필요</t>
+          <t>기존 9/20 계약을 9/17 저녁 조기 반납으로 변경 필요</t>
         </is>
       </c>
       <c r="U14" s="119" t="n">
-        <v>46255</v>
+        <v>46259</v>
       </c>
       <c r="V14" s="63" t="inlineStr">
         <is>
-          <t>확약서 확인(2026-08-21): 계약 반납 9/20(일) 09:00 · Avignon TGV 지점 일요일 영업 10:00~19:00 이라 09:00 대면 반납 불가 · 결정 DEC-A08 은 9/19(토) 18:15 조기 반납</t>
+          <t>확약서 계약 반납은 9/20 09:00 · 일정 정본은 Day 20(9/17) 18:30 이전 반납 · 변경 완료 전 기존 바우처 조건 유효</t>
         </is>
       </c>
     </row>
@@ -9130,7 +9131,7 @@
         </is>
       </c>
       <c r="E21" s="119" t="n">
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="F21" s="100" t="n"/>
       <c r="G21" s="100" t="inlineStr">
@@ -9168,15 +9169,15 @@
       </c>
       <c r="T21" s="100" t="inlineStr">
         <is>
-          <t>결합권·입장시간</t>
+          <t>Day 22 Palais 결합권·입장시간 확인</t>
         </is>
       </c>
       <c r="U21" s="119" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
       <c r="V21" s="63" t="inlineStr">
         <is>
-          <t>기존 예약이 있으면 날짜 고정 여부 확인</t>
+          <t>Avignon 핵심 도보일은 9/19</t>
         </is>
       </c>
     </row>
@@ -10522,7 +10523,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Gordes</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -10534,7 +10535,7 @@
       <c r="I8" s="100" t="str"/>
       <c r="J8" s="100" t="inlineStr">
         <is>
-          <t>미조사</t>
+          <t>재확인</t>
         </is>
       </c>
       <c r="K8" s="100" t="str"/>
@@ -10542,17 +10543,17 @@
       <c r="M8" s="100" t="str"/>
       <c r="N8" s="100" t="inlineStr">
         <is>
-          <t>45분</t>
+          <t>약 1시간 10분</t>
         </is>
       </c>
       <c r="O8" s="100" t="inlineStr">
         <is>
-          <t>주차·농가 체크인</t>
+          <t>체크인·주차·차내수하물</t>
         </is>
       </c>
       <c r="P8" s="100" t="inlineStr">
         <is>
-          <t>경유마을 1곳만</t>
+          <t>Optional 마을 삭제</t>
         </is>
       </c>
       <c r="Q8" s="100" t="inlineStr">
@@ -10560,7 +10561,9 @@
           <t>07/08</t>
         </is>
       </c>
-      <c r="R8" s="119" t="str"/>
+      <c r="R8" s="119" t="n">
+        <v>46259</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
@@ -10569,11 +10572,11 @@
         </is>
       </c>
       <c r="B9" s="116" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Gordes</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -10598,17 +10601,17 @@
       <c r="M9" s="100" t="str"/>
       <c r="N9" s="100" t="inlineStr">
         <is>
-          <t>45분</t>
+          <t>약 1시간</t>
         </is>
       </c>
       <c r="O9" s="100" t="inlineStr">
         <is>
-          <t>농가 3박·Avignon 9/16 체크인 변경</t>
+          <t>Gordes 체크아웃·Avignon 5박 체크인</t>
         </is>
       </c>
       <c r="P9" s="100" t="inlineStr">
         <is>
-          <t>Avignon 직행</t>
+          <t>Fontaine 삭제 후 직행</t>
         </is>
       </c>
       <c r="Q9" s="100" t="inlineStr">
@@ -10617,7 +10620,7 @@
         </is>
       </c>
       <c r="R9" s="119" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="10">
@@ -10641,7 +10644,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>렌터카 반납+TGV</t>
+          <t>TGV</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -10669,22 +10672,22 @@
       <c r="L10" s="100" t="str"/>
       <c r="M10" s="100" t="inlineStr">
         <is>
-          <t>Avignon TGV역 09:00 반납 후 승차</t>
+          <t>차량 절차 없이 Avignon TGV에서 승차</t>
         </is>
       </c>
       <c r="N10" s="100" t="inlineStr">
         <is>
-          <t>90분</t>
+          <t>역 도착 40분 이상 여유</t>
         </is>
       </c>
       <c r="O10" s="100" t="inlineStr">
         <is>
-          <t>렌터카 반납·TGV 날짜 변경 필요</t>
+          <t>수하물·플랫폼·짐 보관</t>
         </is>
       </c>
       <c r="P10" s="100" t="inlineStr">
         <is>
-          <t>더 이른 열차 또는 택시</t>
+          <t>도착 후 숙소권 휴식</t>
         </is>
       </c>
       <c r="Q10" s="100" t="inlineStr">
@@ -10693,7 +10696,7 @@
         </is>
       </c>
       <c r="R10" s="119" t="n">
-        <v>46243</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="11">
@@ -12047,7 +12050,7 @@
       </c>
       <c r="H8" s="100" t="inlineStr">
         <is>
-          <t>5+4+4·주차·당일치기·렌터카</t>
+          <t>Aix 4박·Gordes 2박·Avignon 5박·9/17 차량 반납</t>
         </is>
       </c>
       <c r="I8" s="100" t="str"/>
@@ -13648,12 +13651,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>재확인</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F17" s="63" t="inlineStr">
         <is>
-          <t>9/13~9/16 · 3박 · 예약 변경 필요</t>
+          <t>9/13~9/15 · Gordes 2박</t>
         </is>
       </c>
     </row>
@@ -13668,7 +13671,7 @@
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>Marseille / Arles</t>
+          <t>Avignon allocation</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -13678,7 +13681,7 @@
       </c>
       <c r="F18" s="63" t="inlineStr">
         <is>
-          <t>9/11·9/19 기본 일정</t>
+          <t>9/15~9/20 · 5박 · 9/17 차량 반납</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(itinerary): align Provence content with canonical schedule (#220)
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -2214,6 +2214,7 @@
       <c r="G1" s="98" t="n"/>
       <c r="H1" s="98" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="88" t="inlineStr">
         <is>
@@ -2726,17 +2727,17 @@
       </c>
       <c r="B15" s="100" t="inlineStr">
         <is>
-          <t>Gordes</t>
+          <t>L'Isle-sur-la-Sorgue·Avignon</t>
         </is>
       </c>
       <c r="C15" s="100" t="inlineStr">
         <is>
-          <t>시장·돌마을·장바구니</t>
+          <t>수로·물레방아·Avignon 체크인</t>
         </is>
       </c>
       <c r="D15" s="100" t="inlineStr">
         <is>
-          <t>오전</t>
+          <t>오전·오후</t>
         </is>
       </c>
       <c r="E15" s="100" t="inlineStr">
@@ -2746,7 +2747,7 @@
       </c>
       <c r="F15" s="100" t="inlineStr">
         <is>
-          <t>마을생활</t>
+          <t>물의 Provence·거점 전환</t>
         </is>
       </c>
       <c r="G15" s="100" t="inlineStr">
@@ -2768,17 +2769,17 @@
       </c>
       <c r="B16" s="100" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Saint-Rémy·Les Baux</t>
         </is>
       </c>
       <c r="C16" s="100" t="inlineStr">
         <is>
-          <t>농가 식탁·스케치·세탁</t>
+          <t>수요시장·석회암 마을</t>
         </is>
       </c>
       <c r="D16" s="100" t="inlineStr">
         <is>
-          <t>오후</t>
+          <t>오전·오후</t>
         </is>
       </c>
       <c r="E16" s="100" t="inlineStr">
@@ -2788,7 +2789,7 @@
       </c>
       <c r="F16" s="100" t="inlineStr">
         <is>
-          <t>농가체험 핵심</t>
+          <t>시장·Alpilles</t>
         </is>
       </c>
       <c r="G16" s="100" t="inlineStr">
@@ -2810,17 +2811,17 @@
       </c>
       <c r="B17" s="100" t="inlineStr">
         <is>
-          <t>Avignon</t>
+          <t>Arles</t>
         </is>
       </c>
       <c r="C17" s="100" t="inlineStr">
         <is>
-          <t>Palais–Pont 파노라마</t>
+          <t>Arènes·Théâtre·Saint-Trophime</t>
         </is>
       </c>
       <c r="D17" s="100" t="inlineStr">
         <is>
-          <t>오후</t>
+          <t>전일</t>
         </is>
       </c>
       <c r="E17" s="100" t="inlineStr">
@@ -2830,7 +2831,7 @@
       </c>
       <c r="F17" s="100" t="inlineStr">
         <is>
-          <t>도시상징</t>
+          <t>JEP·로마유산</t>
         </is>
       </c>
       <c r="G17" s="100" t="inlineStr">
@@ -2852,17 +2853,17 @@
       </c>
       <c r="B18" s="100" t="inlineStr">
         <is>
-          <t>Uzès</t>
+          <t>Avignon</t>
         </is>
       </c>
       <c r="C18" s="100" t="inlineStr">
         <is>
-          <t>시장 장보기</t>
+          <t>Les Halles·Palais·Rocher·Pont</t>
         </is>
       </c>
       <c r="D18" s="100" t="inlineStr">
         <is>
-          <t>오전</t>
+          <t>전일</t>
         </is>
       </c>
       <c r="E18" s="100" t="inlineStr">
@@ -2872,7 +2873,7 @@
       </c>
       <c r="F18" s="100" t="inlineStr">
         <is>
-          <t>프로방스 시장</t>
+          <t>교황도시 핵심</t>
         </is>
       </c>
       <c r="G18" s="100" t="inlineStr">
@@ -3289,7 +3290,7 @@
       </c>
       <c r="G4" s="100" t="inlineStr">
         <is>
-          <t>Nice 5·Aix 4·Luberon 3·Avignon 4·Lyon 4·Paris 15박 + 기내 1박(10/9→10/10)</t>
+          <t>Barcelona 3·Bàscara 3·Nice 5·Aix 4·Gordes 2·Avignon 5·Lyon 4·Paris 15박 + 기내 1박</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3312,7 @@
       </c>
       <c r="D5" s="100" t="inlineStr">
         <is>
-          <t>3/3/5/4/3/4/4/15박</t>
+          <t>3/3/5/4/2/5/4/15박</t>
         </is>
       </c>
       <c r="E5" s="100" t="inlineStr">
@@ -3326,7 +3327,7 @@
       </c>
       <c r="G5" s="100" t="inlineStr">
         <is>
-          <t>Luberon·Avignon·Lyon·Paris 기존 예약 변경 필요 · 마지막 밤은 기내</t>
+          <t>Gordes·Avignon 숙소 후보 확정 필요 · 마지막 밤은 기내</t>
         </is>
       </c>
     </row>
@@ -3488,12 +3489,12 @@
       </c>
       <c r="D10" s="100" t="inlineStr">
         <is>
-          <t>9/9 NCE 인수, 9/20 Avignon 반납</t>
+          <t>9/9 Nice-Ville 인수, 9/17 Avignon TGV 반납</t>
         </is>
       </c>
       <c r="E10" s="100" t="inlineStr">
         <is>
-          <t>업체·예약번호·9/20 반납 변경 확인</t>
+          <t>기존 9/20 계약을 9/17 18:30 이전 반납으로 변경</t>
         </is>
       </c>
       <c r="F10" s="100" t="inlineStr">
@@ -3717,7 +3718,7 @@
       </c>
       <c r="B17" s="100" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Gordes</t>
         </is>
       </c>
       <c r="C17" s="100" t="inlineStr">
@@ -3727,12 +3728,12 @@
       </c>
       <c r="D17" s="100" t="inlineStr">
         <is>
-          <t>3박 · 예약 변경 필요</t>
+          <t>2박 · 9/13~9/15</t>
         </is>
       </c>
       <c r="E17" s="100" t="inlineStr">
         <is>
-          <t>기존 4박 예약을 9/13~9/16으로 변경</t>
+          <t>숙소 후보·주차·체크인 확정</t>
         </is>
       </c>
       <c r="F17" s="100" t="inlineStr">
@@ -3760,12 +3761,12 @@
       </c>
       <c r="D18" s="100" t="inlineStr">
         <is>
-          <t>4박 · 9/16~9/20</t>
+          <t>5박 · 9/15~9/20</t>
         </is>
       </c>
       <c r="E18" s="100" t="inlineStr">
         <is>
-          <t>기존 체크인일 변경 확인</t>
+          <t>숙소 후보·주차·체크인 확정</t>
         </is>
       </c>
       <c r="F18" s="100" t="inlineStr">
@@ -3996,7 +3997,7 @@
     <row r="1" ht="30" customHeight="1" s="92">
       <c r="A1" s="115" t="inlineStr">
         <is>
-          <t>TP Europe Travel — Master Itinerary v1.2 (43일·42박 · Paris 16박)</t>
+          <t>TP Europe Travel — Master Itinerary v1.2 (43일·42박 · Paris 15박 + 기내 1박)</t>
         </is>
       </c>
       <c r="B1" s="98" t="n"/>
@@ -5373,13 +5374,13 @@
       <c r="J19" s="100" t="n"/>
       <c r="K19" s="100" t="inlineStr">
         <is>
-          <t>Aix→Lourmarin→농가</t>
+          <t>Aix→Lourmarin→Gordes</t>
         </is>
       </c>
       <c r="L19" s="100" t="n"/>
       <c r="M19" s="100" t="n"/>
       <c r="N19" s="100" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O19" s="100" t="inlineStr">
         <is>
@@ -5388,12 +5389,12 @@
       </c>
       <c r="P19" s="100" t="inlineStr">
         <is>
-          <t>농가 3박 변경</t>
+          <t>Gordes 2박·Lourmarin 점심</t>
         </is>
       </c>
       <c r="Q19" s="100" t="inlineStr">
         <is>
-          <t>경유지 축소</t>
+          <t>Lacoste→Bonnieux 순으로 삭제</t>
         </is>
       </c>
       <c r="R19" s="100" t="inlineStr">
@@ -5402,7 +5403,7 @@
         </is>
       </c>
       <c r="S19" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="20">
@@ -5438,7 +5439,7 @@
       <c r="J20" s="100" t="n"/>
       <c r="K20" s="100" t="inlineStr">
         <is>
-          <t>농가↔Roussillon·선택마을</t>
+          <t>Gordes↔Roussillon·Sénanque</t>
         </is>
       </c>
       <c r="L20" s="100" t="n"/>
@@ -5453,12 +5454,12 @@
       </c>
       <c r="P20" s="100" t="inlineStr">
         <is>
-          <t>주차·오커길</t>
+          <t>Sénanque 슬롯·오커길</t>
         </is>
       </c>
       <c r="Q20" s="100" t="inlineStr">
         <is>
-          <t>두 번째 마을 삭제</t>
+          <t>Goult→Ménerbes 순으로 삭제</t>
         </is>
       </c>
       <c r="R20" s="100" t="inlineStr">
@@ -5467,7 +5468,7 @@
         </is>
       </c>
       <c r="S20" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="21">
@@ -5503,7 +5504,7 @@
       <c r="J21" s="100" t="n"/>
       <c r="K21" s="100" t="inlineStr">
         <is>
-          <t>농가↔Gordes·Bories</t>
+          <t>Gordes→L'Isle→Avignon</t>
         </is>
       </c>
       <c r="L21" s="100" t="n"/>
@@ -5518,21 +5519,21 @@
       </c>
       <c r="P21" s="100" t="inlineStr">
         <is>
-          <t>시장·주차</t>
+          <t>Avignon 5박·주차</t>
         </is>
       </c>
       <c r="Q21" s="100" t="inlineStr">
         <is>
-          <t>Ménerbes/Oppède 삭제</t>
+          <t>Fontaine 삭제 후 Avignon 직행</t>
         </is>
       </c>
       <c r="R21" s="100" t="inlineStr">
         <is>
-          <t>08_Luberon_Farmhouse_v2.0.md</t>
+          <t>09_Avignon_Alpilles_Pont_du_Gard_v2.0.md</t>
         </is>
       </c>
       <c r="S21" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="22">
@@ -5568,13 +5569,13 @@
       <c r="J22" s="100" t="n"/>
       <c r="K22" s="100" t="inlineStr">
         <is>
-          <t>Luberon→Avignon</t>
+          <t>Avignon↔Saint-Rémy·Les Baux</t>
         </is>
       </c>
       <c r="L22" s="100" t="n"/>
       <c r="M22" s="100" t="n"/>
       <c r="N22" s="100" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O22" s="100" t="inlineStr">
         <is>
@@ -5583,12 +5584,12 @@
       </c>
       <c r="P22" s="100" t="inlineStr">
         <is>
-          <t>농가·Avignon 숙소 변경</t>
+          <t>시장·Château 운영</t>
         </is>
       </c>
       <c r="Q22" s="100" t="inlineStr">
         <is>
-          <t>추가마을·저녁관람 삭제</t>
+          <t>Orange 삭제</t>
         </is>
       </c>
       <c r="R22" s="100" t="inlineStr">
@@ -5597,7 +5598,7 @@
         </is>
       </c>
       <c r="S22" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="23">
@@ -5633,13 +5634,13 @@
       <c r="J23" s="100" t="n"/>
       <c r="K23" s="100" t="inlineStr">
         <is>
-          <t>성벽 안 도보</t>
+          <t>Avignon→Uzès→Pont du Gard→Nîmes→Avignon TGV</t>
         </is>
       </c>
       <c r="L23" s="100" t="n"/>
       <c r="M23" s="100" t="n"/>
       <c r="N23" s="100" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O23" s="100" t="inlineStr">
         <is>
@@ -5648,12 +5649,12 @@
       </c>
       <c r="P23" s="100" t="inlineStr">
         <is>
-          <t>Palais des Papes</t>
+          <t>18:30 이전 Hertz 조기 반납</t>
         </is>
       </c>
       <c r="Q23" s="100" t="inlineStr">
         <is>
-          <t>추가 미술관 삭제</t>
+          <t>Nîmes 체류부터 축소</t>
         </is>
       </c>
       <c r="R23" s="100" t="inlineStr">
@@ -5662,7 +5663,7 @@
         </is>
       </c>
       <c r="S23" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="24">
@@ -5698,13 +5699,13 @@
       <c r="J24" s="100" t="n"/>
       <c r="K24" s="100" t="inlineStr">
         <is>
-          <t>Avignon↔Uzès·Pont du Gard</t>
+          <t>Avignon Centre↔Arles TER</t>
         </is>
       </c>
       <c r="L24" s="100" t="n"/>
       <c r="M24" s="100" t="n"/>
       <c r="N24" s="100" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O24" s="100" t="inlineStr">
         <is>
@@ -5713,12 +5714,12 @@
       </c>
       <c r="P24" s="100" t="inlineStr">
         <is>
-          <t>주차·Pont</t>
+          <t>TER·JEP 재확인</t>
         </is>
       </c>
       <c r="Q24" s="100" t="inlineStr">
         <is>
-          <t>Pont 실내전시 삭제</t>
+          <t>선택시설 삭제</t>
         </is>
       </c>
       <c r="R24" s="100" t="inlineStr">
@@ -5727,7 +5728,7 @@
         </is>
       </c>
       <c r="S24" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="25">
@@ -5763,13 +5764,13 @@
       <c r="J25" s="100" t="n"/>
       <c r="K25" s="100" t="inlineStr">
         <is>
-          <t>Avignon Centre↔Arles 철도</t>
+          <t>성벽 안 도보</t>
         </is>
       </c>
       <c r="L25" s="100" t="n"/>
       <c r="M25" s="100" t="n"/>
       <c r="N25" s="100" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O25" s="100" t="inlineStr">
         <is>
@@ -5778,12 +5779,12 @@
       </c>
       <c r="P25" s="100" t="inlineStr">
         <is>
-          <t>TER·JEP 재확인</t>
+          <t>Palais·식당</t>
         </is>
       </c>
       <c r="Q25" s="100" t="inlineStr">
         <is>
-          <t>LUMA/Alyscamps/고대박물관 삭제</t>
+          <t>추가 미술관 삭제</t>
         </is>
       </c>
       <c r="R25" s="100" t="inlineStr">
@@ -5792,7 +5793,7 @@
         </is>
       </c>
       <c r="S25" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="26">
@@ -5819,7 +5820,7 @@
       </c>
       <c r="F26" s="100" t="inlineStr">
         <is>
-          <t>렌터카 반납·TGV·Lyon 도착</t>
+          <t>TGV 이동 &amp; Lyon 적응</t>
         </is>
       </c>
       <c r="G26" s="100" t="n"/>
@@ -5834,7 +5835,7 @@
       <c r="L26" s="100" t="n"/>
       <c r="M26" s="100" t="n"/>
       <c r="N26" s="100" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O26" s="100" t="inlineStr">
         <is>
@@ -5843,12 +5844,12 @@
       </c>
       <c r="P26" s="100" t="inlineStr">
         <is>
-          <t>렌터카·TGV 변경</t>
+          <t>TGV·짐 보관</t>
         </is>
       </c>
       <c r="Q26" s="100" t="inlineStr">
         <is>
-          <t>Lyon 도착 후 체크인만</t>
+          <t>Lyon 도착 후 숙소권 휴식</t>
         </is>
       </c>
       <c r="R26" s="100" t="inlineStr">
@@ -5857,7 +5858,7 @@
         </is>
       </c>
       <c r="S26" s="117" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="27">
@@ -8070,7 +8071,7 @@
       </c>
       <c r="D8" s="100" t="inlineStr">
         <is>
-          <t>Luberon 농가 숙소 3박</t>
+          <t>Gordes 숙소 2박</t>
         </is>
       </c>
       <c r="E8" s="119" t="n">
@@ -8112,15 +8113,15 @@
       </c>
       <c r="T8" s="100" t="inlineStr">
         <is>
-          <t>기존 4박→3박 예약 변경 필요; 입지·주방·세탁·주차</t>
+          <t>9/13 체크인·9/15 체크아웃·주차·야간 출입 확인</t>
         </is>
       </c>
       <c r="U8" s="119" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
       <c r="V8" s="63" t="inlineStr">
         <is>
-          <t>9/16 체크아웃으로 변경 완료 여부 미확인</t>
+          <t>Gordes 2박 숙소 후보 확정 필요</t>
         </is>
       </c>
     </row>
@@ -8142,11 +8143,11 @@
       </c>
       <c r="D9" s="100" t="inlineStr">
         <is>
-          <t>Avignon 숙소 4박</t>
+          <t>Avignon 숙소 5박</t>
         </is>
       </c>
       <c r="E9" s="119" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="F9" s="100" t="n"/>
       <c r="G9" s="100" t="inlineStr">
@@ -8184,15 +8185,15 @@
       </c>
       <c r="T9" s="100" t="inlineStr">
         <is>
-          <t>기존 9/17 체크인→9/16 변경 필요; 주차·TGV 반납 동선</t>
+          <t>9/15 체크인·9/20 체크아웃·성벽 안 생활권·주차 확인</t>
         </is>
       </c>
       <c r="U9" s="119" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
       <c r="V9" s="63" t="inlineStr">
         <is>
-          <t>예약 변경 필요</t>
+          <t>Avignon 5박 숙소 후보 확정 필요</t>
         </is>
       </c>
     </row>
@@ -8578,7 +8579,7 @@
       </c>
       <c r="F14" s="100" t="inlineStr">
         <is>
-          <t>9/9 09:00 인수 · 9/20 09:00 반납</t>
+          <t>계약 9/20 09:00 · 운영계획 9/17 18:30 이전 반납(변경 필요)</t>
         </is>
       </c>
       <c r="G14" s="100" t="inlineStr">
@@ -8634,15 +8635,15 @@
       </c>
       <c r="T14" s="100" t="inlineStr">
         <is>
-          <t>9/9 인수·9/20 반납으로 예약 변경 필요</t>
+          <t>기존 9/20 계약을 9/17 저녁 조기 반납으로 변경 필요</t>
         </is>
       </c>
       <c r="U14" s="119" t="n">
-        <v>46255</v>
+        <v>46259</v>
       </c>
       <c r="V14" s="63" t="inlineStr">
         <is>
-          <t>확약서 확인(2026-08-21): 계약 반납 9/20(일) 09:00 · Avignon TGV 지점 일요일 영업 10:00~19:00 이라 09:00 대면 반납 불가 · 결정 DEC-A08 은 9/19(토) 18:15 조기 반납</t>
+          <t>확약서 계약 반납은 9/20 09:00 · 일정 정본은 Day 20(9/17) 18:30 이전 반납 · 변경 완료 전 기존 바우처 조건 유효</t>
         </is>
       </c>
     </row>
@@ -9130,7 +9131,7 @@
         </is>
       </c>
       <c r="E21" s="119" t="n">
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="F21" s="100" t="n"/>
       <c r="G21" s="100" t="inlineStr">
@@ -9168,15 +9169,15 @@
       </c>
       <c r="T21" s="100" t="inlineStr">
         <is>
-          <t>결합권·입장시간</t>
+          <t>Day 22 Palais 결합권·입장시간 확인</t>
         </is>
       </c>
       <c r="U21" s="119" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
       <c r="V21" s="63" t="inlineStr">
         <is>
-          <t>기존 예약이 있으면 날짜 고정 여부 확인</t>
+          <t>Avignon 핵심 도보일은 9/19</t>
         </is>
       </c>
     </row>
@@ -10522,7 +10523,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Gordes</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -10534,7 +10535,7 @@
       <c r="I8" s="100" t="str"/>
       <c r="J8" s="100" t="inlineStr">
         <is>
-          <t>미조사</t>
+          <t>재확인</t>
         </is>
       </c>
       <c r="K8" s="100" t="str"/>
@@ -10542,17 +10543,17 @@
       <c r="M8" s="100" t="str"/>
       <c r="N8" s="100" t="inlineStr">
         <is>
-          <t>45분</t>
+          <t>약 1시간 10분</t>
         </is>
       </c>
       <c r="O8" s="100" t="inlineStr">
         <is>
-          <t>주차·농가 체크인</t>
+          <t>체크인·주차·차내수하물</t>
         </is>
       </c>
       <c r="P8" s="100" t="inlineStr">
         <is>
-          <t>경유마을 1곳만</t>
+          <t>Optional 마을 삭제</t>
         </is>
       </c>
       <c r="Q8" s="100" t="inlineStr">
@@ -10560,7 +10561,9 @@
           <t>07/08</t>
         </is>
       </c>
-      <c r="R8" s="119" t="str"/>
+      <c r="R8" s="119" t="n">
+        <v>46259</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
@@ -10569,11 +10572,11 @@
         </is>
       </c>
       <c r="B9" s="116" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Luberon</t>
+          <t>Gordes</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -10598,17 +10601,17 @@
       <c r="M9" s="100" t="str"/>
       <c r="N9" s="100" t="inlineStr">
         <is>
-          <t>45분</t>
+          <t>약 1시간</t>
         </is>
       </c>
       <c r="O9" s="100" t="inlineStr">
         <is>
-          <t>농가 3박·Avignon 9/16 체크인 변경</t>
+          <t>Gordes 체크아웃·Avignon 5박 체크인</t>
         </is>
       </c>
       <c r="P9" s="100" t="inlineStr">
         <is>
-          <t>Avignon 직행</t>
+          <t>Fontaine 삭제 후 직행</t>
         </is>
       </c>
       <c r="Q9" s="100" t="inlineStr">
@@ -10617,7 +10620,7 @@
         </is>
       </c>
       <c r="R9" s="119" t="n">
-        <v>46238</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="10">
@@ -10641,7 +10644,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>렌터카 반납+TGV</t>
+          <t>TGV</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -10669,22 +10672,22 @@
       <c r="L10" s="100" t="str"/>
       <c r="M10" s="100" t="inlineStr">
         <is>
-          <t>Avignon TGV역 09:00 반납 후 승차</t>
+          <t>차량 절차 없이 Avignon TGV에서 승차</t>
         </is>
       </c>
       <c r="N10" s="100" t="inlineStr">
         <is>
-          <t>90분</t>
+          <t>역 도착 40분 이상 여유</t>
         </is>
       </c>
       <c r="O10" s="100" t="inlineStr">
         <is>
-          <t>렌터카 반납·TGV 날짜 변경 필요</t>
+          <t>수하물·플랫폼·짐 보관</t>
         </is>
       </c>
       <c r="P10" s="100" t="inlineStr">
         <is>
-          <t>더 이른 열차 또는 택시</t>
+          <t>도착 후 숙소권 휴식</t>
         </is>
       </c>
       <c r="Q10" s="100" t="inlineStr">
@@ -10693,7 +10696,7 @@
         </is>
       </c>
       <c r="R10" s="119" t="n">
-        <v>46243</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="11">
@@ -12047,7 +12050,7 @@
       </c>
       <c r="H8" s="100" t="inlineStr">
         <is>
-          <t>5+4+4·주차·당일치기·렌터카</t>
+          <t>Aix 4박·Gordes 2박·Avignon 5박·9/17 차량 반납</t>
         </is>
       </c>
       <c r="I8" s="100" t="str"/>
@@ -13648,12 +13651,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>재확인</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F17" s="63" t="inlineStr">
         <is>
-          <t>9/13~9/16 · 3박 · 예약 변경 필요</t>
+          <t>9/13~9/15 · Gordes 2박</t>
         </is>
       </c>
     </row>
@@ -13668,7 +13671,7 @@
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>Marseille / Arles</t>
+          <t>Avignon allocation</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -13678,7 +13681,7 @@
       </c>
       <c r="F18" s="63" t="inlineStr">
         <is>
-          <t>9/11·9/19 기본 일정</t>
+          <t>9/15~9/20 · 5박 · 9/17 차량 반납</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RS01 CI fix: 배포 실패 2건 해소 — validate_itinerary 구일정 기대값·트래커 Accommodation 시트·장소 링크 (#235)
- scripts/validate_itinerary.py: R005/R006 기대값(9/14·9/16 4박), Day 12/13/14/16 필수 콘텐츠 맵,
  선택안 금지 링크(day-16), 홈 정본/폐기 패턴(5박↔4박) — RS01 기준으로 갱신
- 트래커 Accommodation 시트: Moustiers 1박 행 신설, Aix/Gordes/Avignon 날짜·박수 갱신
- 신규 장소 5곳 공식정보 bare URL → 마크다운 링크 (ux_check 통과)
- CI Build 파이프라인 9종 + 테스트 155개 전부 통과 재현


Claude-Session: https://claude.ai/code/session_01TWV79mSYmwdvVVhtquLh7R

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -2214,7 +2214,6 @@
       <c r="G1" s="98" t="n"/>
       <c r="H1" s="98" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="88" t="inlineStr">
         <is>
@@ -10890,7 +10889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:T12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="92" min="1" max="1"/>
@@ -11282,104 +11281,64 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>Aix-en-Provence</t>
-        </is>
-      </c>
-      <c r="B7" s="116" t="n">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Moustiers-Sainte-Marie</t>
+        </is>
+      </c>
+      <c r="B7" s="128" t="n">
         <v>46274</v>
       </c>
-      <c r="C7" s="116" t="n">
-        <v>46278</v>
+      <c r="C7" s="128" t="n">
+        <v>46275</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>예약완료</t>
-        </is>
-      </c>
-      <c r="F7" s="100" t="inlineStr">
-        <is>
-          <t>Résidence Les Toits de Méjanes (Méjanes 도서관 권역)</t>
-        </is>
-      </c>
-      <c r="G7" s="100" t="inlineStr">
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Moustiers 마을 또는 인근 생활권 (현지 결정)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="H7" s="120" t="n"/>
-      <c r="I7" s="120" t="n"/>
-      <c r="J7" s="120" t="n"/>
-      <c r="K7" s="119" t="n"/>
-      <c r="L7" s="100" t="inlineStr">
-        <is>
-          <t>HMSSBEA4PJ · Airbnb</t>
-        </is>
-      </c>
-      <c r="M7" s="100" t="inlineStr">
-        <is>
-          <t>2 Place Coimbra, Résidence Les Toits de Méjanes, entrée A, 6e étage, 13090 Aix-en-Provence, France</t>
-        </is>
-      </c>
-      <c r="N7" s="100" t="inlineStr">
-        <is>
-          <t>체크인 15:00 / 체크아웃 14:00</t>
-        </is>
-      </c>
-      <c r="O7" s="100" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="P7" s="100" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="Q7" s="100" t="inlineStr">
-        <is>
-          <t>필수</t>
-        </is>
-      </c>
-      <c r="R7" s="100" t="inlineStr">
-        <is>
-          <t>확인</t>
-        </is>
-      </c>
-      <c r="S7" s="100" t="n"/>
-      <c r="T7" s="63" t="inlineStr">
-        <is>
-          <t>4박·주차·주방·9/11 Marseille 기본</t>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>RS01: Verdon 1박 신설 — 도착 전 확보 최우선</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>Gordes</t>
+          <t>Aix-en-Provence</t>
         </is>
       </c>
       <c r="B8" s="116" t="n">
-        <v>46278</v>
+        <v>46275</v>
       </c>
       <c r="C8" s="116" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>재확인</t>
+          <t>예약완료</t>
         </is>
       </c>
       <c r="F8" s="100" t="inlineStr">
         <is>
-          <t>Gordes 및 루베롱 북부 권역 (후보 미정)</t>
+          <t>Résidence Les Toits de Méjanes (Méjanes 도서관 권역)</t>
         </is>
       </c>
       <c r="G8" s="100" t="inlineStr">
@@ -11390,10 +11349,22 @@
       <c r="H8" s="120" t="n"/>
       <c r="I8" s="120" t="n"/>
       <c r="J8" s="120" t="n"/>
-      <c r="K8" s="119" t="str"/>
-      <c r="L8" s="100" t="str"/>
-      <c r="M8" s="100" t="str"/>
-      <c r="N8" s="100" t="str"/>
+      <c r="K8" s="119" t="n"/>
+      <c r="L8" s="100" t="inlineStr">
+        <is>
+          <t>HMSSBEA4PJ · Airbnb</t>
+        </is>
+      </c>
+      <c r="M8" s="100" t="inlineStr">
+        <is>
+          <t>2 Place Coimbra, Résidence Les Toits de Méjanes, entrée A, 6e étage, 13090 Aix-en-Provence, France</t>
+        </is>
+      </c>
+      <c r="N8" s="100" t="inlineStr">
+        <is>
+          <t>체크인 15:00 / 체크아웃 14:00</t>
+        </is>
+      </c>
       <c r="O8" s="100" t="inlineStr">
         <is>
           <t>필수</t>
@@ -11414,27 +11385,27 @@
           <t>확인</t>
         </is>
       </c>
-      <c r="S8" s="100" t="str"/>
+      <c r="S8" s="100" t="n"/>
       <c r="T8" s="63" t="inlineStr">
         <is>
-          <t>Gordes 2박 숙소 후보 확정 필요</t>
+          <t>RS01: 9/10 체크인·9/14 체크아웃으로 날짜 변경 완료 (예약 유지)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>Avignon</t>
+          <t>Gordes</t>
         </is>
       </c>
       <c r="B9" s="116" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="C9" s="116" t="n">
-        <v>46285</v>
+        <v>46281</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -11443,7 +11414,7 @@
       </c>
       <c r="F9" s="100" t="inlineStr">
         <is>
-          <t>성벽 안(intra-muros) 도보 생활권 · La Terrasse du Clocher 등</t>
+          <t>Gordes 및 루베롱 북부 권역 (후보 미정)</t>
         </is>
       </c>
       <c r="G9" s="100" t="inlineStr">
@@ -11460,12 +11431,12 @@
       <c r="N9" s="100" t="str"/>
       <c r="O9" s="100" t="inlineStr">
         <is>
-          <t>선호</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="P9" s="100" t="inlineStr">
         <is>
-          <t>선호</t>
+          <t>필수</t>
         </is>
       </c>
       <c r="Q9" s="100" t="inlineStr">
@@ -11481,33 +11452,33 @@
       <c r="S9" s="100" t="str"/>
       <c r="T9" s="63" t="inlineStr">
         <is>
-          <t>Avignon 5박 숙소·주차·체크인 창 확정 필요</t>
+          <t>RS01: 9/14~9/16으로 변경 · 후보 미정</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Avignon</t>
         </is>
       </c>
       <c r="B10" s="116" t="n">
+        <v>46281</v>
+      </c>
+      <c r="C10" s="116" t="n">
         <v>46285</v>
-      </c>
-      <c r="C10" s="116" t="n">
-        <v>46289</v>
       </c>
       <c r="D10" t="n">
         <v>4</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>예약완료</t>
+          <t>재확인</t>
         </is>
       </c>
       <c r="F10" s="100" t="inlineStr">
         <is>
-          <t>Lagrange Aparthotel Lyon Lumière · Monplaisir (3구)</t>
+          <t>성벽 안(intra-muros) 도보 생활권 · La Terrasse du Clocher 등</t>
         </is>
       </c>
       <c r="G10" s="100" t="inlineStr">
@@ -11516,126 +11487,190 @@
         </is>
       </c>
       <c r="H10" s="120" t="n"/>
-      <c r="I10" s="120" t="n">
-        <v>433.82</v>
-      </c>
+      <c r="I10" s="120" t="n"/>
       <c r="J10" s="120" t="n"/>
       <c r="K10" s="119" t="str"/>
-      <c r="L10" s="100" t="inlineStr">
+      <c r="L10" s="100" t="str"/>
+      <c r="M10" s="100" t="str"/>
+      <c r="N10" s="100" t="str"/>
+      <c r="O10" s="100" t="inlineStr">
+        <is>
+          <t>선호</t>
+        </is>
+      </c>
+      <c r="P10" s="100" t="inlineStr">
+        <is>
+          <t>선호</t>
+        </is>
+      </c>
+      <c r="Q10" s="100" t="inlineStr">
+        <is>
+          <t>필수</t>
+        </is>
+      </c>
+      <c r="R10" s="100" t="inlineStr">
+        <is>
+          <t>확인</t>
+        </is>
+      </c>
+      <c r="S10" s="100" t="str"/>
+      <c r="T10" s="63" t="inlineStr">
+        <is>
+          <t>RS01: 4박으로 축소 (9/16~9/20) · 후보 미정</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="B11" s="116" t="n">
+        <v>46285</v>
+      </c>
+      <c r="C11" s="116" t="n">
+        <v>46289</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>예약완료</t>
+        </is>
+      </c>
+      <c r="F11" s="100" t="inlineStr">
+        <is>
+          <t>Lagrange Aparthotel Lyon Lumière · Monplaisir (3구)</t>
+        </is>
+      </c>
+      <c r="G11" s="100" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H11" s="120" t="n"/>
+      <c r="I11" s="120" t="n">
+        <v>433.82</v>
+      </c>
+      <c r="J11" s="120" t="n"/>
+      <c r="K11" s="119" t="str"/>
+      <c r="L11" s="100" t="inlineStr">
         <is>
           <t>5882.730.884</t>
         </is>
       </c>
-      <c r="M10" s="100" t="inlineStr">
+      <c r="M11" s="100" t="inlineStr">
         <is>
           <t>81-85 Cours Albert Thomas, 69003 Lyon, France</t>
         </is>
       </c>
-      <c r="N10" s="100" t="inlineStr">
+      <c r="N11" s="100" t="inlineStr">
         <is>
           <t>체크인 9/20 15:00 · 체크아웃 9/24 11:00</t>
         </is>
       </c>
-      <c r="O10" s="100" t="inlineStr">
+      <c r="O11" s="100" t="inlineStr">
         <is>
           <t>선호</t>
         </is>
       </c>
-      <c r="P10" s="100" t="inlineStr">
+      <c r="P11" s="100" t="inlineStr">
         <is>
           <t>선호</t>
         </is>
       </c>
-      <c r="Q10" s="100" t="inlineStr">
+      <c r="Q11" s="100" t="inlineStr">
         <is>
           <t>불필요</t>
         </is>
       </c>
-      <c r="R10" s="100" t="inlineStr">
+      <c r="R11" s="100" t="inlineStr">
         <is>
           <t>필수</t>
         </is>
       </c>
-      <c r="S10" s="100" t="inlineStr">
+      <c r="S11" s="100" t="inlineStr">
         <is>
           <t>https://www.booking.com</t>
         </is>
       </c>
-      <c r="T10" s="63" t="inlineStr">
+      <c r="T11" s="63" t="inlineStr">
         <is>
           <t>2026-08-14 예약 확정 · booking.com · €433.82 · 전화 +33 4 81 76 28 00 · 메트로 D Sans Souci·Monplaisir-Lumière 도보권 · 아파트호텔(주방)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="B11" s="116" t="n">
+      <c r="B12" s="116" t="n">
         <v>46289</v>
       </c>
-      <c r="C11" s="116" t="n">
+      <c r="C12" s="116" t="n">
         <v>46304</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D12" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr">
         <is>
           <t>예약완료</t>
         </is>
       </c>
-      <c r="F11" s="49" t="inlineStr">
+      <c r="F12" s="49" t="inlineStr">
         <is>
           <t>파리 15구 · Rue de Lourmel (Dupleix·Commerce 권역)</t>
         </is>
       </c>
-      <c r="G11" s="49" t="inlineStr">
+      <c r="G12" s="49" t="inlineStr">
         <is>
           <t>KRW</t>
         </is>
       </c>
-      <c r="H11" s="121" t="n">
+      <c r="H12" s="121" t="n">
         <v>5000000</v>
       </c>
-      <c r="I11" s="121" t="n"/>
-      <c r="J11" s="121" t="n"/>
-      <c r="K11" s="122" t="str"/>
-      <c r="L11" s="49" t="str"/>
-      <c r="M11" s="49" t="inlineStr">
+      <c r="I12" s="121" t="n"/>
+      <c r="J12" s="121" t="n"/>
+      <c r="K12" s="122" t="str"/>
+      <c r="L12" s="49" t="str"/>
+      <c r="M12" s="49" t="inlineStr">
         <is>
           <t>78 Rue de Lourmel, 75015 Paris, Île-de-France, France</t>
         </is>
       </c>
-      <c r="N11" s="49" t="inlineStr">
+      <c r="N12" s="49" t="inlineStr">
         <is>
           <t>체크인 15:00 / 체크아웃 11:00</t>
         </is>
       </c>
-      <c r="O11" s="49" t="inlineStr">
+      <c r="O12" s="49" t="inlineStr">
         <is>
           <t>필수</t>
         </is>
       </c>
-      <c r="P11" s="49" t="inlineStr">
+      <c r="P12" s="49" t="inlineStr">
         <is>
           <t>필수</t>
         </is>
       </c>
-      <c r="Q11" s="49" t="inlineStr">
+      <c r="Q12" s="49" t="inlineStr">
         <is>
           <t>불필요</t>
         </is>
       </c>
-      <c r="R11" s="49" t="inlineStr">
+      <c r="R12" s="49" t="inlineStr">
         <is>
           <t>필수</t>
         </is>
       </c>
-      <c r="S11" s="49" t="str"/>
-      <c r="T11" s="66" t="inlineStr">
+      <c r="S12" s="49" t="str"/>
+      <c r="T12" s="66" t="inlineStr">
         <is>
           <t>기존 15박 예약을 9/24~10/9로 날짜 이동 필요; 9/24 생활 완충일 · 10/9 출국</t>
         </is>

</xml_diff>

<commit_message>
Swap Paris museum dates and record confirmed tickets
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -6162,7 +6162,7 @@
       </c>
       <c r="P31" s="100" t="inlineStr">
         <is>
-          <t>없음</t>
+          <t>Grand Palais 세잔전 9/25 17:00 예약 확정</t>
         </is>
       </c>
       <c r="Q31" s="100" t="inlineStr">
@@ -6283,37 +6283,37 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>방향잡기</t>
+          <t>고전 도시공간</t>
         </is>
       </c>
       <c r="F33" s="100" t="inlineStr">
         <is>
-          <t>고전 파리 오리엔테이션</t>
+          <t>Belle Époque &amp; Classical Paris</t>
         </is>
       </c>
       <c r="G33" s="100" t="inlineStr">
         <is>
-          <t>Tuileries</t>
+          <t>Marché Convention·Pichard 후 숙소 점심·휴식</t>
         </is>
       </c>
       <c r="H33" s="100" t="inlineStr">
         <is>
-          <t>Palais Royal 부근</t>
+          <t>숙소 점심</t>
         </is>
       </c>
       <c r="I33" s="100" t="inlineStr">
         <is>
-          <t>Palais Royal·Opéra 지구·Garnier 외관/낮 관람</t>
+          <t>Petit Palais 13:00→Tuileries 15:00→Palais Royal 16:10→Opéra Garnier 17:30</t>
         </is>
       </c>
       <c r="J33" s="100" t="inlineStr">
         <is>
-          <t>자유저녁</t>
+          <t>Bouillon Chartier Montparnasse 저녁</t>
         </is>
       </c>
       <c r="K33" s="100" t="inlineStr">
         <is>
-          <t>도보</t>
+          <t>메트로 8+1호선·도보</t>
         </is>
       </c>
       <c r="L33" s="100" t="inlineStr">
@@ -6334,14 +6334,10 @@
           <t>검토중</t>
         </is>
       </c>
-      <c r="P33" s="100" t="inlineStr">
-        <is>
-          <t>Garnier 조건부</t>
-        </is>
-      </c>
+      <c r="P33" s="100" t="inlineStr"/>
       <c r="Q33" s="100" t="inlineStr">
         <is>
-          <t>Garnier는 외관만</t>
+          <t>야외 구간 단축</t>
         </is>
       </c>
       <c r="R33" s="100" t="inlineStr">
@@ -6462,7 +6458,7 @@
       </c>
       <c r="F35" s="100" t="inlineStr">
         <is>
-          <t>Orsay 또는 Orangerie</t>
+          <t>Musée d'Orsay 집중 관람 &amp; Musée Rodin</t>
         </is>
       </c>
       <c r="G35" s="100" t="inlineStr">
@@ -6477,7 +6473,7 @@
       </c>
       <c r="I35" s="100" t="inlineStr">
         <is>
-          <t>미술관 한 곳</t>
+          <t>Musée d'Orsay 09:30→7구 점심→Musée Rodin 14:30→Invalides 외관</t>
         </is>
       </c>
       <c r="J35" s="100" t="inlineStr">
@@ -6510,12 +6506,12 @@
       </c>
       <c r="P35" s="100" t="inlineStr">
         <is>
-          <t>R020</t>
+          <t>Orsay 09:30·Rodin 14:30</t>
         </is>
       </c>
       <c r="Q35" s="100" t="inlineStr">
         <is>
-          <t>두 번째 관 금지</t>
+          <t>오랑주리는 화요일 휴관 — Orsay 일정 유지</t>
         </is>
       </c>
       <c r="R35" s="100" t="inlineStr">
@@ -6546,37 +6542,37 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>고정 경험</t>
+          <t>미술·패션</t>
         </is>
       </c>
       <c r="F36" s="100" t="inlineStr">
         <is>
-          <t>Fashion Week 공개동선 반일</t>
+          <t>Monet &amp; Contemporary Paris / Fashion</t>
         </is>
       </c>
       <c r="G36" s="100" t="inlineStr">
         <is>
-          <t>여유로운 오전</t>
+          <t>09:15 숙소 출발</t>
         </is>
       </c>
       <c r="H36" s="100" t="inlineStr">
         <is>
-          <t>Palais de Tokyo 권역</t>
+          <t>Chez Savy 12:15</t>
         </is>
       </c>
       <c r="I36" s="100" t="inlineStr">
         <is>
-          <t>Palais de Tokyo 일대→Avenue Montaigne→Rue Saint-Honoré→Palais Royal</t>
+          <t>Orangerie 10:00–11:30→Avenue Montaigne→Grand Palais 공개 동선→Président Wilson→Palais de Tokyo·Alma/Seine</t>
         </is>
       </c>
       <c r="J36" s="100" t="inlineStr">
         <is>
-          <t>늦은 행사 없이 귀가</t>
+          <t>Stéphane Martin 19:30</t>
         </is>
       </c>
       <c r="K36" s="100" t="inlineStr">
         <is>
-          <t>도보·메트로</t>
+          <t>메트로 8·9호선·도보</t>
         </is>
       </c>
       <c r="L36" s="100" t="inlineStr">
@@ -6599,12 +6595,12 @@
       </c>
       <c r="P36" s="100" t="inlineStr">
         <is>
-          <t>공개행사 재확인</t>
+          <t>Orangerie 10:00 예약 확정·Fashion Week 공개행사 재확인</t>
         </is>
       </c>
       <c r="Q36" s="100" t="inlineStr">
         <is>
-          <t>공식 공개 팝업만 추가</t>
+          <t>수련 우선·Walter-Guillaume 주요작 후 11:30 종료</t>
         </is>
       </c>
       <c r="R36" s="100" t="inlineStr">
@@ -7529,7 +7525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V33"/>
+  <dimension ref="A1:V35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="92" min="1" max="1"/>
@@ -9310,7 +9306,11 @@
         </is>
       </c>
       <c r="U23" s="119" t="n"/>
-      <c r="V23" s="63" t="n"/>
+      <c r="V23" s="63" t="inlineStr">
+        <is>
+          <t>Grand Palais 9/25 17:00·Orangerie 9/30 10:00은 별도 확정 행 참조; 이 행은 나머지 미술관 예약</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
@@ -10044,6 +10044,124 @@
       <c r="V33" t="inlineStr">
         <is>
           <t>전자항공권 확인(2026-08-21): OZ502 · 무료 수하물 1PC · 총액 KRW 485,400/인 (마일리지 발권, 2026-08-21 발권)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>R031</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>입장권</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Grand Palais — Cézanne et nous</t>
+        </is>
+      </c>
+      <c r="E34" s="128" t="n">
+        <v>46290</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>확정</t>
+        </is>
+      </c>
+      <c r="I34" s="128" t="n"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>https://www.grandpalais.fr/</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>11_Paris_Long_Stay_v2.0.md</t>
+        </is>
+      </c>
+      <c r="U34" s="128" t="n">
+        <v>46271</v>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>사용자 예약 완료 확인 · 예약번호·금액·취소조건 미제공</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>R032</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>입장권</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Musée de l'Orangerie</t>
+        </is>
+      </c>
+      <c r="E35" s="128" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>확정</t>
+        </is>
+      </c>
+      <c r="I35" s="128" t="n"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>https://www.musee-orangerie.fr/</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>11_Paris_Long_Stay_v2.0.md</t>
+        </is>
+      </c>
+      <c r="U35" s="128" t="n">
+        <v>46271</v>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>사용자 예약 완료 확인 · 예약번호·금액·취소조건 미제공</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Paris PMP itinerary and trip execution UI
</commit_message>
<xml_diff>
--- a/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
+++ b/source/OPERATIONS/TP_Europe_Travel_Master_Tracker_v1.2.xlsx
@@ -6203,12 +6203,12 @@
       </c>
       <c r="F32" s="100" t="inlineStr">
         <is>
-          <t>Saint-Germain·Luxembourg·Seine</t>
+          <t>PMP 시작 — Sainte-Chapelle &amp; Conciergerie</t>
         </is>
       </c>
       <c r="G32" s="100" t="inlineStr">
         <is>
-          <t>늦은 시작·가벼운 운동</t>
+          <t>오전 생활 일정·숙소 휴식</t>
         </is>
       </c>
       <c r="H32" s="100" t="inlineStr">
@@ -6218,12 +6218,12 @@
       </c>
       <c r="I32" s="100" t="inlineStr">
         <is>
-          <t>Luxembourg Gardens·Seine 산책</t>
+          <t>Sainte-Chapelle 15:00(PMP 최초 사용)→Conciergerie→Île de la Cité</t>
         </is>
       </c>
       <c r="J32" s="100" t="inlineStr">
         <is>
-          <t>무예약</t>
+          <t>Bouillon Racine</t>
         </is>
       </c>
       <c r="K32" s="100" t="inlineStr">
@@ -6249,7 +6249,11 @@
           <t>검토중</t>
         </is>
       </c>
-      <c r="P32" s="100" t="n"/>
+      <c r="P32" s="100" t="inlineStr">
+        <is>
+          <t>PMP 6일/144시간 구매완료</t>
+        </is>
+      </c>
       <c r="Q32" s="100" t="inlineStr">
         <is>
           <t>Luxembourg까지만</t>
@@ -6288,22 +6292,22 @@
       </c>
       <c r="F33" s="100" t="inlineStr">
         <is>
-          <t>Belle Époque &amp; Classical Paris</t>
+          <t>Picasso·Notre-Dame &amp; Classical Paris</t>
         </is>
       </c>
       <c r="G33" s="100" t="inlineStr">
         <is>
-          <t>Marché Convention·Pichard 후 숙소 점심·휴식</t>
+          <t>Marché Convention·Pichard</t>
         </is>
       </c>
       <c r="H33" s="100" t="inlineStr">
         <is>
-          <t>숙소 점심</t>
+          <t>Le Marais</t>
         </is>
       </c>
       <c r="I33" s="100" t="inlineStr">
         <is>
-          <t>Petit Palais 13:00→Tuileries 15:00→Palais Royal 16:10→Opéra Garnier 17:30</t>
+          <t>Picasso 10:30(PMP)→Notre-Dame(무료)→Tuileries→Palais Royal→Garnier</t>
         </is>
       </c>
       <c r="J33" s="100" t="inlineStr">
@@ -6334,7 +6338,11 @@
           <t>검토중</t>
         </is>
       </c>
-      <c r="P33" s="100" t="inlineStr"/>
+      <c r="P33" s="100" t="inlineStr">
+        <is>
+          <t>Notre-Dame PMP 불필요</t>
+        </is>
+      </c>
       <c r="Q33" s="100" t="inlineStr">
         <is>
           <t>야외 구간 단축</t>
@@ -6388,7 +6396,7 @@
       </c>
       <c r="I34" s="100" t="inlineStr">
         <is>
-          <t>쇼핑·북마레/주거지 산책</t>
+          <t>Moreau→Fashion Week·Marais→Arc de Triomphe Optional(PMP)</t>
         </is>
       </c>
       <c r="J34" s="100" t="inlineStr">
@@ -6419,7 +6427,11 @@
           <t>검토중</t>
         </is>
       </c>
-      <c r="P34" s="100" t="n"/>
+      <c r="P34" s="100" t="inlineStr">
+        <is>
+          <t>Arc de Triomphe 선택</t>
+        </is>
+      </c>
       <c r="Q34" s="100" t="inlineStr">
         <is>
           <t>숙소권 쇼핑만</t>
@@ -6453,42 +6465,42 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>박물관</t>
+          <t>근교·왕실문화</t>
         </is>
       </c>
       <c r="F35" s="100" t="inlineStr">
         <is>
-          <t>Musée d'Orsay 집중 관람 &amp; Musée Rodin</t>
+          <t>Versailles Palace &amp; Gardens</t>
         </is>
       </c>
       <c r="G35" s="100" t="inlineStr">
         <is>
-          <t>느린 아침</t>
+          <t>08:30 숙소 출발</t>
         </is>
       </c>
       <c r="H35" s="100" t="inlineStr">
         <is>
-          <t>관람 전 점심</t>
+          <t>La Flottille 12:45</t>
         </is>
       </c>
       <c r="I35" s="100" t="inlineStr">
         <is>
-          <t>Musée d'Orsay 09:30→7구 점심→Musée Rodin 14:30→Invalides 외관</t>
+          <t>RER C→Versailles 본관 10:00 전후→Gardens→Trianon 선택</t>
         </is>
       </c>
       <c r="J35" s="100" t="inlineStr">
         <is>
-          <t>저녁 비움</t>
+          <t>Le Grand Pan 20:00</t>
         </is>
       </c>
       <c r="K35" s="100" t="inlineStr">
         <is>
-          <t>메트로·도보</t>
+          <t>RER C·영지 도보</t>
         </is>
       </c>
       <c r="L35" s="100" t="inlineStr">
         <is>
-          <t>선택 산책</t>
+          <t>Trianon·왕비의 촌락</t>
         </is>
       </c>
       <c r="M35" s="100" t="inlineStr">
@@ -6496,8 +6508,10 @@
           <t>미술관 스케치</t>
         </is>
       </c>
-      <c r="N35" s="100" t="n">
-        <v>3</v>
+      <c r="N35" s="100" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="O35" s="100" t="inlineStr">
         <is>
@@ -6506,12 +6520,12 @@
       </c>
       <c r="P35" s="100" t="inlineStr">
         <is>
-          <t>Orsay 09:30·Rodin 14:30</t>
+          <t>Versailles Passport 10:00 전후·La Flottille·Le Grand Pan</t>
         </is>
       </c>
       <c r="Q35" s="100" t="inlineStr">
         <is>
-          <t>오랑주리는 화요일 휴관 — Orsay 일정 유지</t>
+          <t>RER C·Passport 슬롯 확인, 피로 시 미니트레인</t>
         </is>
       </c>
       <c r="R35" s="100" t="inlineStr">
@@ -6562,7 +6576,7 @@
       </c>
       <c r="I36" s="100" t="inlineStr">
         <is>
-          <t>Orangerie 10:00–11:30→Avenue Montaigne→Grand Palais 공개 동선→Président Wilson→Palais de Tokyo·Alma/Seine</t>
+          <t>Orangerie 10:00→Chez Savy→Fashion Week→Guimet 14:40→Palais de Tokyo</t>
         </is>
       </c>
       <c r="J36" s="100" t="inlineStr">
@@ -6595,7 +6609,7 @@
       </c>
       <c r="P36" s="100" t="inlineStr">
         <is>
-          <t>Orangerie 10:00 예약 확정·Fashion Week 공개행사 재확인</t>
+          <t>Orangerie 예약완료·Guimet PMP</t>
         </is>
       </c>
       <c r="Q36" s="100" t="inlineStr">
@@ -6631,42 +6645,42 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>동네 산책</t>
+          <t>미술·조각</t>
         </is>
       </c>
       <c r="F37" s="100" t="inlineStr">
         <is>
-          <t>Rossini 오페라일</t>
+          <t>Impressionism &amp; Sculpture — Orsay &amp; Rodin</t>
         </is>
       </c>
       <c r="G37" s="100" t="inlineStr">
         <is>
-          <t>운동·느린 아침</t>
+          <t>09:30 숙소 출발</t>
         </is>
       </c>
       <c r="H37" s="100" t="inlineStr">
         <is>
-          <t>가벼운 점심</t>
+          <t>Café Varenne 13:00</t>
         </is>
       </c>
       <c r="I37" s="100" t="inlineStr">
         <is>
-          <t>Place des Vosges·Bastille 산책</t>
+          <t>Musée d'Orsay 10:30(확정)→Musée Rodin 14:15→Invalides 선택</t>
         </is>
       </c>
       <c r="J37" s="100" t="inlineStr">
         <is>
-          <t>저녁 — 공연 대체안 검토 중</t>
+          <t>Café du Commerce 18:30</t>
         </is>
       </c>
       <c r="K37" s="100" t="inlineStr">
         <is>
-          <t>Opéra Bastille 왕복</t>
+          <t>메트로 8·12호선·도보</t>
         </is>
       </c>
       <c r="L37" s="100" t="inlineStr">
         <is>
-          <t>운동</t>
+          <t>Invalides 외관</t>
         </is>
       </c>
       <c r="M37" s="100" t="inlineStr">
@@ -6674,22 +6688,24 @@
           <t>Place des Vosges</t>
         </is>
       </c>
-      <c r="N37" s="100" t="n">
-        <v>5</v>
+      <c r="N37" s="100" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="O37" s="100" t="inlineStr">
         <is>
-          <t>검토중</t>
+          <t>확정</t>
         </is>
       </c>
       <c r="P37" s="100" t="inlineStr">
         <is>
-          <t>R021</t>
+          <t>Orsay 10:30 예약 확정·Rodin 14:15 권장</t>
         </is>
       </c>
       <c r="Q37" s="100" t="inlineStr">
         <is>
-          <t>10/7 공연 백업</t>
+          <t>10/1 상설 중심, 10/6 Mary Cassatt 특별전 재방문과 분리</t>
         </is>
       </c>
       <c r="R37" s="100" t="inlineStr">
@@ -6725,12 +6741,12 @@
       </c>
       <c r="F38" s="100" t="inlineStr">
         <is>
-          <t>오페라 뒤 회복일</t>
+          <t>Louvre 11:00 — PMP 마지막 핵심 사용</t>
         </is>
       </c>
       <c r="G38" s="100" t="inlineStr">
         <is>
-          <t>늦은 시작</t>
+          <t>10:15 출발</t>
         </is>
       </c>
       <c r="H38" s="100" t="inlineStr">
@@ -6740,7 +6756,7 @@
       </c>
       <c r="I38" s="100" t="inlineStr">
         <is>
-          <t>시장·서점·카페·스케치</t>
+          <t>Louvre 11:00~15:00→Cour Carrée·Seine</t>
         </is>
       </c>
       <c r="J38" s="100" t="inlineStr">
@@ -6771,7 +6787,11 @@
           <t>검토중</t>
         </is>
       </c>
-      <c r="P38" s="100" t="n"/>
+      <c r="P38" s="100" t="inlineStr">
+        <is>
+          <t>Louvre 11:00·PMP last planned use</t>
+        </is>
+      </c>
       <c r="Q38" s="100" t="inlineStr">
         <is>
           <t>완전 휴식 가능</t>
@@ -6947,7 +6967,7 @@
       </c>
       <c r="P40" s="100" t="inlineStr">
         <is>
-          <t>R023</t>
+          <t>Qatar Prix de l'Arc de Triomphe General Entry 예약완료</t>
         </is>
       </c>
       <c r="Q40" s="100" t="inlineStr">
@@ -7073,7 +7093,7 @@
       </c>
       <c r="F42" s="100" t="inlineStr">
         <is>
-          <t>동부 파리 생활일</t>
+          <t>Orsay Mary Cassatt 특별전 &amp; 마레</t>
         </is>
       </c>
       <c r="G42" s="100" t="inlineStr">
@@ -7088,7 +7108,7 @@
       </c>
       <c r="I42" s="100" t="inlineStr">
         <is>
-          <t>Belleville 또는 다른 동네</t>
+          <t>Orsay Mary Cassatt→Carnavalet·Place des Vosges</t>
         </is>
       </c>
       <c r="J42" s="100" t="inlineStr">
@@ -7121,7 +7141,7 @@
       </c>
       <c r="P42" s="100" t="inlineStr">
         <is>
-          <t>R022 백업</t>
+          <t>10/1 상설 방문과 독립 유지</t>
         </is>
       </c>
       <c r="Q42" s="100" t="inlineStr">
@@ -7251,7 +7271,7 @@
       </c>
       <c r="F44" s="100" t="inlineStr">
         <is>
-          <t>Chaillot·Este Mundo 선택</t>
+          <t>MAM &amp; Trocadéro 고별 일몰</t>
         </is>
       </c>
       <c r="G44" s="100" t="inlineStr">
@@ -7266,7 +7286,7 @@
       </c>
       <c r="I44" s="100" t="inlineStr">
         <is>
-          <t>Trocadéro·Chaillot</t>
+          <t>Musée d'Art Moderne→Trocadéro</t>
         </is>
       </c>
       <c r="J44" s="100" t="inlineStr">
@@ -7299,7 +7319,7 @@
       </c>
       <c r="P44" s="100" t="inlineStr">
         <is>
-          <t>R024 조건부</t>
+          <t>Guimet는 9/30으로 이동</t>
         </is>
       </c>
       <c r="Q44" s="100" t="inlineStr">
@@ -7525,7 +7545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V35"/>
+  <dimension ref="A1:V38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="92" min="1" max="1"/>
@@ -9308,7 +9328,7 @@
       <c r="U23" s="119" t="n"/>
       <c r="V23" s="63" t="inlineStr">
         <is>
-          <t>Grand Palais 9/25 17:00·Orangerie 9/30 10:00은 별도 확정 행 참조; 이 행은 나머지 미술관 예약</t>
+          <t>Grand Palais 9/25 17:00·Orangerie 9/30 10:00·Orsay 10/1 10:30은 별도 확정 행 참조; 이 행은 나머지 미술관 예약</t>
         </is>
       </c>
     </row>
@@ -9496,7 +9516,11 @@
       <c r="E26" s="119" t="n">
         <v>46299</v>
       </c>
-      <c r="F26" s="100" t="n"/>
+      <c r="F26" s="100" t="inlineStr">
+        <is>
+          <t>General Entry</t>
+        </is>
+      </c>
       <c r="G26" s="100" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9504,7 +9528,7 @@
       </c>
       <c r="H26" s="100" t="inlineStr">
         <is>
-          <t>미예약</t>
+          <t>확정</t>
         </is>
       </c>
       <c r="I26" s="119" t="n">
@@ -9544,7 +9568,7 @@
       </c>
       <c r="V26" s="63" t="inlineStr">
         <is>
-          <t>France Galop BOOK NOW 확인</t>
+          <t>사용자 예약 완료 확인 · General Entry · 지정석/VIP 아님</t>
         </is>
       </c>
     </row>
@@ -10162,6 +10186,183 @@
       <c r="V35" t="inlineStr">
         <is>
           <t>사용자 예약 완료 확인 · 예약번호·금액·취소조건 미제공</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>R033</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>입장권</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Musée d'Orsay — Permanent Collection</t>
+        </is>
+      </c>
+      <c r="E36" s="128" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>확정</t>
+        </is>
+      </c>
+      <c r="I36" s="128" t="n"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>https://www.musee-orsay.fr/</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>11_Paris_Long_Stay_v2.0.md</t>
+        </is>
+      </c>
+      <c r="U36" s="128" t="n">
+        <v>46271</v>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>사용자 예약 완료 확인 · 10/1 상설 컬렉션 · 예약번호·금액·취소조건 미제공</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>R034</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>입장권</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Château de Versailles — Passport</t>
+        </is>
+      </c>
+      <c r="E37" s="128" t="n">
+        <v>46294</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>10:00 전후</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>확정</t>
+        </is>
+      </c>
+      <c r="I37" s="128" t="n"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>https://www.chateauversailles.fr/</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>11_Paris_Long_Stay_v2.0.md</t>
+        </is>
+      </c>
+      <c r="U37" s="128" t="n">
+        <v>46271</v>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>사용자 예약 완료 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>R035</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>입장권</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Paris Museum Pass — 6-day / 144-hour</t>
+        </is>
+      </c>
+      <c r="E38" s="128" t="n">
+        <v>46291</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>15:00 첫 사용</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>확정</t>
+        </is>
+      </c>
+      <c r="I38" s="128" t="n"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>https://www.parismuseumpass.fr/</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>11_Paris_Long_Stay_v2.0.md</t>
+        </is>
+      </c>
+      <c r="U38" s="128" t="n">
+        <v>46271</v>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>구매완료 · Sainte-Chapelle 첫 사용 → 10/2 Louvre 11:00 마지막 계획</t>
         </is>
       </c>
     </row>

</xml_diff>